<commit_message>
cambios en billetes, monedas y detalles nuevo
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930B0F76-9037-408A-8331-E55D3340DBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B92A672-E0C8-47DB-B814-E0CC3621B0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RUTA" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="100">
   <si>
     <t>RECORRIDO</t>
   </si>
@@ -328,6 +328,12 @@
   </si>
   <si>
     <t>{{transf_valor}}</t>
+  </si>
+  <si>
+    <t>{{extraction.rendicion.cant_fact.valor}}</t>
+  </si>
+  <si>
+    <t>{{extraction.rendicion.valor_total.valor}}</t>
   </si>
 </sst>
 </file>
@@ -1445,170 +1451,170 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2203,9 +2209,11 @@
       <c r="A9" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="119"/>
-      <c r="C9" s="110"/>
-      <c r="D9" s="110"/>
+      <c r="B9" s="174" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="175"/>
+      <c r="D9" s="176"/>
       <c r="E9" s="110"/>
       <c r="F9" s="119"/>
       <c r="G9" s="110"/>
@@ -2257,9 +2265,11 @@
       <c r="A11" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="119"/>
-      <c r="C11" s="110"/>
-      <c r="D11" s="119"/>
+      <c r="B11" s="174" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="175"/>
+      <c r="D11" s="176"/>
       <c r="E11" s="110"/>
       <c r="F11" s="119"/>
       <c r="G11" s="110"/>
@@ -2284,9 +2294,11 @@
       <c r="A12" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="119"/>
-      <c r="C12" s="110"/>
-      <c r="D12" s="119"/>
+      <c r="B12" s="174" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="175"/>
+      <c r="D12" s="176"/>
       <c r="E12" s="110"/>
       <c r="F12" s="119"/>
       <c r="G12" s="110"/>
@@ -2311,9 +2323,11 @@
       <c r="A13" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="119"/>
-      <c r="C13" s="110"/>
-      <c r="D13" s="119"/>
+      <c r="B13" s="174" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="175"/>
+      <c r="D13" s="176"/>
       <c r="E13" s="110"/>
       <c r="F13" s="119"/>
       <c r="G13" s="110"/>
@@ -2338,9 +2352,11 @@
       <c r="A14" s="128" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="110"/>
-      <c r="D14" s="119"/>
+      <c r="B14" s="174" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="175"/>
+      <c r="D14" s="176"/>
       <c r="E14" s="110"/>
       <c r="F14" s="119"/>
       <c r="G14" s="110"/>
@@ -2365,9 +2381,11 @@
       <c r="A15" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="119"/>
-      <c r="C15" s="110"/>
-      <c r="D15" s="119"/>
+      <c r="B15" s="174" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="175"/>
+      <c r="D15" s="176"/>
       <c r="E15" s="110"/>
       <c r="F15" s="119"/>
       <c r="G15" s="110"/>
@@ -2392,9 +2410,11 @@
       <c r="A16" s="128" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="119"/>
-      <c r="C16" s="110"/>
-      <c r="D16" s="119"/>
+      <c r="B16" s="174" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="175"/>
+      <c r="D16" s="176"/>
       <c r="E16" s="110"/>
       <c r="F16" s="119"/>
       <c r="G16" s="110"/>
@@ -2419,9 +2439,11 @@
       <c r="A17" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="119"/>
-      <c r="C17" s="110"/>
-      <c r="D17" s="119"/>
+      <c r="B17" s="174" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="175"/>
+      <c r="D17" s="176"/>
       <c r="E17" s="110"/>
       <c r="F17" s="119"/>
       <c r="G17" s="110"/>
@@ -2447,11 +2469,11 @@
         <v>11</v>
       </c>
       <c r="B18" s="119">
-        <f t="shared" ref="B18:O18" si="0">SUM(B9:B17)</f>
+        <f>SUM(B9:B17)</f>
         <v>0</v>
       </c>
       <c r="C18" s="119">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B18:O18" si="0">SUM(C9:C17)</f>
         <v>0</v>
       </c>
       <c r="D18" s="119">
@@ -2680,17 +2702,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="206" t="s">
+      <c r="M22" s="173" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="206"/>
-      <c r="O22" s="206"/>
-      <c r="P22" s="206"/>
-      <c r="Q22" s="206"/>
-      <c r="R22" s="206"/>
-      <c r="S22" s="206"/>
-      <c r="T22" s="206"/>
-      <c r="U22" s="206"/>
+      <c r="N22" s="173"/>
+      <c r="O22" s="173"/>
+      <c r="P22" s="173"/>
+      <c r="Q22" s="173"/>
+      <c r="R22" s="173"/>
+      <c r="S22" s="173"/>
+      <c r="T22" s="173"/>
+      <c r="U22" s="173"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2699,20 +2721,19 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="215" t="s">
+      <c r="N23" s="189" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="216"/>
-      <c r="P23" s="216"/>
-      <c r="Q23" s="216"/>
-      <c r="R23" s="216"/>
-      <c r="S23" s="217"/>
+      <c r="O23" s="190"/>
+      <c r="P23" s="190"/>
+      <c r="Q23" s="190"/>
+      <c r="R23" s="190"/>
+      <c r="S23" s="191"/>
       <c r="T23" s="142" t="s">
         <v>38</v>
       </c>
-      <c r="U23" s="115" t="e">
-        <f>B6+C6+D6+E6+F6+G6+H6+I6+J6+K6+L6+M6+N6+O6+P6+Q6+R6+S6+T6+U6+V6+W6+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!</f>
-        <v>#VALUE!</v>
+      <c r="U23" s="115" t="s">
+        <v>98</v>
       </c>
       <c r="W23" s="96" t="s">
         <v>44</v>
@@ -2725,24 +2746,23 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="218" t="s">
+      <c r="N24" s="192" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="219"/>
-      <c r="P24" s="219"/>
-      <c r="Q24" s="219"/>
-      <c r="R24" s="219"/>
-      <c r="S24" s="220"/>
+      <c r="O24" s="193"/>
+      <c r="P24" s="193"/>
+      <c r="Q24" s="193"/>
+      <c r="R24" s="193"/>
+      <c r="S24" s="194"/>
       <c r="T24" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="U24" s="116" t="e">
-        <f>B7+C7+D7+E7+F7+G7+H7+I7+J7+K7+L7+M7+N7+O7+P7+Q7+R7+S7+T7+U7+V7+W7+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="W24" s="141" t="e">
+      <c r="U24" s="116" t="s">
+        <v>99</v>
+      </c>
+      <c r="W24" s="141" t="str">
         <f>U23</f>
-        <v>#VALUE!</v>
+        <v>{{extraction.rendicion.cant_fact.valor}}</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
@@ -2754,21 +2774,21 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="221" t="s">
+      <c r="M25" s="195" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="222"/>
-      <c r="O25" s="223"/>
-      <c r="P25" s="224"/>
-      <c r="Q25" s="198" t="s">
+      <c r="N25" s="196"/>
+      <c r="O25" s="197"/>
+      <c r="P25" s="198"/>
+      <c r="Q25" s="174" t="s">
         <v>64</v>
       </c>
-      <c r="R25" s="199"/>
-      <c r="S25" s="200"/>
-      <c r="T25" s="225" t="s">
+      <c r="R25" s="175"/>
+      <c r="S25" s="176"/>
+      <c r="T25" s="171" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="226"/>
+      <c r="U25" s="172"/>
       <c r="V25" s="13"/>
       <c r="W25" s="86" t="s">
         <v>45</v>
@@ -2784,12 +2804,12 @@
       <c r="N26" s="84"/>
       <c r="O26" s="151"/>
       <c r="P26" s="152"/>
-      <c r="Q26" s="198" t="e">
+      <c r="Q26" s="174" t="e">
         <f>B10+C10+D10+E10+F10+G10+H10+I10+J10+K10+L10+N10+O10+P10+Q10+R10+S10+T10+U10+V10+W10+#REF!+#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="R26" s="199"/>
-      <c r="S26" s="200"/>
+      <c r="R26" s="175"/>
+      <c r="S26" s="176"/>
       <c r="T26" s="149"/>
       <c r="U26" s="150"/>
       <c r="V26" s="13"/>
@@ -2800,30 +2820,30 @@
         <f>B1</f>
         <v>{{extraction.conductor.valor}}</v>
       </c>
-      <c r="J27" s="162">
+      <c r="J27" s="162" t="str">
         <f>B9</f>
-        <v>0</v>
+        <v>{{extraction.rendicion.efectivo_total.valor}}</v>
       </c>
       <c r="L27"/>
       <c r="M27" s="83" t="s">
         <v>18</v>
       </c>
       <c r="N27" s="84"/>
-      <c r="O27" s="193"/>
-      <c r="P27" s="194"/>
-      <c r="Q27" s="198" t="s">
+      <c r="O27" s="177"/>
+      <c r="P27" s="178"/>
+      <c r="Q27" s="174" t="s">
         <v>65</v>
       </c>
-      <c r="R27" s="199"/>
-      <c r="S27" s="200"/>
-      <c r="T27" s="213" t="s">
+      <c r="R27" s="175"/>
+      <c r="S27" s="176"/>
+      <c r="T27" s="187" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="214"/>
+      <c r="U27" s="188"/>
       <c r="V27" s="19"/>
-      <c r="W27" s="97" t="e">
+      <c r="W27" s="97" t="str">
         <f>U24</f>
-        <v>#VALUE!</v>
+        <v>{{extraction.rendicion.valor_total.valor}}</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
@@ -2836,21 +2856,21 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="191" t="s">
+      <c r="M28" s="183" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="192"/>
-      <c r="O28" s="193"/>
-      <c r="P28" s="194"/>
-      <c r="Q28" s="198" t="s">
+      <c r="N28" s="184"/>
+      <c r="O28" s="177"/>
+      <c r="P28" s="178"/>
+      <c r="Q28" s="174" t="s">
         <v>66</v>
       </c>
-      <c r="R28" s="199"/>
-      <c r="S28" s="200"/>
-      <c r="T28" s="211" t="s">
+      <c r="R28" s="175"/>
+      <c r="S28" s="176"/>
+      <c r="T28" s="185" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="212"/>
+      <c r="U28" s="186"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2865,24 +2885,24 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="191" t="s">
+      <c r="M29" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="192"/>
-      <c r="O29" s="193"/>
-      <c r="P29" s="194"/>
-      <c r="Q29" s="198" t="s">
+      <c r="N29" s="184"/>
+      <c r="O29" s="177"/>
+      <c r="P29" s="178"/>
+      <c r="Q29" s="174" t="s">
         <v>67</v>
       </c>
-      <c r="R29" s="199"/>
-      <c r="S29" s="200"/>
-      <c r="T29" s="207" t="s">
+      <c r="R29" s="175"/>
+      <c r="S29" s="176"/>
+      <c r="T29" s="179" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="208"/>
-      <c r="W29" s="98" t="e">
+      <c r="U29" s="180"/>
+      <c r="W29" s="98" t="str">
         <f>U23</f>
-        <v>#VALUE!</v>
+        <v>{{extraction.rendicion.cant_fact.valor}}</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
@@ -2896,21 +2916,21 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="191" t="s">
+      <c r="M30" s="183" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="192"/>
-      <c r="O30" s="193"/>
+      <c r="N30" s="184"/>
+      <c r="O30" s="177"/>
       <c r="P30" s="205"/>
-      <c r="Q30" s="198" t="s">
+      <c r="Q30" s="174" t="s">
         <v>68</v>
       </c>
-      <c r="R30" s="199"/>
-      <c r="S30" s="200"/>
-      <c r="T30" s="209" t="s">
+      <c r="R30" s="175"/>
+      <c r="S30" s="176"/>
+      <c r="T30" s="181" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="210"/>
+      <c r="U30" s="182"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2928,17 +2948,17 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="191" t="s">
+      <c r="M31" s="183" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="192"/>
-      <c r="O31" s="193"/>
-      <c r="P31" s="194"/>
-      <c r="Q31" s="198" t="s">
+      <c r="N31" s="184"/>
+      <c r="O31" s="177"/>
+      <c r="P31" s="178"/>
+      <c r="Q31" s="174" t="s">
         <v>69</v>
       </c>
-      <c r="R31" s="199"/>
-      <c r="S31" s="200"/>
+      <c r="R31" s="175"/>
+      <c r="S31" s="176"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2953,17 +2973,17 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="191" t="s">
+      <c r="M32" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="192"/>
-      <c r="O32" s="193"/>
-      <c r="P32" s="194"/>
-      <c r="Q32" s="198" t="s">
+      <c r="N32" s="184"/>
+      <c r="O32" s="177"/>
+      <c r="P32" s="178"/>
+      <c r="Q32" s="174" t="s">
         <v>70</v>
       </c>
-      <c r="R32" s="199"/>
-      <c r="S32" s="200"/>
+      <c r="R32" s="175"/>
+      <c r="S32" s="176"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="86" t="s">
@@ -2985,13 +3005,13 @@
         <v>25</v>
       </c>
       <c r="N33" s="85"/>
-      <c r="O33" s="193"/>
-      <c r="P33" s="194"/>
-      <c r="Q33" s="198" t="s">
+      <c r="O33" s="177"/>
+      <c r="P33" s="178"/>
+      <c r="Q33" s="174" t="s">
         <v>71</v>
       </c>
-      <c r="R33" s="199"/>
-      <c r="S33" s="200"/>
+      <c r="R33" s="175"/>
+      <c r="S33" s="176"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="138" t="e">
@@ -3016,11 +3036,11 @@
       <c r="N34" s="202"/>
       <c r="O34" s="203"/>
       <c r="P34" s="204"/>
-      <c r="Q34" s="198" t="s">
+      <c r="Q34" s="174" t="s">
         <v>72</v>
       </c>
-      <c r="R34" s="199"/>
-      <c r="S34" s="200"/>
+      <c r="R34" s="175"/>
+      <c r="S34" s="176"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3038,23 +3058,23 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="195" t="s">
+      <c r="M35" s="209" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="196"/>
-      <c r="O35" s="197"/>
-      <c r="P35" s="181" t="s">
+      <c r="N35" s="210"/>
+      <c r="O35" s="211"/>
+      <c r="P35" s="199" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="183"/>
-      <c r="R35" s="181" t="s">
+      <c r="Q35" s="200"/>
+      <c r="R35" s="199" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="183"/>
-      <c r="T35" s="181" t="s">
+      <c r="S35" s="200"/>
+      <c r="T35" s="199" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="183"/>
+      <c r="U35" s="200"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3154,10 +3174,10 @@
       <c r="L38" s="114">
         <v>2</v>
       </c>
-      <c r="M38" s="179" t="s">
+      <c r="M38" s="207" t="s">
         <v>42</v>
       </c>
-      <c r="N38" s="180"/>
+      <c r="N38" s="208"/>
       <c r="O38" s="46" t="s">
         <v>65</v>
       </c>
@@ -3267,8 +3287,8 @@
       <c r="A43" s="112"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="188"/>
-      <c r="E43" s="188"/>
+      <c r="D43" s="206"/>
+      <c r="E43" s="206"/>
       <c r="F43" s="51"/>
       <c r="G43" s="8"/>
       <c r="I43" s="136"/>
@@ -3294,8 +3314,8 @@
       <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="188"/>
-      <c r="E44" s="188"/>
+      <c r="D44" s="206"/>
+      <c r="E44" s="206"/>
       <c r="F44" s="52"/>
       <c r="H44" s="68"/>
       <c r="I44" s="13"/>
@@ -3318,8 +3338,8 @@
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="43"/>
-      <c r="D45" s="188"/>
-      <c r="E45" s="188"/>
+      <c r="D45" s="206"/>
+      <c r="E45" s="206"/>
       <c r="F45" s="23"/>
       <c r="H45" s="68"/>
       <c r="I45" s="13"/>
@@ -3341,8 +3361,8 @@
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="43"/>
-      <c r="D46" s="188"/>
-      <c r="E46" s="188"/>
+      <c r="D46" s="206"/>
+      <c r="E46" s="206"/>
       <c r="F46" s="53"/>
       <c r="H46" s="68"/>
       <c r="I46" s="13"/>
@@ -3364,8 +3384,8 @@
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="43"/>
-      <c r="D47" s="188"/>
-      <c r="E47" s="188"/>
+      <c r="D47" s="206"/>
+      <c r="E47" s="206"/>
       <c r="F47" s="17"/>
       <c r="G47" s="1"/>
       <c r="H47" s="68"/>
@@ -3392,8 +3412,8 @@
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="43"/>
-      <c r="D48" s="188"/>
-      <c r="E48" s="188"/>
+      <c r="D48" s="206"/>
+      <c r="E48" s="206"/>
       <c r="F48" s="23"/>
       <c r="G48" s="1"/>
       <c r="H48" s="68"/>
@@ -3416,8 +3436,8 @@
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="43"/>
-      <c r="D49" s="188"/>
-      <c r="E49" s="188"/>
+      <c r="D49" s="206"/>
+      <c r="E49" s="206"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
       <c r="H49" s="50"/>
@@ -3464,8 +3484,8 @@
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="43"/>
-      <c r="D51" s="175"/>
-      <c r="E51" s="175"/>
+      <c r="D51" s="219"/>
+      <c r="E51" s="219"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="50"/>
@@ -3488,8 +3508,8 @@
       <c r="A52" s="20"/>
       <c r="B52" s="55"/>
       <c r="C52" s="43"/>
-      <c r="D52" s="177"/>
-      <c r="E52" s="177"/>
+      <c r="D52" s="218"/>
+      <c r="E52" s="218"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="50"/>
@@ -3512,8 +3532,8 @@
       <c r="A53" s="25"/>
       <c r="B53" s="55"/>
       <c r="C53" s="43"/>
-      <c r="D53" s="174"/>
-      <c r="E53" s="174"/>
+      <c r="D53" s="217"/>
+      <c r="E53" s="217"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="50"/>
@@ -3534,8 +3554,8 @@
       <c r="A54" s="20"/>
       <c r="B54" s="55"/>
       <c r="C54" s="43"/>
-      <c r="D54" s="174"/>
-      <c r="E54" s="174"/>
+      <c r="D54" s="217"/>
+      <c r="E54" s="217"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="50"/>
@@ -3666,8 +3686,8 @@
       <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="43"/>
-      <c r="D60" s="174"/>
-      <c r="E60" s="174"/>
+      <c r="D60" s="217"/>
+      <c r="E60" s="217"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="50"/>
@@ -3754,8 +3774,8 @@
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="43"/>
-      <c r="D64" s="174"/>
-      <c r="E64" s="174"/>
+      <c r="D64" s="217"/>
+      <c r="E64" s="217"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="50"/>
@@ -3776,18 +3796,18 @@
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="43"/>
-      <c r="D65" s="174"/>
-      <c r="E65" s="174"/>
+      <c r="D65" s="217"/>
+      <c r="E65" s="217"/>
       <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="50"/>
       <c r="I65" s="54"/>
       <c r="J65" s="57"/>
       <c r="L65"/>
-      <c r="M65" s="179" t="s">
+      <c r="M65" s="207" t="s">
         <v>34</v>
       </c>
-      <c r="N65" s="180"/>
+      <c r="N65" s="208"/>
       <c r="O65" s="46" t="s">
         <v>66</v>
       </c>
@@ -3814,8 +3834,8 @@
       <c r="A66" s="25"/>
       <c r="B66"/>
       <c r="C66" s="95"/>
-      <c r="D66" s="174"/>
-      <c r="E66" s="174"/>
+      <c r="D66" s="217"/>
+      <c r="E66" s="217"/>
       <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="50"/>
@@ -3843,29 +3863,29 @@
       <c r="I67" s="54"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="181" t="s">
+      <c r="M67" s="199" t="s">
         <v>47</v>
       </c>
-      <c r="N67" s="182"/>
-      <c r="O67" s="183"/>
-      <c r="P67" s="189"/>
-      <c r="Q67" s="190"/>
-      <c r="R67" s="181" t="s">
+      <c r="N67" s="216"/>
+      <c r="O67" s="200"/>
+      <c r="P67" s="220"/>
+      <c r="Q67" s="221"/>
+      <c r="R67" s="199" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="182"/>
-      <c r="T67" s="184" t="str">
+      <c r="S67" s="216"/>
+      <c r="T67" s="212" t="str">
         <f>Q25</f>
         <v>{{extraction.rendicion.efectivo_total.valor}}</v>
       </c>
-      <c r="U67" s="185"/>
+      <c r="U67" s="213"/>
     </row>
     <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="174"/>
-      <c r="E68" s="174"/>
+      <c r="D68" s="217"/>
+      <c r="E68" s="217"/>
       <c r="F68" s="67"/>
       <c r="G68" s="1"/>
       <c r="H68" s="50"/>
@@ -3886,33 +3906,33 @@
       <c r="A69" s="25"/>
       <c r="B69" s="95"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="174"/>
-      <c r="E69" s="174"/>
+      <c r="D69" s="217"/>
+      <c r="E69" s="217"/>
       <c r="F69" s="67"/>
       <c r="G69" s="1"/>
       <c r="H69" s="50"/>
       <c r="I69" s="54"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="179" t="s">
+      <c r="M69" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="N69" s="186"/>
-      <c r="O69" s="186"/>
-      <c r="P69" s="186"/>
-      <c r="Q69" s="186"/>
-      <c r="R69" s="186"/>
-      <c r="S69" s="186"/>
-      <c r="T69" s="186"/>
-      <c r="U69" s="187"/>
+      <c r="N69" s="214"/>
+      <c r="O69" s="214"/>
+      <c r="P69" s="214"/>
+      <c r="Q69" s="214"/>
+      <c r="R69" s="214"/>
+      <c r="S69" s="214"/>
+      <c r="T69" s="214"/>
+      <c r="U69" s="215"/>
       <c r="V69" s="55"/>
     </row>
     <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
       <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="174"/>
-      <c r="E70" s="174"/>
+      <c r="D70" s="217"/>
+      <c r="E70" s="217"/>
       <c r="F70" s="67"/>
       <c r="G70" s="1"/>
       <c r="H70" s="50"/>
@@ -3949,8 +3969,8 @@
       <c r="A71" s="25"/>
       <c r="B71" s="130"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="174"/>
-      <c r="E71" s="174"/>
+      <c r="D71" s="217"/>
+      <c r="E71" s="217"/>
       <c r="F71" s="67"/>
       <c r="G71" s="1"/>
       <c r="H71" s="50"/>
@@ -3968,10 +3988,10 @@
         <v>91</v>
       </c>
       <c r="Q71" s="65"/>
-      <c r="R71" s="178" t="s">
+      <c r="R71" s="223" t="s">
         <v>6</v>
       </c>
-      <c r="S71" s="178"/>
+      <c r="S71" s="223"/>
       <c r="T71" s="159" t="s">
         <v>92</v>
       </c>
@@ -3983,8 +4003,8 @@
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B72" s="55"/>
       <c r="C72" s="94"/>
-      <c r="D72" s="174"/>
-      <c r="E72" s="174"/>
+      <c r="D72" s="217"/>
+      <c r="E72" s="217"/>
       <c r="F72" s="67"/>
       <c r="I72" s="130"/>
       <c r="L72"/>
@@ -3993,8 +4013,8 @@
       <c r="O72" s="18"/>
       <c r="P72" s="91"/>
       <c r="Q72" s="60"/>
-      <c r="R72" s="171"/>
-      <c r="S72" s="171"/>
+      <c r="R72" s="224"/>
+      <c r="S72" s="224"/>
       <c r="T72" s="69"/>
       <c r="U72" s="100"/>
       <c r="V72" s="55"/>
@@ -4021,10 +4041,10 @@
         <v>96</v>
       </c>
       <c r="Q73" s="60"/>
-      <c r="R73" s="171" t="s">
+      <c r="R73" s="224" t="s">
         <v>10</v>
       </c>
-      <c r="S73" s="171"/>
+      <c r="S73" s="224"/>
       <c r="T73" s="69" t="s">
         <v>97</v>
       </c>
@@ -4038,8 +4058,8 @@
       <c r="O74" s="147"/>
       <c r="P74" s="91"/>
       <c r="Q74" s="60"/>
-      <c r="R74" s="171"/>
-      <c r="S74" s="171"/>
+      <c r="R74" s="224"/>
+      <c r="S74" s="224"/>
       <c r="T74" s="69"/>
       <c r="U74" s="100"/>
       <c r="V74" s="55"/>
@@ -4053,10 +4073,10 @@
       <c r="O75" s="165"/>
       <c r="P75" s="166"/>
       <c r="Q75" s="167"/>
-      <c r="R75" s="176"/>
-      <c r="S75" s="176"/>
-      <c r="T75" s="172"/>
-      <c r="U75" s="173"/>
+      <c r="R75" s="222"/>
+      <c r="S75" s="222"/>
+      <c r="T75" s="225"/>
+      <c r="U75" s="226"/>
       <c r="V75" s="55"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4070,8 +4090,8 @@
       <c r="Q76" s="167"/>
       <c r="R76" s="168"/>
       <c r="S76" s="168"/>
-      <c r="T76" s="172"/>
-      <c r="U76" s="173"/>
+      <c r="T76" s="225"/>
+      <c r="U76" s="226"/>
       <c r="V76" s="55"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4248,29 +4268,51 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="72">
-    <mergeCell ref="T25:U25"/>
-    <mergeCell ref="M22:U22"/>
-    <mergeCell ref="Q26:S26"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="Q29:S29"/>
-    <mergeCell ref="T29:U29"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="T28:U28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="Q28:S28"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="Q27:S27"/>
-    <mergeCell ref="T27:U27"/>
-    <mergeCell ref="N23:S23"/>
-    <mergeCell ref="N24:S24"/>
+  <mergeCells count="80">
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="M69:U69"/>
+    <mergeCell ref="R67:S67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="P67:Q67"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="D44:E44"/>
     <mergeCell ref="M25:N25"/>
     <mergeCell ref="O25:P25"/>
     <mergeCell ref="Q25:S25"/>
@@ -4283,44 +4325,30 @@
     <mergeCell ref="Q34:S34"/>
     <mergeCell ref="O30:P30"/>
     <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="M32:N32"/>
     <mergeCell ref="O32:P32"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M35:O35"/>
     <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="T67:U67"/>
-    <mergeCell ref="M69:U69"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T75:U75"/>
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="M22:U22"/>
+    <mergeCell ref="Q26:S26"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="Q29:S29"/>
+    <mergeCell ref="T29:U29"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="Q28:S28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="Q27:S27"/>
+    <mergeCell ref="T27:U27"/>
+    <mergeCell ref="N23:S23"/>
+    <mergeCell ref="N24:S24"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
cambios en billetes, monedas y detalles nuevo dos
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B92A672-E0C8-47DB-B814-E0CC3621B0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90075A0A-0C6D-49CB-A4E0-D1F4E8A05D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RUTA" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="100">
   <si>
     <t>RECORRIDO</t>
   </si>
@@ -228,9 +228,6 @@
     <t>{{extraction.fecha.valor}}</t>
   </si>
   <si>
-    <t>{{extraction.rendicion.efectivo_total.valor}}</t>
-  </si>
-  <si>
     <t>{{extraction.rendicion.cheques_al_dia.valor}}</t>
   </si>
   <si>
@@ -330,10 +327,13 @@
     <t>{{transf_valor}}</t>
   </si>
   <si>
-    <t>{{extraction.rendicion.cant_fact.valor}}</t>
-  </si>
-  <si>
-    <t>{{extraction.rendicion.valor_total.valor}}</t>
+    <t>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</t>
+  </si>
+  <si>
+    <t>{{extraction.rendicion.detalles_cheques.total_monedas.valor}}</t>
+  </si>
+  <si>
+    <t>{{transf_banco}}</t>
   </si>
 </sst>
 </file>
@@ -1451,15 +1451,6 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1469,6 +1460,9 @@
     <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1481,10 +1475,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1493,12 +1487,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1522,6 +1510,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1556,6 +1550,12 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1590,31 +1590,31 @@
     <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1986,7 +1986,7 @@
         <v>50</v>
       </c>
       <c r="B1" s="127" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C1" s="143"/>
       <c r="D1" s="143"/>
@@ -2015,7 +2015,7 @@
         <v>51</v>
       </c>
       <c r="B2" s="127" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C2" s="143"/>
       <c r="D2" s="143"/>
@@ -2098,7 +2098,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="154" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C5" s="154"/>
       <c r="D5" s="154"/>
@@ -2127,7 +2127,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -2156,7 +2156,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="155" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="155"/>
       <c r="D7" s="155"/>
@@ -2209,11 +2209,11 @@
       <c r="A9" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="174" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="175"/>
-      <c r="D9" s="176"/>
+      <c r="B9" s="171" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="172"/>
+      <c r="D9" s="173"/>
       <c r="E9" s="110"/>
       <c r="F9" s="119"/>
       <c r="G9" s="110"/>
@@ -2238,9 +2238,11 @@
       <c r="A10" s="128" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="119"/>
-      <c r="C10" s="110"/>
-      <c r="D10" s="110"/>
+      <c r="B10" s="171" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="172"/>
+      <c r="D10" s="173"/>
       <c r="E10" s="110"/>
       <c r="F10" s="119"/>
       <c r="G10" s="110"/>
@@ -2265,11 +2267,11 @@
       <c r="A11" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="174" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="175"/>
-      <c r="D11" s="176"/>
+      <c r="B11" s="171" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="172"/>
+      <c r="D11" s="173"/>
       <c r="E11" s="110"/>
       <c r="F11" s="119"/>
       <c r="G11" s="110"/>
@@ -2294,11 +2296,11 @@
       <c r="A12" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="174" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="175"/>
-      <c r="D12" s="176"/>
+      <c r="B12" s="171" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="172"/>
+      <c r="D12" s="173"/>
       <c r="E12" s="110"/>
       <c r="F12" s="119"/>
       <c r="G12" s="110"/>
@@ -2323,11 +2325,11 @@
       <c r="A13" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="174" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="175"/>
-      <c r="D13" s="176"/>
+      <c r="B13" s="171" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="172"/>
+      <c r="D13" s="173"/>
       <c r="E13" s="110"/>
       <c r="F13" s="119"/>
       <c r="G13" s="110"/>
@@ -2352,11 +2354,11 @@
       <c r="A14" s="128" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="174" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="175"/>
-      <c r="D14" s="176"/>
+      <c r="B14" s="171" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="172"/>
+      <c r="D14" s="173"/>
       <c r="E14" s="110"/>
       <c r="F14" s="119"/>
       <c r="G14" s="110"/>
@@ -2381,11 +2383,11 @@
       <c r="A15" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="174" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="175"/>
-      <c r="D15" s="176"/>
+      <c r="B15" s="171" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="172"/>
+      <c r="D15" s="173"/>
       <c r="E15" s="110"/>
       <c r="F15" s="119"/>
       <c r="G15" s="110"/>
@@ -2410,11 +2412,11 @@
       <c r="A16" s="128" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="174" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="175"/>
-      <c r="D16" s="176"/>
+      <c r="B16" s="171" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="172"/>
+      <c r="D16" s="173"/>
       <c r="E16" s="110"/>
       <c r="F16" s="119"/>
       <c r="G16" s="110"/>
@@ -2439,11 +2441,11 @@
       <c r="A17" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="174" t="s">
-        <v>71</v>
-      </c>
-      <c r="C17" s="175"/>
-      <c r="D17" s="176"/>
+      <c r="B17" s="171" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="172"/>
+      <c r="D17" s="173"/>
       <c r="E17" s="110"/>
       <c r="F17" s="119"/>
       <c r="G17" s="110"/>
@@ -2473,7 +2475,7 @@
         <v>0</v>
       </c>
       <c r="C18" s="119">
-        <f t="shared" ref="B18:O18" si="0">SUM(C9:C17)</f>
+        <f t="shared" ref="C18:O18" si="0">SUM(C9:C17)</f>
         <v>0</v>
       </c>
       <c r="D18" s="119">
@@ -2702,17 +2704,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="173" t="s">
+      <c r="M22" s="174" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="173"/>
-      <c r="O22" s="173"/>
-      <c r="P22" s="173"/>
-      <c r="Q22" s="173"/>
-      <c r="R22" s="173"/>
-      <c r="S22" s="173"/>
-      <c r="T22" s="173"/>
-      <c r="U22" s="173"/>
+      <c r="N22" s="174"/>
+      <c r="O22" s="174"/>
+      <c r="P22" s="174"/>
+      <c r="Q22" s="174"/>
+      <c r="R22" s="174"/>
+      <c r="S22" s="174"/>
+      <c r="T22" s="174"/>
+      <c r="U22" s="174"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2721,19 +2723,19 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="189" t="s">
+      <c r="N23" s="185" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="190"/>
-      <c r="P23" s="190"/>
-      <c r="Q23" s="190"/>
-      <c r="R23" s="190"/>
-      <c r="S23" s="191"/>
+      <c r="O23" s="186"/>
+      <c r="P23" s="186"/>
+      <c r="Q23" s="186"/>
+      <c r="R23" s="186"/>
+      <c r="S23" s="187"/>
       <c r="T23" s="142" t="s">
         <v>38</v>
       </c>
       <c r="U23" s="115" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="W23" s="96" t="s">
         <v>44</v>
@@ -2746,23 +2748,23 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="192" t="s">
+      <c r="N24" s="188" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="193"/>
-      <c r="P24" s="193"/>
-      <c r="Q24" s="193"/>
-      <c r="R24" s="193"/>
-      <c r="S24" s="194"/>
+      <c r="O24" s="189"/>
+      <c r="P24" s="189"/>
+      <c r="Q24" s="189"/>
+      <c r="R24" s="189"/>
+      <c r="S24" s="190"/>
       <c r="T24" s="117" t="s">
         <v>11</v>
       </c>
       <c r="U24" s="116" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="W24" s="141" t="str">
         <f>U23</f>
-        <v>{{extraction.rendicion.cant_fact.valor}}</v>
+        <v>{{extraction.cant_fact.valor}}</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
@@ -2774,21 +2776,21 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="195" t="s">
+      <c r="M25" s="193" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="196"/>
-      <c r="O25" s="197"/>
-      <c r="P25" s="198"/>
-      <c r="Q25" s="174" t="s">
-        <v>64</v>
-      </c>
-      <c r="R25" s="175"/>
-      <c r="S25" s="176"/>
-      <c r="T25" s="171" t="s">
+      <c r="N25" s="194"/>
+      <c r="O25" s="195"/>
+      <c r="P25" s="196"/>
+      <c r="Q25" s="171" t="s">
+        <v>97</v>
+      </c>
+      <c r="R25" s="172"/>
+      <c r="S25" s="173"/>
+      <c r="T25" s="191" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="172"/>
+      <c r="U25" s="192"/>
       <c r="V25" s="13"/>
       <c r="W25" s="86" t="s">
         <v>45</v>
@@ -2804,12 +2806,11 @@
       <c r="N26" s="84"/>
       <c r="O26" s="151"/>
       <c r="P26" s="152"/>
-      <c r="Q26" s="174" t="e">
-        <f>B10+C10+D10+E10+F10+G10+H10+I10+J10+K10+L10+N10+O10+P10+Q10+R10+S10+T10+U10+V10+W10+#REF!+#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="R26" s="175"/>
-      <c r="S26" s="176"/>
+      <c r="Q26" s="171" t="s">
+        <v>98</v>
+      </c>
+      <c r="R26" s="172"/>
+      <c r="S26" s="173"/>
       <c r="T26" s="149"/>
       <c r="U26" s="150"/>
       <c r="V26" s="13"/>
@@ -2822,28 +2823,28 @@
       </c>
       <c r="J27" s="162" t="str">
         <f>B9</f>
-        <v>{{extraction.rendicion.efectivo_total.valor}}</v>
+        <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
       <c r="L27"/>
       <c r="M27" s="83" t="s">
         <v>18</v>
       </c>
       <c r="N27" s="84"/>
-      <c r="O27" s="177"/>
-      <c r="P27" s="178"/>
-      <c r="Q27" s="174" t="s">
-        <v>65</v>
-      </c>
-      <c r="R27" s="175"/>
-      <c r="S27" s="176"/>
-      <c r="T27" s="187" t="s">
+      <c r="O27" s="175"/>
+      <c r="P27" s="176"/>
+      <c r="Q27" s="171" t="s">
+        <v>64</v>
+      </c>
+      <c r="R27" s="172"/>
+      <c r="S27" s="173"/>
+      <c r="T27" s="183" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="188"/>
+      <c r="U27" s="184"/>
       <c r="V27" s="19"/>
       <c r="W27" s="97" t="str">
         <f>U24</f>
-        <v>{{extraction.rendicion.valor_total.valor}}</v>
+        <v>{{extraction.valor_total.valor}}</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
@@ -2856,21 +2857,21 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="183" t="s">
+      <c r="M28" s="181" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="184"/>
-      <c r="O28" s="177"/>
-      <c r="P28" s="178"/>
-      <c r="Q28" s="174" t="s">
-        <v>66</v>
-      </c>
-      <c r="R28" s="175"/>
-      <c r="S28" s="176"/>
-      <c r="T28" s="185" t="s">
+      <c r="N28" s="182"/>
+      <c r="O28" s="175"/>
+      <c r="P28" s="176"/>
+      <c r="Q28" s="171" t="s">
+        <v>65</v>
+      </c>
+      <c r="R28" s="172"/>
+      <c r="S28" s="173"/>
+      <c r="T28" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="186"/>
+      <c r="U28" s="180"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2885,24 +2886,24 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="183" t="s">
+      <c r="M29" s="181" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="184"/>
-      <c r="O29" s="177"/>
-      <c r="P29" s="178"/>
-      <c r="Q29" s="174" t="s">
-        <v>67</v>
-      </c>
-      <c r="R29" s="175"/>
-      <c r="S29" s="176"/>
-      <c r="T29" s="179" t="s">
+      <c r="N29" s="182"/>
+      <c r="O29" s="175"/>
+      <c r="P29" s="176"/>
+      <c r="Q29" s="171" t="s">
+        <v>66</v>
+      </c>
+      <c r="R29" s="172"/>
+      <c r="S29" s="173"/>
+      <c r="T29" s="177" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="180"/>
+      <c r="U29" s="178"/>
       <c r="W29" s="98" t="str">
         <f>U23</f>
-        <v>{{extraction.rendicion.cant_fact.valor}}</v>
+        <v>{{extraction.cant_fact.valor}}</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
@@ -2916,21 +2917,21 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="183" t="s">
+      <c r="M30" s="181" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="184"/>
-      <c r="O30" s="177"/>
-      <c r="P30" s="205"/>
-      <c r="Q30" s="174" t="s">
-        <v>68</v>
-      </c>
-      <c r="R30" s="175"/>
-      <c r="S30" s="176"/>
-      <c r="T30" s="181" t="s">
+      <c r="N30" s="182"/>
+      <c r="O30" s="175"/>
+      <c r="P30" s="203"/>
+      <c r="Q30" s="171" t="s">
+        <v>67</v>
+      </c>
+      <c r="R30" s="172"/>
+      <c r="S30" s="173"/>
+      <c r="T30" s="204" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="182"/>
+      <c r="U30" s="205"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2948,17 +2949,17 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="183" t="s">
+      <c r="M31" s="181" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="184"/>
-      <c r="O31" s="177"/>
-      <c r="P31" s="178"/>
-      <c r="Q31" s="174" t="s">
-        <v>69</v>
-      </c>
-      <c r="R31" s="175"/>
-      <c r="S31" s="176"/>
+      <c r="N31" s="182"/>
+      <c r="O31" s="175"/>
+      <c r="P31" s="176"/>
+      <c r="Q31" s="171" t="s">
+        <v>68</v>
+      </c>
+      <c r="R31" s="172"/>
+      <c r="S31" s="173"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2973,17 +2974,17 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="183" t="s">
+      <c r="M32" s="181" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="184"/>
-      <c r="O32" s="177"/>
-      <c r="P32" s="178"/>
-      <c r="Q32" s="174" t="s">
-        <v>70</v>
-      </c>
-      <c r="R32" s="175"/>
-      <c r="S32" s="176"/>
+      <c r="N32" s="182"/>
+      <c r="O32" s="175"/>
+      <c r="P32" s="176"/>
+      <c r="Q32" s="171" t="s">
+        <v>69</v>
+      </c>
+      <c r="R32" s="172"/>
+      <c r="S32" s="173"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="86" t="s">
@@ -3005,13 +3006,13 @@
         <v>25</v>
       </c>
       <c r="N33" s="85"/>
-      <c r="O33" s="177"/>
-      <c r="P33" s="178"/>
-      <c r="Q33" s="174" t="s">
-        <v>71</v>
-      </c>
-      <c r="R33" s="175"/>
-      <c r="S33" s="176"/>
+      <c r="O33" s="175"/>
+      <c r="P33" s="176"/>
+      <c r="Q33" s="171" t="s">
+        <v>70</v>
+      </c>
+      <c r="R33" s="172"/>
+      <c r="S33" s="173"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="138" t="e">
@@ -3030,17 +3031,17 @@
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="201" t="s">
+      <c r="M34" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="202"/>
-      <c r="O34" s="203"/>
-      <c r="P34" s="204"/>
-      <c r="Q34" s="174" t="s">
-        <v>72</v>
-      </c>
-      <c r="R34" s="175"/>
-      <c r="S34" s="176"/>
+      <c r="N34" s="200"/>
+      <c r="O34" s="201"/>
+      <c r="P34" s="202"/>
+      <c r="Q34" s="171" t="s">
+        <v>71</v>
+      </c>
+      <c r="R34" s="172"/>
+      <c r="S34" s="173"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3063,18 +3064,18 @@
       </c>
       <c r="N35" s="210"/>
       <c r="O35" s="211"/>
-      <c r="P35" s="199" t="s">
+      <c r="P35" s="197" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="200"/>
-      <c r="R35" s="199" t="s">
+      <c r="Q35" s="198"/>
+      <c r="R35" s="197" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="200"/>
-      <c r="T35" s="199" t="s">
+      <c r="S35" s="198"/>
+      <c r="T35" s="197" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="200"/>
+      <c r="U35" s="198"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3135,31 +3136,31 @@
       </c>
       <c r="L37"/>
       <c r="M37" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="N37" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="N37" s="38" t="s">
+      <c r="O37" s="39" t="s">
         <v>82</v>
       </c>
-      <c r="O37" s="39" t="s">
+      <c r="P37" s="40" t="s">
         <v>83</v>
       </c>
-      <c r="P37" s="40" t="s">
+      <c r="Q37" s="81" t="s">
         <v>84</v>
       </c>
-      <c r="Q37" s="81" t="s">
+      <c r="R37" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="R37" s="41" t="s">
+      <c r="S37" s="82" t="s">
         <v>86</v>
       </c>
-      <c r="S37" s="82" t="s">
+      <c r="T37" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="T37" s="42" t="s">
+      <c r="U37" s="78" t="s">
         <v>88</v>
-      </c>
-      <c r="U37" s="78" t="s">
-        <v>89</v>
       </c>
       <c r="V37" s="1"/>
       <c r="W37" s="18" t="s">
@@ -3179,7 +3180,7 @@
       </c>
       <c r="N38" s="208"/>
       <c r="O38" s="46" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P38" s="42"/>
       <c r="Q38" s="79"/>
@@ -3484,8 +3485,8 @@
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="43"/>
-      <c r="D51" s="219"/>
-      <c r="E51" s="219"/>
+      <c r="D51" s="220"/>
+      <c r="E51" s="220"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="50"/>
@@ -3508,8 +3509,8 @@
       <c r="A52" s="20"/>
       <c r="B52" s="55"/>
       <c r="C52" s="43"/>
-      <c r="D52" s="218"/>
-      <c r="E52" s="218"/>
+      <c r="D52" s="221"/>
+      <c r="E52" s="221"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="50"/>
@@ -3809,25 +3810,25 @@
       </c>
       <c r="N65" s="208"/>
       <c r="O65" s="46" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P65" s="56" t="s">
         <v>11</v>
       </c>
       <c r="Q65" s="46" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R65" s="56" t="s">
         <v>11</v>
       </c>
       <c r="S65" s="46" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T65" s="56" t="s">
         <v>11</v>
       </c>
       <c r="U65" s="46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="66" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3863,20 +3864,20 @@
       <c r="I67" s="54"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="199" t="s">
+      <c r="M67" s="197" t="s">
         <v>47</v>
       </c>
       <c r="N67" s="216"/>
-      <c r="O67" s="200"/>
-      <c r="P67" s="220"/>
-      <c r="Q67" s="221"/>
-      <c r="R67" s="199" t="s">
+      <c r="O67" s="198"/>
+      <c r="P67" s="218"/>
+      <c r="Q67" s="219"/>
+      <c r="R67" s="197" t="s">
         <v>37</v>
       </c>
       <c r="S67" s="216"/>
       <c r="T67" s="212" t="str">
         <f>Q25</f>
-        <v>{{extraction.rendicion.efectivo_total.valor}}</v>
+        <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
       <c r="U67" s="213"/>
     </row>
@@ -3978,26 +3979,26 @@
       <c r="J71" s="23"/>
       <c r="L71"/>
       <c r="M71" s="63" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N71" s="64"/>
       <c r="O71" s="169" t="s">
         <v>43</v>
       </c>
       <c r="P71" s="66" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q71" s="65"/>
+      <c r="R71" s="226" t="s">
+        <v>6</v>
+      </c>
+      <c r="S71" s="226"/>
+      <c r="T71" s="159" t="s">
         <v>91</v>
-      </c>
-      <c r="Q71" s="65"/>
-      <c r="R71" s="223" t="s">
-        <v>6</v>
-      </c>
-      <c r="S71" s="223"/>
-      <c r="T71" s="159" t="s">
-        <v>92</v>
       </c>
       <c r="U71" s="160"/>
       <c r="V71" s="55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4028,17 +4029,17 @@
       <c r="F73" s="67"/>
       <c r="I73" s="130"/>
       <c r="L73" s="49" t="s">
+        <v>93</v>
+      </c>
+      <c r="M73" s="89" t="s">
         <v>94</v>
-      </c>
-      <c r="M73" s="89" t="s">
-        <v>95</v>
       </c>
       <c r="N73" s="90"/>
       <c r="O73" s="18" t="s">
         <v>43</v>
       </c>
       <c r="P73" s="91" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q73" s="60"/>
       <c r="R73" s="224" t="s">
@@ -4046,9 +4047,11 @@
       </c>
       <c r="S73" s="224"/>
       <c r="T73" s="69" t="s">
-        <v>97</v>
-      </c>
-      <c r="U73" s="100"/>
+        <v>96</v>
+      </c>
+      <c r="U73" s="100" t="s">
+        <v>99</v>
+      </c>
       <c r="V73" s="55"/>
     </row>
     <row r="74" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4073,10 +4076,10 @@
       <c r="O75" s="165"/>
       <c r="P75" s="166"/>
       <c r="Q75" s="167"/>
-      <c r="R75" s="222"/>
-      <c r="S75" s="222"/>
-      <c r="T75" s="225"/>
-      <c r="U75" s="226"/>
+      <c r="R75" s="225"/>
+      <c r="S75" s="225"/>
+      <c r="T75" s="222"/>
+      <c r="U75" s="223"/>
       <c r="V75" s="55"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4090,8 +4093,8 @@
       <c r="Q76" s="167"/>
       <c r="R76" s="168"/>
       <c r="S76" s="168"/>
-      <c r="T76" s="225"/>
-      <c r="U76" s="226"/>
+      <c r="T76" s="222"/>
+      <c r="U76" s="223"/>
       <c r="V76" s="55"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4268,10 +4271,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="80">
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
+  <mergeCells count="81">
     <mergeCell ref="T76:U76"/>
     <mergeCell ref="R74:S74"/>
     <mergeCell ref="B13:D13"/>
@@ -4285,11 +4285,12 @@
     <mergeCell ref="R72:S72"/>
     <mergeCell ref="T75:U75"/>
     <mergeCell ref="M65:N65"/>
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D64:E64"/>
     <mergeCell ref="D71:E71"/>
     <mergeCell ref="D72:E72"/>
     <mergeCell ref="D52:E52"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
     <mergeCell ref="D48:E48"/>
     <mergeCell ref="D49:E49"/>
     <mergeCell ref="D60:E60"/>
@@ -4298,6 +4299,7 @@
     <mergeCell ref="D51:E51"/>
     <mergeCell ref="D65:E65"/>
     <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D64:E64"/>
     <mergeCell ref="T67:U67"/>
     <mergeCell ref="M69:U69"/>
     <mergeCell ref="R67:S67"/>
@@ -4305,7 +4307,7 @@
     <mergeCell ref="D70:E70"/>
     <mergeCell ref="P67:Q67"/>
     <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="M67:O67"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="D46:E46"/>
@@ -4313,9 +4315,11 @@
     <mergeCell ref="M38:N38"/>
     <mergeCell ref="M35:O35"/>
     <mergeCell ref="D44:E44"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="Q25:S25"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="D43:E43"/>
     <mergeCell ref="R35:S35"/>
     <mergeCell ref="T35:U35"/>
     <mergeCell ref="O33:P33"/>
@@ -4323,17 +4327,17 @@
     <mergeCell ref="M34:N34"/>
     <mergeCell ref="O34:P34"/>
     <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="O32:P32"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="O31:P31"/>
     <mergeCell ref="Q31:S31"/>
     <mergeCell ref="M30:N30"/>
     <mergeCell ref="T25:U25"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="Q25:S25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="M22:U22"/>
     <mergeCell ref="Q26:S26"/>
     <mergeCell ref="O29:P29"/>

</xml_diff>

<commit_message>
agrupacion y los grandes
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90075A0A-0C6D-49CB-A4E0-D1F4E8A05D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703A2F14-26FE-40C5-A4C3-CF31C833DAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RUTA" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="100">
   <si>
     <t>RECORRIDO</t>
   </si>
@@ -1011,7 +1011,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="227">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1451,6 +1451,15 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1460,26 +1469,54 @@
     <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1487,28 +1524,37 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1529,93 +1575,56 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2209,11 +2218,11 @@
       <c r="A9" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="171" t="s">
+      <c r="B9" s="227" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="172"/>
-      <c r="D9" s="173"/>
+      <c r="C9" s="228"/>
+      <c r="D9" s="229"/>
       <c r="E9" s="110"/>
       <c r="F9" s="119"/>
       <c r="G9" s="110"/>
@@ -2238,11 +2247,11 @@
       <c r="A10" s="128" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="171" t="s">
+      <c r="B10" s="227" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="172"/>
-      <c r="D10" s="173"/>
+      <c r="C10" s="228"/>
+      <c r="D10" s="229"/>
       <c r="E10" s="110"/>
       <c r="F10" s="119"/>
       <c r="G10" s="110"/>
@@ -2267,11 +2276,11 @@
       <c r="A11" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="171" t="s">
+      <c r="B11" s="227" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="172"/>
-      <c r="D11" s="173"/>
+      <c r="C11" s="228"/>
+      <c r="D11" s="229"/>
       <c r="E11" s="110"/>
       <c r="F11" s="119"/>
       <c r="G11" s="110"/>
@@ -2296,11 +2305,11 @@
       <c r="A12" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="171" t="s">
+      <c r="B12" s="227" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="172"/>
-      <c r="D12" s="173"/>
+      <c r="C12" s="228"/>
+      <c r="D12" s="229"/>
       <c r="E12" s="110"/>
       <c r="F12" s="119"/>
       <c r="G12" s="110"/>
@@ -2325,11 +2334,11 @@
       <c r="A13" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="171" t="s">
+      <c r="B13" s="227" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="172"/>
-      <c r="D13" s="173"/>
+      <c r="C13" s="228"/>
+      <c r="D13" s="229"/>
       <c r="E13" s="110"/>
       <c r="F13" s="119"/>
       <c r="G13" s="110"/>
@@ -2354,11 +2363,11 @@
       <c r="A14" s="128" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="171" t="s">
+      <c r="B14" s="227" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="172"/>
-      <c r="D14" s="173"/>
+      <c r="C14" s="228"/>
+      <c r="D14" s="229"/>
       <c r="E14" s="110"/>
       <c r="F14" s="119"/>
       <c r="G14" s="110"/>
@@ -2383,11 +2392,11 @@
       <c r="A15" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="171" t="s">
+      <c r="B15" s="227" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="172"/>
-      <c r="D15" s="173"/>
+      <c r="C15" s="228"/>
+      <c r="D15" s="229"/>
       <c r="E15" s="110"/>
       <c r="F15" s="119"/>
       <c r="G15" s="110"/>
@@ -2412,11 +2421,11 @@
       <c r="A16" s="128" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="171" t="s">
+      <c r="B16" s="227" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="172"/>
-      <c r="D16" s="173"/>
+      <c r="C16" s="228"/>
+      <c r="D16" s="229"/>
       <c r="E16" s="110"/>
       <c r="F16" s="119"/>
       <c r="G16" s="110"/>
@@ -2441,11 +2450,11 @@
       <c r="A17" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="171" t="s">
+      <c r="B17" s="227" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="172"/>
-      <c r="D17" s="173"/>
+      <c r="C17" s="228"/>
+      <c r="D17" s="229"/>
       <c r="E17" s="110"/>
       <c r="F17" s="119"/>
       <c r="G17" s="110"/>
@@ -2704,17 +2713,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="174" t="s">
+      <c r="M22" s="214" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="174"/>
-      <c r="O22" s="174"/>
-      <c r="P22" s="174"/>
-      <c r="Q22" s="174"/>
-      <c r="R22" s="174"/>
-      <c r="S22" s="174"/>
-      <c r="T22" s="174"/>
-      <c r="U22" s="174"/>
+      <c r="N22" s="214"/>
+      <c r="O22" s="214"/>
+      <c r="P22" s="214"/>
+      <c r="Q22" s="214"/>
+      <c r="R22" s="214"/>
+      <c r="S22" s="214"/>
+      <c r="T22" s="214"/>
+      <c r="U22" s="214"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2723,14 +2732,14 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="185" t="s">
+      <c r="N23" s="221" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="186"/>
-      <c r="P23" s="186"/>
-      <c r="Q23" s="186"/>
-      <c r="R23" s="186"/>
-      <c r="S23" s="187"/>
+      <c r="O23" s="222"/>
+      <c r="P23" s="222"/>
+      <c r="Q23" s="222"/>
+      <c r="R23" s="222"/>
+      <c r="S23" s="223"/>
       <c r="T23" s="142" t="s">
         <v>38</v>
       </c>
@@ -2748,23 +2757,22 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="188" t="s">
+      <c r="N24" s="224" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="189"/>
-      <c r="P24" s="189"/>
-      <c r="Q24" s="189"/>
-      <c r="R24" s="189"/>
-      <c r="S24" s="190"/>
+      <c r="O24" s="225"/>
+      <c r="P24" s="225"/>
+      <c r="Q24" s="225"/>
+      <c r="R24" s="225"/>
+      <c r="S24" s="226"/>
       <c r="T24" s="117" t="s">
         <v>11</v>
       </c>
       <c r="U24" s="116" t="s">
         <v>79</v>
       </c>
-      <c r="W24" s="141" t="str">
-        <f>U23</f>
-        <v>{{extraction.cant_fact.valor}}</v>
+      <c r="W24" s="141" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
@@ -2776,21 +2784,21 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="193" t="s">
+      <c r="M25" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="194"/>
-      <c r="O25" s="195"/>
-      <c r="P25" s="196"/>
-      <c r="Q25" s="171" t="s">
+      <c r="N25" s="210"/>
+      <c r="O25" s="211"/>
+      <c r="P25" s="212"/>
+      <c r="Q25" s="174" t="s">
         <v>97</v>
       </c>
-      <c r="R25" s="172"/>
-      <c r="S25" s="173"/>
-      <c r="T25" s="191" t="s">
+      <c r="R25" s="175"/>
+      <c r="S25" s="176"/>
+      <c r="T25" s="207" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="192"/>
+      <c r="U25" s="208"/>
       <c r="V25" s="13"/>
       <c r="W25" s="86" t="s">
         <v>45</v>
@@ -2806,11 +2814,11 @@
       <c r="N26" s="84"/>
       <c r="O26" s="151"/>
       <c r="P26" s="152"/>
-      <c r="Q26" s="171" t="s">
+      <c r="Q26" s="174" t="s">
         <v>98</v>
       </c>
-      <c r="R26" s="172"/>
-      <c r="S26" s="173"/>
+      <c r="R26" s="175"/>
+      <c r="S26" s="176"/>
       <c r="T26" s="149"/>
       <c r="U26" s="150"/>
       <c r="V26" s="13"/>
@@ -2830,21 +2838,20 @@
         <v>18</v>
       </c>
       <c r="N27" s="84"/>
-      <c r="O27" s="175"/>
-      <c r="P27" s="176"/>
-      <c r="Q27" s="171" t="s">
+      <c r="O27" s="199"/>
+      <c r="P27" s="200"/>
+      <c r="Q27" s="174" t="s">
         <v>64</v>
       </c>
-      <c r="R27" s="172"/>
-      <c r="S27" s="173"/>
-      <c r="T27" s="183" t="s">
+      <c r="R27" s="175"/>
+      <c r="S27" s="176"/>
+      <c r="T27" s="219" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="184"/>
+      <c r="U27" s="220"/>
       <c r="V27" s="19"/>
-      <c r="W27" s="97" t="str">
-        <f>U24</f>
-        <v>{{extraction.valor_total.valor}}</v>
+      <c r="W27" s="97" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
@@ -2857,21 +2864,21 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="181" t="s">
+      <c r="M28" s="194" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="182"/>
-      <c r="O28" s="175"/>
-      <c r="P28" s="176"/>
-      <c r="Q28" s="171" t="s">
+      <c r="N28" s="195"/>
+      <c r="O28" s="199"/>
+      <c r="P28" s="200"/>
+      <c r="Q28" s="174" t="s">
         <v>65</v>
       </c>
-      <c r="R28" s="172"/>
-      <c r="S28" s="173"/>
-      <c r="T28" s="179" t="s">
+      <c r="R28" s="175"/>
+      <c r="S28" s="176"/>
+      <c r="T28" s="217" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="180"/>
+      <c r="U28" s="218"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2886,21 +2893,21 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="181" t="s">
+      <c r="M29" s="194" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="182"/>
-      <c r="O29" s="175"/>
-      <c r="P29" s="176"/>
-      <c r="Q29" s="171" t="s">
+      <c r="N29" s="195"/>
+      <c r="O29" s="199"/>
+      <c r="P29" s="200"/>
+      <c r="Q29" s="174" t="s">
         <v>66</v>
       </c>
-      <c r="R29" s="172"/>
-      <c r="S29" s="173"/>
-      <c r="T29" s="177" t="s">
+      <c r="R29" s="175"/>
+      <c r="S29" s="176"/>
+      <c r="T29" s="215" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="178"/>
+      <c r="U29" s="216"/>
       <c r="W29" s="98" t="str">
         <f>U23</f>
         <v>{{extraction.cant_fact.valor}}</v>
@@ -2917,21 +2924,21 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="181" t="s">
+      <c r="M30" s="194" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="182"/>
-      <c r="O30" s="175"/>
-      <c r="P30" s="203"/>
-      <c r="Q30" s="171" t="s">
+      <c r="N30" s="195"/>
+      <c r="O30" s="199"/>
+      <c r="P30" s="213"/>
+      <c r="Q30" s="174" t="s">
         <v>67</v>
       </c>
-      <c r="R30" s="172"/>
-      <c r="S30" s="173"/>
-      <c r="T30" s="204" t="s">
+      <c r="R30" s="175"/>
+      <c r="S30" s="176"/>
+      <c r="T30" s="201" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="205"/>
+      <c r="U30" s="202"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2949,17 +2956,17 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="181" t="s">
+      <c r="M31" s="194" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="182"/>
-      <c r="O31" s="175"/>
-      <c r="P31" s="176"/>
-      <c r="Q31" s="171" t="s">
+      <c r="N31" s="195"/>
+      <c r="O31" s="199"/>
+      <c r="P31" s="200"/>
+      <c r="Q31" s="174" t="s">
         <v>68</v>
       </c>
-      <c r="R31" s="172"/>
-      <c r="S31" s="173"/>
+      <c r="R31" s="175"/>
+      <c r="S31" s="176"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2974,17 +2981,17 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="181" t="s">
+      <c r="M32" s="194" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="182"/>
-      <c r="O32" s="175"/>
-      <c r="P32" s="176"/>
-      <c r="Q32" s="171" t="s">
+      <c r="N32" s="195"/>
+      <c r="O32" s="199"/>
+      <c r="P32" s="200"/>
+      <c r="Q32" s="174" t="s">
         <v>69</v>
       </c>
-      <c r="R32" s="172"/>
-      <c r="S32" s="173"/>
+      <c r="R32" s="175"/>
+      <c r="S32" s="176"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="86" t="s">
@@ -3006,13 +3013,13 @@
         <v>25</v>
       </c>
       <c r="N33" s="85"/>
-      <c r="O33" s="175"/>
-      <c r="P33" s="176"/>
-      <c r="Q33" s="171" t="s">
+      <c r="O33" s="199"/>
+      <c r="P33" s="200"/>
+      <c r="Q33" s="174" t="s">
         <v>70</v>
       </c>
-      <c r="R33" s="172"/>
-      <c r="S33" s="173"/>
+      <c r="R33" s="175"/>
+      <c r="S33" s="176"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="138" t="e">
@@ -3031,17 +3038,17 @@
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="199" t="s">
+      <c r="M34" s="203" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="200"/>
-      <c r="O34" s="201"/>
-      <c r="P34" s="202"/>
-      <c r="Q34" s="171" t="s">
+      <c r="N34" s="204"/>
+      <c r="O34" s="205"/>
+      <c r="P34" s="206"/>
+      <c r="Q34" s="174" t="s">
         <v>71</v>
       </c>
-      <c r="R34" s="172"/>
-      <c r="S34" s="173"/>
+      <c r="R34" s="175"/>
+      <c r="S34" s="176"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3059,23 +3066,23 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="209" t="s">
+      <c r="M35" s="196" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="210"/>
-      <c r="O35" s="211"/>
-      <c r="P35" s="197" t="s">
+      <c r="N35" s="197"/>
+      <c r="O35" s="198"/>
+      <c r="P35" s="189" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="198"/>
-      <c r="R35" s="197" t="s">
+      <c r="Q35" s="193"/>
+      <c r="R35" s="189" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="198"/>
-      <c r="T35" s="197" t="s">
+      <c r="S35" s="193"/>
+      <c r="T35" s="189" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="198"/>
+      <c r="U35" s="193"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3175,10 +3182,10 @@
       <c r="L38" s="114">
         <v>2</v>
       </c>
-      <c r="M38" s="207" t="s">
+      <c r="M38" s="179" t="s">
         <v>42</v>
       </c>
-      <c r="N38" s="208"/>
+      <c r="N38" s="180"/>
       <c r="O38" s="46" t="s">
         <v>64</v>
       </c>
@@ -3288,8 +3295,8 @@
       <c r="A43" s="112"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="206"/>
-      <c r="E43" s="206"/>
+      <c r="D43" s="183"/>
+      <c r="E43" s="183"/>
       <c r="F43" s="51"/>
       <c r="G43" s="8"/>
       <c r="I43" s="136"/>
@@ -3315,8 +3322,8 @@
       <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="206"/>
-      <c r="E44" s="206"/>
+      <c r="D44" s="183"/>
+      <c r="E44" s="183"/>
       <c r="F44" s="52"/>
       <c r="H44" s="68"/>
       <c r="I44" s="13"/>
@@ -3339,8 +3346,8 @@
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="43"/>
-      <c r="D45" s="206"/>
-      <c r="E45" s="206"/>
+      <c r="D45" s="183"/>
+      <c r="E45" s="183"/>
       <c r="F45" s="23"/>
       <c r="H45" s="68"/>
       <c r="I45" s="13"/>
@@ -3362,8 +3369,8 @@
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="43"/>
-      <c r="D46" s="206"/>
-      <c r="E46" s="206"/>
+      <c r="D46" s="183"/>
+      <c r="E46" s="183"/>
       <c r="F46" s="53"/>
       <c r="H46" s="68"/>
       <c r="I46" s="13"/>
@@ -3385,8 +3392,8 @@
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="43"/>
-      <c r="D47" s="206"/>
-      <c r="E47" s="206"/>
+      <c r="D47" s="183"/>
+      <c r="E47" s="183"/>
       <c r="F47" s="17"/>
       <c r="G47" s="1"/>
       <c r="H47" s="68"/>
@@ -3413,8 +3420,8 @@
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="43"/>
-      <c r="D48" s="206"/>
-      <c r="E48" s="206"/>
+      <c r="D48" s="183"/>
+      <c r="E48" s="183"/>
       <c r="F48" s="23"/>
       <c r="G48" s="1"/>
       <c r="H48" s="68"/>
@@ -3437,8 +3444,8 @@
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="43"/>
-      <c r="D49" s="206"/>
-      <c r="E49" s="206"/>
+      <c r="D49" s="183"/>
+      <c r="E49" s="183"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
       <c r="H49" s="50"/>
@@ -3485,8 +3492,8 @@
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="43"/>
-      <c r="D51" s="220"/>
-      <c r="E51" s="220"/>
+      <c r="D51" s="184"/>
+      <c r="E51" s="184"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="50"/>
@@ -3509,8 +3516,8 @@
       <c r="A52" s="20"/>
       <c r="B52" s="55"/>
       <c r="C52" s="43"/>
-      <c r="D52" s="221"/>
-      <c r="E52" s="221"/>
+      <c r="D52" s="182"/>
+      <c r="E52" s="182"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="50"/>
@@ -3533,8 +3540,8 @@
       <c r="A53" s="25"/>
       <c r="B53" s="55"/>
       <c r="C53" s="43"/>
-      <c r="D53" s="217"/>
-      <c r="E53" s="217"/>
+      <c r="D53" s="181"/>
+      <c r="E53" s="181"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="50"/>
@@ -3555,8 +3562,8 @@
       <c r="A54" s="20"/>
       <c r="B54" s="55"/>
       <c r="C54" s="43"/>
-      <c r="D54" s="217"/>
-      <c r="E54" s="217"/>
+      <c r="D54" s="181"/>
+      <c r="E54" s="181"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="50"/>
@@ -3687,8 +3694,8 @@
       <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="43"/>
-      <c r="D60" s="217"/>
-      <c r="E60" s="217"/>
+      <c r="D60" s="181"/>
+      <c r="E60" s="181"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="50"/>
@@ -3775,8 +3782,8 @@
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="43"/>
-      <c r="D64" s="217"/>
-      <c r="E64" s="217"/>
+      <c r="D64" s="181"/>
+      <c r="E64" s="181"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="50"/>
@@ -3797,18 +3804,18 @@
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="43"/>
-      <c r="D65" s="217"/>
-      <c r="E65" s="217"/>
+      <c r="D65" s="181"/>
+      <c r="E65" s="181"/>
       <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="50"/>
       <c r="I65" s="54"/>
       <c r="J65" s="57"/>
       <c r="L65"/>
-      <c r="M65" s="207" t="s">
+      <c r="M65" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="N65" s="208"/>
+      <c r="N65" s="180"/>
       <c r="O65" s="46" t="s">
         <v>65</v>
       </c>
@@ -3835,8 +3842,8 @@
       <c r="A66" s="25"/>
       <c r="B66"/>
       <c r="C66" s="95"/>
-      <c r="D66" s="217"/>
-      <c r="E66" s="217"/>
+      <c r="D66" s="181"/>
+      <c r="E66" s="181"/>
       <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="50"/>
@@ -3864,29 +3871,29 @@
       <c r="I67" s="54"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="197" t="s">
+      <c r="M67" s="189" t="s">
         <v>47</v>
       </c>
-      <c r="N67" s="216"/>
-      <c r="O67" s="198"/>
-      <c r="P67" s="218"/>
-      <c r="Q67" s="219"/>
-      <c r="R67" s="197" t="s">
+      <c r="N67" s="190"/>
+      <c r="O67" s="193"/>
+      <c r="P67" s="191"/>
+      <c r="Q67" s="192"/>
+      <c r="R67" s="189" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="216"/>
-      <c r="T67" s="212" t="str">
+      <c r="S67" s="190"/>
+      <c r="T67" s="185" t="str">
         <f>Q25</f>
         <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
-      <c r="U67" s="213"/>
+      <c r="U67" s="186"/>
     </row>
     <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="217"/>
-      <c r="E68" s="217"/>
+      <c r="D68" s="181"/>
+      <c r="E68" s="181"/>
       <c r="F68" s="67"/>
       <c r="G68" s="1"/>
       <c r="H68" s="50"/>
@@ -3907,33 +3914,33 @@
       <c r="A69" s="25"/>
       <c r="B69" s="95"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="217"/>
-      <c r="E69" s="217"/>
+      <c r="D69" s="181"/>
+      <c r="E69" s="181"/>
       <c r="F69" s="67"/>
       <c r="G69" s="1"/>
       <c r="H69" s="50"/>
       <c r="I69" s="54"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="207" t="s">
+      <c r="M69" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="N69" s="214"/>
-      <c r="O69" s="214"/>
-      <c r="P69" s="214"/>
-      <c r="Q69" s="214"/>
-      <c r="R69" s="214"/>
-      <c r="S69" s="214"/>
-      <c r="T69" s="214"/>
-      <c r="U69" s="215"/>
+      <c r="N69" s="187"/>
+      <c r="O69" s="187"/>
+      <c r="P69" s="187"/>
+      <c r="Q69" s="187"/>
+      <c r="R69" s="187"/>
+      <c r="S69" s="187"/>
+      <c r="T69" s="187"/>
+      <c r="U69" s="188"/>
       <c r="V69" s="55"/>
     </row>
     <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
       <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="217"/>
-      <c r="E70" s="217"/>
+      <c r="D70" s="181"/>
+      <c r="E70" s="181"/>
       <c r="F70" s="67"/>
       <c r="G70" s="1"/>
       <c r="H70" s="50"/>
@@ -3970,8 +3977,8 @@
       <c r="A71" s="25"/>
       <c r="B71" s="130"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="217"/>
-      <c r="E71" s="217"/>
+      <c r="D71" s="181"/>
+      <c r="E71" s="181"/>
       <c r="F71" s="67"/>
       <c r="G71" s="1"/>
       <c r="H71" s="50"/>
@@ -3989,10 +3996,10 @@
         <v>90</v>
       </c>
       <c r="Q71" s="65"/>
-      <c r="R71" s="226" t="s">
+      <c r="R71" s="178" t="s">
         <v>6</v>
       </c>
-      <c r="S71" s="226"/>
+      <c r="S71" s="178"/>
       <c r="T71" s="159" t="s">
         <v>91</v>
       </c>
@@ -4004,8 +4011,8 @@
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B72" s="55"/>
       <c r="C72" s="94"/>
-      <c r="D72" s="217"/>
-      <c r="E72" s="217"/>
+      <c r="D72" s="181"/>
+      <c r="E72" s="181"/>
       <c r="F72" s="67"/>
       <c r="I72" s="130"/>
       <c r="L72"/>
@@ -4014,8 +4021,8 @@
       <c r="O72" s="18"/>
       <c r="P72" s="91"/>
       <c r="Q72" s="60"/>
-      <c r="R72" s="224"/>
-      <c r="S72" s="224"/>
+      <c r="R72" s="173"/>
+      <c r="S72" s="173"/>
       <c r="T72" s="69"/>
       <c r="U72" s="100"/>
       <c r="V72" s="55"/>
@@ -4042,10 +4049,10 @@
         <v>95</v>
       </c>
       <c r="Q73" s="60"/>
-      <c r="R73" s="224" t="s">
+      <c r="R73" s="173" t="s">
         <v>10</v>
       </c>
-      <c r="S73" s="224"/>
+      <c r="S73" s="173"/>
       <c r="T73" s="69" t="s">
         <v>96</v>
       </c>
@@ -4061,8 +4068,8 @@
       <c r="O74" s="147"/>
       <c r="P74" s="91"/>
       <c r="Q74" s="60"/>
-      <c r="R74" s="224"/>
-      <c r="S74" s="224"/>
+      <c r="R74" s="173"/>
+      <c r="S74" s="173"/>
       <c r="T74" s="69"/>
       <c r="U74" s="100"/>
       <c r="V74" s="55"/>
@@ -4076,10 +4083,10 @@
       <c r="O75" s="165"/>
       <c r="P75" s="166"/>
       <c r="Q75" s="167"/>
-      <c r="R75" s="225"/>
-      <c r="S75" s="225"/>
-      <c r="T75" s="222"/>
-      <c r="U75" s="223"/>
+      <c r="R75" s="177"/>
+      <c r="S75" s="177"/>
+      <c r="T75" s="171"/>
+      <c r="U75" s="172"/>
       <c r="V75" s="55"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4093,8 +4100,8 @@
       <c r="Q76" s="167"/>
       <c r="R76" s="168"/>
       <c r="S76" s="168"/>
-      <c r="T76" s="222"/>
-      <c r="U76" s="223"/>
+      <c r="T76" s="171"/>
+      <c r="U76" s="172"/>
       <c r="V76" s="55"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4271,73 +4278,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="81">
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T75:U75"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="T67:U67"/>
-    <mergeCell ref="M69:U69"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="O32:P32"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="T25:U25"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="Q25:S25"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="B10:D10"/>
+  <mergeCells count="72">
     <mergeCell ref="M22:U22"/>
     <mergeCell ref="Q26:S26"/>
     <mergeCell ref="O29:P29"/>
@@ -4353,6 +4294,63 @@
     <mergeCell ref="T27:U27"/>
     <mergeCell ref="N23:S23"/>
     <mergeCell ref="N24:S24"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="Q25:S25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="M69:U69"/>
+    <mergeCell ref="R67:S67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="P67:Q67"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D52:E52"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
cambios con ia y excel
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703A2F14-26FE-40C5-A4C3-CF31C833DAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4471384-CCBC-42F4-ACE5-5288FF607315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="103">
   <si>
     <t>RECORRIDO</t>
   </si>
@@ -334,6 +334,15 @@
   </si>
   <si>
     <t>{{transf_banco}}</t>
+  </si>
+  <si>
+    <t>{{chq_dia_fechas}}</t>
+  </si>
+  <si>
+    <t>{{chq_dia_bancos}}</t>
+  </si>
+  <si>
+    <t>{{chq_dia_valores}}</t>
   </si>
 </sst>
 </file>
@@ -1451,13 +1460,16 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1469,162 +1481,159 @@
     <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="5" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2218,11 +2227,11 @@
       <c r="A9" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="227" t="s">
+      <c r="B9" s="171" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="228"/>
-      <c r="D9" s="229"/>
+      <c r="C9" s="172"/>
+      <c r="D9" s="173"/>
       <c r="E9" s="110"/>
       <c r="F9" s="119"/>
       <c r="G9" s="110"/>
@@ -2247,11 +2256,11 @@
       <c r="A10" s="128" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="227" t="s">
+      <c r="B10" s="171" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="228"/>
-      <c r="D10" s="229"/>
+      <c r="C10" s="172"/>
+      <c r="D10" s="173"/>
       <c r="E10" s="110"/>
       <c r="F10" s="119"/>
       <c r="G10" s="110"/>
@@ -2276,11 +2285,11 @@
       <c r="A11" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="227" t="s">
+      <c r="B11" s="171" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="228"/>
-      <c r="D11" s="229"/>
+      <c r="C11" s="172"/>
+      <c r="D11" s="173"/>
       <c r="E11" s="110"/>
       <c r="F11" s="119"/>
       <c r="G11" s="110"/>
@@ -2305,11 +2314,11 @@
       <c r="A12" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="227" t="s">
+      <c r="B12" s="171" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="228"/>
-      <c r="D12" s="229"/>
+      <c r="C12" s="172"/>
+      <c r="D12" s="173"/>
       <c r="E12" s="110"/>
       <c r="F12" s="119"/>
       <c r="G12" s="110"/>
@@ -2334,11 +2343,11 @@
       <c r="A13" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="227" t="s">
+      <c r="B13" s="171" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="228"/>
-      <c r="D13" s="229"/>
+      <c r="C13" s="172"/>
+      <c r="D13" s="173"/>
       <c r="E13" s="110"/>
       <c r="F13" s="119"/>
       <c r="G13" s="110"/>
@@ -2363,11 +2372,11 @@
       <c r="A14" s="128" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="227" t="s">
+      <c r="B14" s="171" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="228"/>
-      <c r="D14" s="229"/>
+      <c r="C14" s="172"/>
+      <c r="D14" s="173"/>
       <c r="E14" s="110"/>
       <c r="F14" s="119"/>
       <c r="G14" s="110"/>
@@ -2392,11 +2401,11 @@
       <c r="A15" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="227" t="s">
+      <c r="B15" s="171" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="228"/>
-      <c r="D15" s="229"/>
+      <c r="C15" s="172"/>
+      <c r="D15" s="173"/>
       <c r="E15" s="110"/>
       <c r="F15" s="119"/>
       <c r="G15" s="110"/>
@@ -2421,11 +2430,11 @@
       <c r="A16" s="128" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="227" t="s">
+      <c r="B16" s="171" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="228"/>
-      <c r="D16" s="229"/>
+      <c r="C16" s="172"/>
+      <c r="D16" s="173"/>
       <c r="E16" s="110"/>
       <c r="F16" s="119"/>
       <c r="G16" s="110"/>
@@ -2450,11 +2459,11 @@
       <c r="A17" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="227" t="s">
+      <c r="B17" s="171" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="228"/>
-      <c r="D17" s="229"/>
+      <c r="C17" s="172"/>
+      <c r="D17" s="173"/>
       <c r="E17" s="110"/>
       <c r="F17" s="119"/>
       <c r="G17" s="110"/>
@@ -2713,17 +2722,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="214" t="s">
+      <c r="M22" s="174" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="214"/>
-      <c r="O22" s="214"/>
-      <c r="P22" s="214"/>
-      <c r="Q22" s="214"/>
-      <c r="R22" s="214"/>
-      <c r="S22" s="214"/>
-      <c r="T22" s="214"/>
-      <c r="U22" s="214"/>
+      <c r="N22" s="174"/>
+      <c r="O22" s="174"/>
+      <c r="P22" s="174"/>
+      <c r="Q22" s="174"/>
+      <c r="R22" s="174"/>
+      <c r="S22" s="174"/>
+      <c r="T22" s="174"/>
+      <c r="U22" s="174"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2732,14 +2741,14 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="221" t="s">
+      <c r="N23" s="188" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="222"/>
-      <c r="P23" s="222"/>
-      <c r="Q23" s="222"/>
-      <c r="R23" s="222"/>
-      <c r="S23" s="223"/>
+      <c r="O23" s="189"/>
+      <c r="P23" s="189"/>
+      <c r="Q23" s="189"/>
+      <c r="R23" s="189"/>
+      <c r="S23" s="190"/>
       <c r="T23" s="142" t="s">
         <v>38</v>
       </c>
@@ -2757,14 +2766,14 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="224" t="s">
+      <c r="N24" s="191" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="225"/>
-      <c r="P24" s="225"/>
-      <c r="Q24" s="225"/>
-      <c r="R24" s="225"/>
-      <c r="S24" s="226"/>
+      <c r="O24" s="192"/>
+      <c r="P24" s="192"/>
+      <c r="Q24" s="192"/>
+      <c r="R24" s="192"/>
+      <c r="S24" s="193"/>
       <c r="T24" s="117" t="s">
         <v>11</v>
       </c>
@@ -2784,21 +2793,21 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="209" t="s">
+      <c r="M25" s="196" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="210"/>
-      <c r="O25" s="211"/>
-      <c r="P25" s="212"/>
-      <c r="Q25" s="174" t="s">
+      <c r="N25" s="197"/>
+      <c r="O25" s="198"/>
+      <c r="P25" s="199"/>
+      <c r="Q25" s="175" t="s">
         <v>97</v>
       </c>
-      <c r="R25" s="175"/>
-      <c r="S25" s="176"/>
-      <c r="T25" s="207" t="s">
+      <c r="R25" s="176"/>
+      <c r="S25" s="177"/>
+      <c r="T25" s="194" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="208"/>
+      <c r="U25" s="195"/>
       <c r="V25" s="13"/>
       <c r="W25" s="86" t="s">
         <v>45</v>
@@ -2814,11 +2823,11 @@
       <c r="N26" s="84"/>
       <c r="O26" s="151"/>
       <c r="P26" s="152"/>
-      <c r="Q26" s="174" t="s">
+      <c r="Q26" s="175" t="s">
         <v>98</v>
       </c>
-      <c r="R26" s="175"/>
-      <c r="S26" s="176"/>
+      <c r="R26" s="176"/>
+      <c r="S26" s="177"/>
       <c r="T26" s="149"/>
       <c r="U26" s="150"/>
       <c r="V26" s="13"/>
@@ -2838,17 +2847,17 @@
         <v>18</v>
       </c>
       <c r="N27" s="84"/>
-      <c r="O27" s="199"/>
-      <c r="P27" s="200"/>
-      <c r="Q27" s="174" t="s">
+      <c r="O27" s="178"/>
+      <c r="P27" s="179"/>
+      <c r="Q27" s="175" t="s">
         <v>64</v>
       </c>
-      <c r="R27" s="175"/>
-      <c r="S27" s="176"/>
-      <c r="T27" s="219" t="s">
+      <c r="R27" s="176"/>
+      <c r="S27" s="177"/>
+      <c r="T27" s="186" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="220"/>
+      <c r="U27" s="187"/>
       <c r="V27" s="19"/>
       <c r="W27" s="97" t="s">
         <v>79</v>
@@ -2864,21 +2873,21 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="194" t="s">
+      <c r="M28" s="184" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="195"/>
-      <c r="O28" s="199"/>
-      <c r="P28" s="200"/>
-      <c r="Q28" s="174" t="s">
+      <c r="N28" s="185"/>
+      <c r="O28" s="178"/>
+      <c r="P28" s="179"/>
+      <c r="Q28" s="175" t="s">
         <v>65</v>
       </c>
-      <c r="R28" s="175"/>
-      <c r="S28" s="176"/>
-      <c r="T28" s="217" t="s">
+      <c r="R28" s="176"/>
+      <c r="S28" s="177"/>
+      <c r="T28" s="182" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="218"/>
+      <c r="U28" s="183"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2893,21 +2902,21 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="194" t="s">
+      <c r="M29" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="195"/>
-      <c r="O29" s="199"/>
-      <c r="P29" s="200"/>
-      <c r="Q29" s="174" t="s">
+      <c r="N29" s="185"/>
+      <c r="O29" s="178"/>
+      <c r="P29" s="179"/>
+      <c r="Q29" s="175" t="s">
         <v>66</v>
       </c>
-      <c r="R29" s="175"/>
-      <c r="S29" s="176"/>
-      <c r="T29" s="215" t="s">
+      <c r="R29" s="176"/>
+      <c r="S29" s="177"/>
+      <c r="T29" s="180" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="216"/>
+      <c r="U29" s="181"/>
       <c r="W29" s="98" t="str">
         <f>U23</f>
         <v>{{extraction.cant_fact.valor}}</v>
@@ -2924,17 +2933,17 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="194" t="s">
+      <c r="M30" s="184" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="195"/>
-      <c r="O30" s="199"/>
-      <c r="P30" s="213"/>
-      <c r="Q30" s="174" t="s">
+      <c r="N30" s="185"/>
+      <c r="O30" s="178"/>
+      <c r="P30" s="200"/>
+      <c r="Q30" s="175" t="s">
         <v>67</v>
       </c>
-      <c r="R30" s="175"/>
-      <c r="S30" s="176"/>
+      <c r="R30" s="176"/>
+      <c r="S30" s="177"/>
       <c r="T30" s="201" t="s">
         <v>41</v>
       </c>
@@ -2956,17 +2965,17 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="194" t="s">
+      <c r="M31" s="184" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="195"/>
-      <c r="O31" s="199"/>
-      <c r="P31" s="200"/>
-      <c r="Q31" s="174" t="s">
+      <c r="N31" s="185"/>
+      <c r="O31" s="178"/>
+      <c r="P31" s="179"/>
+      <c r="Q31" s="175" t="s">
         <v>68</v>
       </c>
-      <c r="R31" s="175"/>
-      <c r="S31" s="176"/>
+      <c r="R31" s="176"/>
+      <c r="S31" s="177"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2981,17 +2990,17 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="194" t="s">
+      <c r="M32" s="184" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="195"/>
-      <c r="O32" s="199"/>
-      <c r="P32" s="200"/>
-      <c r="Q32" s="174" t="s">
+      <c r="N32" s="185"/>
+      <c r="O32" s="178"/>
+      <c r="P32" s="179"/>
+      <c r="Q32" s="175" t="s">
         <v>69</v>
       </c>
-      <c r="R32" s="175"/>
-      <c r="S32" s="176"/>
+      <c r="R32" s="176"/>
+      <c r="S32" s="177"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="86" t="s">
@@ -3013,13 +3022,13 @@
         <v>25</v>
       </c>
       <c r="N33" s="85"/>
-      <c r="O33" s="199"/>
-      <c r="P33" s="200"/>
-      <c r="Q33" s="174" t="s">
+      <c r="O33" s="178"/>
+      <c r="P33" s="179"/>
+      <c r="Q33" s="175" t="s">
         <v>70</v>
       </c>
-      <c r="R33" s="175"/>
-      <c r="S33" s="176"/>
+      <c r="R33" s="176"/>
+      <c r="S33" s="177"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="138" t="e">
@@ -3038,17 +3047,17 @@
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="203" t="s">
+      <c r="M34" s="206" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="204"/>
-      <c r="O34" s="205"/>
-      <c r="P34" s="206"/>
-      <c r="Q34" s="174" t="s">
+      <c r="N34" s="207"/>
+      <c r="O34" s="208"/>
+      <c r="P34" s="209"/>
+      <c r="Q34" s="175" t="s">
         <v>71</v>
       </c>
-      <c r="R34" s="175"/>
-      <c r="S34" s="176"/>
+      <c r="R34" s="176"/>
+      <c r="S34" s="177"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3066,23 +3075,23 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="196" t="s">
+      <c r="M35" s="212" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="197"/>
-      <c r="O35" s="198"/>
-      <c r="P35" s="189" t="s">
+      <c r="N35" s="213"/>
+      <c r="O35" s="214"/>
+      <c r="P35" s="204" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="193"/>
-      <c r="R35" s="189" t="s">
+      <c r="Q35" s="205"/>
+      <c r="R35" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="193"/>
-      <c r="T35" s="189" t="s">
+      <c r="S35" s="205"/>
+      <c r="T35" s="204" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="193"/>
+      <c r="U35" s="205"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3182,10 +3191,10 @@
       <c r="L38" s="114">
         <v>2</v>
       </c>
-      <c r="M38" s="179" t="s">
+      <c r="M38" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="N38" s="180"/>
+      <c r="N38" s="211"/>
       <c r="O38" s="46" t="s">
         <v>64</v>
       </c>
@@ -3210,9 +3219,15 @@
       <c r="L39" s="114">
         <v>3</v>
       </c>
-      <c r="M39" s="37"/>
-      <c r="N39" s="38"/>
-      <c r="O39" s="39"/>
+      <c r="M39" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="N39" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="O39" s="39" t="s">
+        <v>102</v>
+      </c>
       <c r="P39" s="42"/>
       <c r="Q39" s="72"/>
       <c r="R39" s="44"/>
@@ -3295,8 +3310,8 @@
       <c r="A43" s="112"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="183"/>
-      <c r="E43" s="183"/>
+      <c r="D43" s="203"/>
+      <c r="E43" s="203"/>
       <c r="F43" s="51"/>
       <c r="G43" s="8"/>
       <c r="I43" s="136"/>
@@ -3322,8 +3337,8 @@
       <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="183"/>
-      <c r="E44" s="183"/>
+      <c r="D44" s="203"/>
+      <c r="E44" s="203"/>
       <c r="F44" s="52"/>
       <c r="H44" s="68"/>
       <c r="I44" s="13"/>
@@ -3346,8 +3361,8 @@
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="43"/>
-      <c r="D45" s="183"/>
-      <c r="E45" s="183"/>
+      <c r="D45" s="203"/>
+      <c r="E45" s="203"/>
       <c r="F45" s="23"/>
       <c r="H45" s="68"/>
       <c r="I45" s="13"/>
@@ -3369,8 +3384,8 @@
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="43"/>
-      <c r="D46" s="183"/>
-      <c r="E46" s="183"/>
+      <c r="D46" s="203"/>
+      <c r="E46" s="203"/>
       <c r="F46" s="53"/>
       <c r="H46" s="68"/>
       <c r="I46" s="13"/>
@@ -3392,8 +3407,8 @@
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="43"/>
-      <c r="D47" s="183"/>
-      <c r="E47" s="183"/>
+      <c r="D47" s="203"/>
+      <c r="E47" s="203"/>
       <c r="F47" s="17"/>
       <c r="G47" s="1"/>
       <c r="H47" s="68"/>
@@ -3420,8 +3435,8 @@
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="43"/>
-      <c r="D48" s="183"/>
-      <c r="E48" s="183"/>
+      <c r="D48" s="203"/>
+      <c r="E48" s="203"/>
       <c r="F48" s="23"/>
       <c r="G48" s="1"/>
       <c r="H48" s="68"/>
@@ -3444,8 +3459,8 @@
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="43"/>
-      <c r="D49" s="183"/>
-      <c r="E49" s="183"/>
+      <c r="D49" s="203"/>
+      <c r="E49" s="203"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
       <c r="H49" s="50"/>
@@ -3492,8 +3507,8 @@
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="43"/>
-      <c r="D51" s="184"/>
-      <c r="E51" s="184"/>
+      <c r="D51" s="223"/>
+      <c r="E51" s="223"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="50"/>
@@ -3516,8 +3531,8 @@
       <c r="A52" s="20"/>
       <c r="B52" s="55"/>
       <c r="C52" s="43"/>
-      <c r="D52" s="182"/>
-      <c r="E52" s="182"/>
+      <c r="D52" s="229"/>
+      <c r="E52" s="229"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="50"/>
@@ -3540,8 +3555,8 @@
       <c r="A53" s="25"/>
       <c r="B53" s="55"/>
       <c r="C53" s="43"/>
-      <c r="D53" s="181"/>
-      <c r="E53" s="181"/>
+      <c r="D53" s="220"/>
+      <c r="E53" s="220"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="50"/>
@@ -3562,8 +3577,8 @@
       <c r="A54" s="20"/>
       <c r="B54" s="55"/>
       <c r="C54" s="43"/>
-      <c r="D54" s="181"/>
-      <c r="E54" s="181"/>
+      <c r="D54" s="220"/>
+      <c r="E54" s="220"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="50"/>
@@ -3694,8 +3709,8 @@
       <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="43"/>
-      <c r="D60" s="181"/>
-      <c r="E60" s="181"/>
+      <c r="D60" s="220"/>
+      <c r="E60" s="220"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="50"/>
@@ -3782,8 +3797,8 @@
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="43"/>
-      <c r="D64" s="181"/>
-      <c r="E64" s="181"/>
+      <c r="D64" s="220"/>
+      <c r="E64" s="220"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="50"/>
@@ -3804,18 +3819,18 @@
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="43"/>
-      <c r="D65" s="181"/>
-      <c r="E65" s="181"/>
+      <c r="D65" s="220"/>
+      <c r="E65" s="220"/>
       <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="50"/>
       <c r="I65" s="54"/>
       <c r="J65" s="57"/>
       <c r="L65"/>
-      <c r="M65" s="179" t="s">
+      <c r="M65" s="210" t="s">
         <v>34</v>
       </c>
-      <c r="N65" s="180"/>
+      <c r="N65" s="211"/>
       <c r="O65" s="46" t="s">
         <v>65</v>
       </c>
@@ -3842,8 +3857,8 @@
       <c r="A66" s="25"/>
       <c r="B66"/>
       <c r="C66" s="95"/>
-      <c r="D66" s="181"/>
-      <c r="E66" s="181"/>
+      <c r="D66" s="220"/>
+      <c r="E66" s="220"/>
       <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="50"/>
@@ -3871,29 +3886,29 @@
       <c r="I67" s="54"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="189" t="s">
+      <c r="M67" s="204" t="s">
         <v>47</v>
       </c>
-      <c r="N67" s="190"/>
-      <c r="O67" s="193"/>
-      <c r="P67" s="191"/>
-      <c r="Q67" s="192"/>
-      <c r="R67" s="189" t="s">
+      <c r="N67" s="219"/>
+      <c r="O67" s="205"/>
+      <c r="P67" s="221"/>
+      <c r="Q67" s="222"/>
+      <c r="R67" s="204" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="190"/>
-      <c r="T67" s="185" t="str">
+      <c r="S67" s="219"/>
+      <c r="T67" s="215" t="str">
         <f>Q25</f>
         <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
-      <c r="U67" s="186"/>
+      <c r="U67" s="216"/>
     </row>
     <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="181"/>
-      <c r="E68" s="181"/>
+      <c r="D68" s="220"/>
+      <c r="E68" s="220"/>
       <c r="F68" s="67"/>
       <c r="G68" s="1"/>
       <c r="H68" s="50"/>
@@ -3914,33 +3929,33 @@
       <c r="A69" s="25"/>
       <c r="B69" s="95"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="181"/>
-      <c r="E69" s="181"/>
+      <c r="D69" s="220"/>
+      <c r="E69" s="220"/>
       <c r="F69" s="67"/>
       <c r="G69" s="1"/>
       <c r="H69" s="50"/>
       <c r="I69" s="54"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="179" t="s">
+      <c r="M69" s="210" t="s">
         <v>35</v>
       </c>
-      <c r="N69" s="187"/>
-      <c r="O69" s="187"/>
-      <c r="P69" s="187"/>
-      <c r="Q69" s="187"/>
-      <c r="R69" s="187"/>
-      <c r="S69" s="187"/>
-      <c r="T69" s="187"/>
-      <c r="U69" s="188"/>
+      <c r="N69" s="217"/>
+      <c r="O69" s="217"/>
+      <c r="P69" s="217"/>
+      <c r="Q69" s="217"/>
+      <c r="R69" s="217"/>
+      <c r="S69" s="217"/>
+      <c r="T69" s="217"/>
+      <c r="U69" s="218"/>
       <c r="V69" s="55"/>
     </row>
     <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
       <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="181"/>
-      <c r="E70" s="181"/>
+      <c r="D70" s="220"/>
+      <c r="E70" s="220"/>
       <c r="F70" s="67"/>
       <c r="G70" s="1"/>
       <c r="H70" s="50"/>
@@ -3977,8 +3992,8 @@
       <c r="A71" s="25"/>
       <c r="B71" s="130"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="181"/>
-      <c r="E71" s="181"/>
+      <c r="D71" s="220"/>
+      <c r="E71" s="220"/>
       <c r="F71" s="67"/>
       <c r="G71" s="1"/>
       <c r="H71" s="50"/>
@@ -3996,10 +4011,10 @@
         <v>90</v>
       </c>
       <c r="Q71" s="65"/>
-      <c r="R71" s="178" t="s">
+      <c r="R71" s="228" t="s">
         <v>6</v>
       </c>
-      <c r="S71" s="178"/>
+      <c r="S71" s="228"/>
       <c r="T71" s="159" t="s">
         <v>91</v>
       </c>
@@ -4011,8 +4026,8 @@
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B72" s="55"/>
       <c r="C72" s="94"/>
-      <c r="D72" s="181"/>
-      <c r="E72" s="181"/>
+      <c r="D72" s="220"/>
+      <c r="E72" s="220"/>
       <c r="F72" s="67"/>
       <c r="I72" s="130"/>
       <c r="L72"/>
@@ -4021,8 +4036,8 @@
       <c r="O72" s="18"/>
       <c r="P72" s="91"/>
       <c r="Q72" s="60"/>
-      <c r="R72" s="173"/>
-      <c r="S72" s="173"/>
+      <c r="R72" s="226"/>
+      <c r="S72" s="226"/>
       <c r="T72" s="69"/>
       <c r="U72" s="100"/>
       <c r="V72" s="55"/>
@@ -4049,10 +4064,10 @@
         <v>95</v>
       </c>
       <c r="Q73" s="60"/>
-      <c r="R73" s="173" t="s">
+      <c r="R73" s="226" t="s">
         <v>10</v>
       </c>
-      <c r="S73" s="173"/>
+      <c r="S73" s="226"/>
       <c r="T73" s="69" t="s">
         <v>96</v>
       </c>
@@ -4068,8 +4083,8 @@
       <c r="O74" s="147"/>
       <c r="P74" s="91"/>
       <c r="Q74" s="60"/>
-      <c r="R74" s="173"/>
-      <c r="S74" s="173"/>
+      <c r="R74" s="226"/>
+      <c r="S74" s="226"/>
       <c r="T74" s="69"/>
       <c r="U74" s="100"/>
       <c r="V74" s="55"/>
@@ -4083,10 +4098,10 @@
       <c r="O75" s="165"/>
       <c r="P75" s="166"/>
       <c r="Q75" s="167"/>
-      <c r="R75" s="177"/>
-      <c r="S75" s="177"/>
-      <c r="T75" s="171"/>
-      <c r="U75" s="172"/>
+      <c r="R75" s="227"/>
+      <c r="S75" s="227"/>
+      <c r="T75" s="224"/>
+      <c r="U75" s="225"/>
       <c r="V75" s="55"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4100,8 +4115,8 @@
       <c r="Q76" s="167"/>
       <c r="R76" s="168"/>
       <c r="S76" s="168"/>
-      <c r="T76" s="171"/>
-      <c r="U76" s="172"/>
+      <c r="T76" s="224"/>
+      <c r="U76" s="225"/>
       <c r="V76" s="55"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4279,6 +4294,62 @@
     </row>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="M69:U69"/>
+    <mergeCell ref="R67:S67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="P67:Q67"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="Q25:S25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
     <mergeCell ref="M22:U22"/>
     <mergeCell ref="Q26:S26"/>
     <mergeCell ref="O29:P29"/>
@@ -4295,62 +4366,6 @@
     <mergeCell ref="N23:S23"/>
     <mergeCell ref="N24:S24"/>
     <mergeCell ref="T25:U25"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="Q25:S25"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="O32:P32"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="T67:U67"/>
-    <mergeCell ref="M69:U69"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T75:U75"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D52:E52"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
problemas docn mobile siell
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121944EB-68AE-4CE1-8C80-B49289578493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49775DE-810D-4758-A059-F713516FBF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RUTA" sheetId="1" r:id="rId1"/>
@@ -1021,7 +1021,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="227">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1409,166 +1409,6 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1584,41 +1424,20 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="171" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1630,6 +1449,166 @@
     </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2079,7 +2058,7 @@
       <c r="S3" s="120"/>
       <c r="T3" s="120"/>
       <c r="U3" s="110"/>
-      <c r="V3" s="224"/>
+      <c r="V3" s="163"/>
       <c r="W3" s="116"/>
     </row>
     <row r="4" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2108,7 +2087,7 @@
       <c r="S4" s="120"/>
       <c r="T4" s="120"/>
       <c r="U4" s="110"/>
-      <c r="V4" s="224"/>
+      <c r="V4" s="163"/>
       <c r="W4" s="116"/>
     </row>
     <row r="5" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2169,440 +2148,440 @@
       <c r="V6" s="111"/>
       <c r="W6" s="111"/>
     </row>
-    <row r="7" spans="1:23" s="213" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" s="45" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="122" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="225" t="s">
+      <c r="B7" s="164" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="225"/>
-      <c r="D7" s="225"/>
-      <c r="E7" s="225"/>
-      <c r="F7" s="225"/>
-      <c r="G7" s="225"/>
-      <c r="H7" s="225"/>
-      <c r="I7" s="225"/>
-      <c r="J7" s="225"/>
-      <c r="K7" s="225"/>
-      <c r="L7" s="225"/>
-      <c r="M7" s="225"/>
-      <c r="N7" s="225"/>
-      <c r="O7" s="225"/>
-      <c r="P7" s="225"/>
-      <c r="Q7" s="225"/>
-      <c r="R7" s="211"/>
-      <c r="S7" s="211"/>
-      <c r="T7" s="211"/>
-      <c r="U7" s="212"/>
-      <c r="V7" s="212"/>
-      <c r="W7" s="212"/>
-    </row>
-    <row r="8" spans="1:23" s="221" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="210"/>
-      <c r="B8" s="212"/>
-      <c r="C8" s="214"/>
-      <c r="D8" s="212"/>
-      <c r="E8" s="214"/>
-      <c r="F8" s="215"/>
-      <c r="G8" s="214"/>
-      <c r="H8" s="212"/>
-      <c r="I8" s="214"/>
-      <c r="J8" s="212"/>
-      <c r="K8" s="214"/>
-      <c r="L8" s="215"/>
-      <c r="M8" s="214"/>
-      <c r="N8" s="215"/>
-      <c r="O8" s="214"/>
-      <c r="P8" s="216"/>
-      <c r="Q8" s="214"/>
-      <c r="R8" s="216"/>
-      <c r="S8" s="214"/>
-      <c r="T8" s="216"/>
-      <c r="U8" s="214"/>
-      <c r="V8" s="215"/>
-      <c r="W8" s="214"/>
-    </row>
-    <row r="9" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="217" t="s">
+      <c r="C7" s="164"/>
+      <c r="D7" s="164"/>
+      <c r="E7" s="164"/>
+      <c r="F7" s="164"/>
+      <c r="G7" s="164"/>
+      <c r="H7" s="164"/>
+      <c r="I7" s="164"/>
+      <c r="J7" s="164"/>
+      <c r="K7" s="164"/>
+      <c r="L7" s="164"/>
+      <c r="M7" s="164"/>
+      <c r="N7" s="164"/>
+      <c r="O7" s="164"/>
+      <c r="P7" s="164"/>
+      <c r="Q7" s="164"/>
+      <c r="R7" s="156"/>
+      <c r="S7" s="156"/>
+      <c r="T7" s="156"/>
+      <c r="U7" s="157"/>
+      <c r="V7" s="157"/>
+      <c r="W7" s="157"/>
+    </row>
+    <row r="8" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="112"/>
+      <c r="B8" s="157"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="157"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="157"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="157"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="110"/>
+      <c r="M8" s="111"/>
+      <c r="N8" s="110"/>
+      <c r="O8" s="111"/>
+      <c r="P8" s="158"/>
+      <c r="Q8" s="111"/>
+      <c r="R8" s="158"/>
+      <c r="S8" s="111"/>
+      <c r="T8" s="158"/>
+      <c r="U8" s="111"/>
+      <c r="V8" s="110"/>
+      <c r="W8" s="111"/>
+    </row>
+    <row r="9" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="113" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="226" t="s">
+      <c r="B9" s="165" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="226"/>
-      <c r="D9" s="226"/>
-      <c r="E9" s="212"/>
-      <c r="F9" s="215"/>
-      <c r="G9" s="212"/>
-      <c r="H9" s="215"/>
-      <c r="I9" s="212"/>
-      <c r="J9" s="215"/>
-      <c r="K9" s="212"/>
-      <c r="L9" s="215"/>
-      <c r="M9" s="212"/>
-      <c r="N9" s="215"/>
-      <c r="O9" s="212"/>
-      <c r="P9" s="216"/>
-      <c r="Q9" s="212"/>
-      <c r="R9" s="216"/>
-      <c r="S9" s="218"/>
-      <c r="T9" s="218"/>
-      <c r="U9" s="212"/>
-      <c r="V9" s="215"/>
-      <c r="W9" s="212"/>
-    </row>
-    <row r="10" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="217" t="s">
+      <c r="C9" s="165"/>
+      <c r="D9" s="165"/>
+      <c r="E9" s="157"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="157"/>
+      <c r="H9" s="110"/>
+      <c r="I9" s="157"/>
+      <c r="J9" s="110"/>
+      <c r="K9" s="157"/>
+      <c r="L9" s="110"/>
+      <c r="M9" s="157"/>
+      <c r="N9" s="110"/>
+      <c r="O9" s="157"/>
+      <c r="P9" s="158"/>
+      <c r="Q9" s="157"/>
+      <c r="R9" s="158"/>
+      <c r="S9" s="159"/>
+      <c r="T9" s="159"/>
+      <c r="U9" s="157"/>
+      <c r="V9" s="110"/>
+      <c r="W9" s="157"/>
+    </row>
+    <row r="10" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="113" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="226" t="s">
+      <c r="B10" s="165" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="226"/>
-      <c r="D10" s="226"/>
-      <c r="E10" s="212"/>
-      <c r="F10" s="215"/>
-      <c r="G10" s="212"/>
-      <c r="H10" s="215"/>
-      <c r="I10" s="212"/>
-      <c r="J10" s="215"/>
-      <c r="K10" s="212"/>
-      <c r="L10" s="215"/>
-      <c r="M10" s="212"/>
-      <c r="N10" s="215"/>
-      <c r="O10" s="212"/>
-      <c r="P10" s="216"/>
-      <c r="Q10" s="212"/>
-      <c r="R10" s="216"/>
-      <c r="S10" s="218"/>
-      <c r="T10" s="218"/>
-      <c r="U10" s="212"/>
-      <c r="V10" s="215"/>
-      <c r="W10" s="212"/>
-    </row>
-    <row r="11" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="217" t="s">
+      <c r="C10" s="165"/>
+      <c r="D10" s="165"/>
+      <c r="E10" s="157"/>
+      <c r="F10" s="110"/>
+      <c r="G10" s="157"/>
+      <c r="H10" s="110"/>
+      <c r="I10" s="157"/>
+      <c r="J10" s="110"/>
+      <c r="K10" s="157"/>
+      <c r="L10" s="110"/>
+      <c r="M10" s="157"/>
+      <c r="N10" s="110"/>
+      <c r="O10" s="157"/>
+      <c r="P10" s="158"/>
+      <c r="Q10" s="157"/>
+      <c r="R10" s="158"/>
+      <c r="S10" s="159"/>
+      <c r="T10" s="159"/>
+      <c r="U10" s="157"/>
+      <c r="V10" s="110"/>
+      <c r="W10" s="157"/>
+    </row>
+    <row r="11" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="226" t="s">
+      <c r="B11" s="165" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="226"/>
-      <c r="D11" s="226"/>
-      <c r="E11" s="212"/>
-      <c r="F11" s="215"/>
-      <c r="G11" s="212"/>
-      <c r="H11" s="215"/>
-      <c r="I11" s="212"/>
-      <c r="J11" s="215"/>
-      <c r="K11" s="212"/>
-      <c r="L11" s="215"/>
-      <c r="M11" s="212"/>
-      <c r="N11" s="215"/>
-      <c r="O11" s="212"/>
-      <c r="P11" s="216"/>
-      <c r="Q11" s="212"/>
-      <c r="R11" s="216"/>
-      <c r="S11" s="218"/>
-      <c r="T11" s="218"/>
-      <c r="U11" s="212"/>
-      <c r="V11" s="215"/>
-      <c r="W11" s="212"/>
-    </row>
-    <row r="12" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="217" t="s">
+      <c r="C11" s="165"/>
+      <c r="D11" s="165"/>
+      <c r="E11" s="157"/>
+      <c r="F11" s="110"/>
+      <c r="G11" s="157"/>
+      <c r="H11" s="110"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="110"/>
+      <c r="K11" s="157"/>
+      <c r="L11" s="110"/>
+      <c r="M11" s="157"/>
+      <c r="N11" s="110"/>
+      <c r="O11" s="157"/>
+      <c r="P11" s="158"/>
+      <c r="Q11" s="157"/>
+      <c r="R11" s="158"/>
+      <c r="S11" s="159"/>
+      <c r="T11" s="159"/>
+      <c r="U11" s="157"/>
+      <c r="V11" s="110"/>
+      <c r="W11" s="157"/>
+    </row>
+    <row r="12" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="113" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="226" t="s">
+      <c r="B12" s="165" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="226"/>
-      <c r="D12" s="226"/>
-      <c r="E12" s="212"/>
-      <c r="F12" s="215"/>
-      <c r="G12" s="212"/>
-      <c r="H12" s="215"/>
-      <c r="I12" s="212"/>
-      <c r="J12" s="215"/>
-      <c r="K12" s="212"/>
-      <c r="L12" s="215"/>
-      <c r="M12" s="212"/>
-      <c r="N12" s="215"/>
-      <c r="O12" s="212"/>
-      <c r="P12" s="216"/>
-      <c r="Q12" s="212"/>
-      <c r="R12" s="216"/>
-      <c r="S12" s="218"/>
-      <c r="T12" s="218"/>
-      <c r="U12" s="212"/>
-      <c r="V12" s="215"/>
-      <c r="W12" s="212"/>
-    </row>
-    <row r="13" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="217" t="s">
+      <c r="C12" s="165"/>
+      <c r="D12" s="165"/>
+      <c r="E12" s="157"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="157"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="157"/>
+      <c r="J12" s="110"/>
+      <c r="K12" s="157"/>
+      <c r="L12" s="110"/>
+      <c r="M12" s="157"/>
+      <c r="N12" s="110"/>
+      <c r="O12" s="157"/>
+      <c r="P12" s="158"/>
+      <c r="Q12" s="157"/>
+      <c r="R12" s="158"/>
+      <c r="S12" s="159"/>
+      <c r="T12" s="159"/>
+      <c r="U12" s="157"/>
+      <c r="V12" s="110"/>
+      <c r="W12" s="157"/>
+    </row>
+    <row r="13" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="226" t="s">
+      <c r="B13" s="165" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="226"/>
-      <c r="D13" s="226"/>
-      <c r="E13" s="212"/>
-      <c r="F13" s="215"/>
-      <c r="G13" s="212"/>
-      <c r="H13" s="215"/>
-      <c r="I13" s="212"/>
-      <c r="J13" s="215"/>
-      <c r="K13" s="212"/>
-      <c r="L13" s="215"/>
-      <c r="M13" s="212"/>
-      <c r="N13" s="215"/>
-      <c r="O13" s="212"/>
-      <c r="P13" s="216"/>
-      <c r="Q13" s="212"/>
-      <c r="R13" s="216"/>
-      <c r="S13" s="218"/>
-      <c r="T13" s="218"/>
-      <c r="U13" s="212"/>
-      <c r="V13" s="215"/>
-      <c r="W13" s="212"/>
-    </row>
-    <row r="14" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="217" t="s">
+      <c r="C13" s="165"/>
+      <c r="D13" s="165"/>
+      <c r="E13" s="157"/>
+      <c r="F13" s="110"/>
+      <c r="G13" s="157"/>
+      <c r="H13" s="110"/>
+      <c r="I13" s="157"/>
+      <c r="J13" s="110"/>
+      <c r="K13" s="157"/>
+      <c r="L13" s="110"/>
+      <c r="M13" s="157"/>
+      <c r="N13" s="110"/>
+      <c r="O13" s="157"/>
+      <c r="P13" s="158"/>
+      <c r="Q13" s="157"/>
+      <c r="R13" s="158"/>
+      <c r="S13" s="159"/>
+      <c r="T13" s="159"/>
+      <c r="U13" s="157"/>
+      <c r="V13" s="110"/>
+      <c r="W13" s="157"/>
+    </row>
+    <row r="14" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="226" t="s">
+      <c r="B14" s="165" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="226"/>
-      <c r="D14" s="226"/>
-      <c r="E14" s="212"/>
-      <c r="F14" s="215"/>
-      <c r="G14" s="212"/>
-      <c r="H14" s="215"/>
-      <c r="I14" s="212"/>
-      <c r="J14" s="215"/>
-      <c r="K14" s="212"/>
-      <c r="L14" s="215"/>
-      <c r="M14" s="212"/>
-      <c r="N14" s="215"/>
-      <c r="O14" s="212"/>
-      <c r="P14" s="216"/>
-      <c r="Q14" s="212"/>
-      <c r="R14" s="216"/>
-      <c r="S14" s="218"/>
-      <c r="T14" s="218"/>
-      <c r="U14" s="212"/>
-      <c r="V14" s="215"/>
-      <c r="W14" s="212"/>
-    </row>
-    <row r="15" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="217" t="s">
+      <c r="C14" s="165"/>
+      <c r="D14" s="165"/>
+      <c r="E14" s="157"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="157"/>
+      <c r="H14" s="110"/>
+      <c r="I14" s="157"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="157"/>
+      <c r="L14" s="110"/>
+      <c r="M14" s="157"/>
+      <c r="N14" s="110"/>
+      <c r="O14" s="157"/>
+      <c r="P14" s="158"/>
+      <c r="Q14" s="157"/>
+      <c r="R14" s="158"/>
+      <c r="S14" s="159"/>
+      <c r="T14" s="159"/>
+      <c r="U14" s="157"/>
+      <c r="V14" s="110"/>
+      <c r="W14" s="157"/>
+    </row>
+    <row r="15" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="113" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="226" t="s">
+      <c r="B15" s="165" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="226"/>
-      <c r="D15" s="226"/>
-      <c r="E15" s="212"/>
-      <c r="F15" s="215"/>
-      <c r="G15" s="212"/>
-      <c r="H15" s="215"/>
-      <c r="I15" s="212"/>
-      <c r="J15" s="215"/>
-      <c r="K15" s="212"/>
-      <c r="L15" s="215"/>
-      <c r="M15" s="212"/>
-      <c r="N15" s="215"/>
-      <c r="O15" s="212"/>
-      <c r="P15" s="216"/>
-      <c r="Q15" s="212"/>
-      <c r="R15" s="216"/>
-      <c r="S15" s="218"/>
-      <c r="T15" s="218"/>
-      <c r="U15" s="212"/>
-      <c r="V15" s="215"/>
-      <c r="W15" s="212"/>
-    </row>
-    <row r="16" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="217" t="s">
+      <c r="C15" s="165"/>
+      <c r="D15" s="165"/>
+      <c r="E15" s="157"/>
+      <c r="F15" s="110"/>
+      <c r="G15" s="157"/>
+      <c r="H15" s="110"/>
+      <c r="I15" s="157"/>
+      <c r="J15" s="110"/>
+      <c r="K15" s="157"/>
+      <c r="L15" s="110"/>
+      <c r="M15" s="157"/>
+      <c r="N15" s="110"/>
+      <c r="O15" s="157"/>
+      <c r="P15" s="158"/>
+      <c r="Q15" s="157"/>
+      <c r="R15" s="158"/>
+      <c r="S15" s="159"/>
+      <c r="T15" s="159"/>
+      <c r="U15" s="157"/>
+      <c r="V15" s="110"/>
+      <c r="W15" s="157"/>
+    </row>
+    <row r="16" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="113" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="226" t="s">
+      <c r="B16" s="165" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="226"/>
-      <c r="D16" s="226"/>
-      <c r="E16" s="212"/>
-      <c r="F16" s="215"/>
-      <c r="G16" s="212"/>
-      <c r="H16" s="215"/>
-      <c r="I16" s="219"/>
-      <c r="J16" s="215"/>
-      <c r="K16" s="219"/>
-      <c r="L16" s="215"/>
-      <c r="M16" s="212"/>
-      <c r="N16" s="215"/>
-      <c r="O16" s="212"/>
-      <c r="P16" s="216"/>
-      <c r="Q16" s="212"/>
-      <c r="R16" s="216"/>
-      <c r="S16" s="218"/>
-      <c r="T16" s="218"/>
-      <c r="U16" s="212"/>
-      <c r="V16" s="215"/>
-      <c r="W16" s="212"/>
-    </row>
-    <row r="17" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="217" t="s">
+      <c r="C16" s="165"/>
+      <c r="D16" s="165"/>
+      <c r="E16" s="157"/>
+      <c r="F16" s="110"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="110"/>
+      <c r="I16" s="160"/>
+      <c r="J16" s="110"/>
+      <c r="K16" s="160"/>
+      <c r="L16" s="110"/>
+      <c r="M16" s="157"/>
+      <c r="N16" s="110"/>
+      <c r="O16" s="157"/>
+      <c r="P16" s="158"/>
+      <c r="Q16" s="157"/>
+      <c r="R16" s="158"/>
+      <c r="S16" s="159"/>
+      <c r="T16" s="159"/>
+      <c r="U16" s="157"/>
+      <c r="V16" s="110"/>
+      <c r="W16" s="157"/>
+    </row>
+    <row r="17" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="113" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="226" t="s">
+      <c r="B17" s="165" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="226"/>
-      <c r="D17" s="226"/>
-      <c r="E17" s="212"/>
-      <c r="F17" s="215"/>
-      <c r="G17" s="212"/>
-      <c r="H17" s="215"/>
-      <c r="I17" s="219"/>
-      <c r="J17" s="215"/>
-      <c r="K17" s="212"/>
-      <c r="L17" s="215"/>
-      <c r="M17" s="212"/>
-      <c r="N17" s="215"/>
-      <c r="O17" s="212"/>
-      <c r="P17" s="216"/>
-      <c r="Q17" s="212"/>
-      <c r="R17" s="216"/>
-      <c r="S17" s="218"/>
-      <c r="T17" s="218"/>
-      <c r="U17" s="212"/>
-      <c r="V17" s="215"/>
-      <c r="W17" s="212"/>
-    </row>
-    <row r="18" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="217" t="s">
+      <c r="C17" s="165"/>
+      <c r="D17" s="165"/>
+      <c r="E17" s="157"/>
+      <c r="F17" s="110"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="110"/>
+      <c r="I17" s="160"/>
+      <c r="J17" s="110"/>
+      <c r="K17" s="157"/>
+      <c r="L17" s="110"/>
+      <c r="M17" s="157"/>
+      <c r="N17" s="110"/>
+      <c r="O17" s="157"/>
+      <c r="P17" s="158"/>
+      <c r="Q17" s="157"/>
+      <c r="R17" s="158"/>
+      <c r="S17" s="159"/>
+      <c r="T17" s="159"/>
+      <c r="U17" s="157"/>
+      <c r="V17" s="110"/>
+      <c r="W17" s="157"/>
+    </row>
+    <row r="18" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="113" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="215">
+      <c r="B18" s="110">
         <f>SUM(B9:B17)</f>
         <v>0</v>
       </c>
-      <c r="C18" s="215">
+      <c r="C18" s="110">
         <f t="shared" ref="C18:O18" si="0">SUM(C9:C17)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="215">
+      <c r="D18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E18" s="215">
+      <c r="E18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="215">
+      <c r="F18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G18" s="215">
+      <c r="G18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="215">
+      <c r="H18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I18" s="215">
+      <c r="I18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="215">
+      <c r="J18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K18" s="215">
+      <c r="K18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L18" s="215">
+      <c r="L18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M18" s="215">
+      <c r="M18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N18" s="215">
+      <c r="N18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O18" s="215">
+      <c r="O18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P18" s="215">
+      <c r="P18" s="110">
         <f t="shared" ref="P18" si="1">SUM(P9:P17)</f>
         <v>0</v>
       </c>
-      <c r="Q18" s="215">
+      <c r="Q18" s="110">
         <f>SUM(Q9:Q17)</f>
         <v>0</v>
       </c>
-      <c r="R18" s="215">
+      <c r="R18" s="110">
         <f>SUM(R9:R17)</f>
         <v>0</v>
       </c>
-      <c r="S18" s="220">
+      <c r="S18" s="116">
         <f>SUM(S9:S17)</f>
         <v>0</v>
       </c>
-      <c r="T18" s="220">
+      <c r="T18" s="116">
         <f>SUM(T9:T17)</f>
         <v>0</v>
       </c>
-      <c r="U18" s="215">
+      <c r="U18" s="110">
         <f t="shared" ref="U18:W18" si="2">SUM(U9:U17)</f>
         <v>0</v>
       </c>
-      <c r="V18" s="215">
+      <c r="V18" s="110">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="W18" s="215">
+      <c r="W18" s="110">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="217"/>
-      <c r="B19" s="215"/>
-      <c r="C19" s="215"/>
-      <c r="D19" s="215"/>
-      <c r="E19" s="215"/>
-      <c r="F19" s="212"/>
-      <c r="G19" s="215"/>
-      <c r="H19" s="215"/>
-      <c r="I19" s="215"/>
-      <c r="J19" s="215"/>
-      <c r="K19" s="215"/>
-      <c r="L19" s="215"/>
-      <c r="M19" s="215"/>
-      <c r="N19" s="215"/>
-      <c r="O19" s="215"/>
-      <c r="P19" s="215"/>
-      <c r="Q19" s="215"/>
-      <c r="R19" s="215"/>
-      <c r="S19" s="220"/>
-      <c r="T19" s="220"/>
-      <c r="U19" s="215"/>
-      <c r="V19" s="215"/>
-      <c r="W19" s="215"/>
-    </row>
-    <row r="20" spans="1:23" s="223" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="113"/>
+      <c r="B19" s="110"/>
+      <c r="C19" s="110"/>
+      <c r="D19" s="110"/>
+      <c r="E19" s="110"/>
+      <c r="F19" s="157"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="110"/>
+      <c r="K19" s="110"/>
+      <c r="L19" s="110"/>
+      <c r="M19" s="110"/>
+      <c r="N19" s="110"/>
+      <c r="O19" s="110"/>
+      <c r="P19" s="110"/>
+      <c r="Q19" s="110"/>
+      <c r="R19" s="110"/>
+      <c r="S19" s="116"/>
+      <c r="T19" s="116"/>
+      <c r="U19" s="110"/>
+      <c r="V19" s="110"/>
+      <c r="W19" s="110"/>
+    </row>
+    <row r="20" spans="1:23" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="113" t="s">
         <v>12</v>
       </c>
@@ -2722,17 +2701,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="168" t="s">
+      <c r="M22" s="198" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="168"/>
-      <c r="O22" s="168"/>
-      <c r="P22" s="168"/>
-      <c r="Q22" s="168"/>
-      <c r="R22" s="168"/>
-      <c r="S22" s="168"/>
-      <c r="T22" s="168"/>
-      <c r="U22" s="168"/>
+      <c r="N22" s="198"/>
+      <c r="O22" s="198"/>
+      <c r="P22" s="198"/>
+      <c r="Q22" s="198"/>
+      <c r="R22" s="198"/>
+      <c r="S22" s="198"/>
+      <c r="T22" s="198"/>
+      <c r="U22" s="198"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2741,14 +2720,14 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="151" t="s">
+      <c r="N23" s="207" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="152"/>
-      <c r="P23" s="152"/>
-      <c r="Q23" s="152"/>
-      <c r="R23" s="152"/>
-      <c r="S23" s="153"/>
+      <c r="O23" s="208"/>
+      <c r="P23" s="208"/>
+      <c r="Q23" s="208"/>
+      <c r="R23" s="208"/>
+      <c r="S23" s="209"/>
       <c r="T23" s="119" t="s">
         <v>38</v>
       </c>
@@ -2766,14 +2745,14 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="154" t="s">
+      <c r="N24" s="210" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="155"/>
-      <c r="P24" s="155"/>
-      <c r="Q24" s="155"/>
-      <c r="R24" s="155"/>
-      <c r="S24" s="156"/>
+      <c r="O24" s="211"/>
+      <c r="P24" s="211"/>
+      <c r="Q24" s="211"/>
+      <c r="R24" s="211"/>
+      <c r="S24" s="212"/>
       <c r="T24" s="108" t="s">
         <v>11</v>
       </c>
@@ -2793,10 +2772,10 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="161" t="s">
+      <c r="M25" s="215" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="162"/>
+      <c r="N25" s="216"/>
       <c r="O25" s="148"/>
       <c r="P25" s="149"/>
       <c r="Q25" s="145" t="s">
@@ -2804,10 +2783,10 @@
       </c>
       <c r="R25" s="146"/>
       <c r="S25" s="147"/>
-      <c r="T25" s="157" t="s">
+      <c r="T25" s="213" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="158"/>
+      <c r="U25" s="214"/>
       <c r="V25" s="13"/>
       <c r="W25" s="82" t="s">
         <v>45</v>
@@ -2823,11 +2802,11 @@
       <c r="N26" s="80"/>
       <c r="O26" s="126"/>
       <c r="P26" s="127"/>
-      <c r="Q26" s="165" t="s">
+      <c r="Q26" s="188" t="s">
         <v>95</v>
       </c>
-      <c r="R26" s="166"/>
-      <c r="S26" s="167"/>
+      <c r="R26" s="189"/>
+      <c r="S26" s="190"/>
       <c r="T26" s="124"/>
       <c r="U26" s="125"/>
       <c r="V26" s="13"/>
@@ -2847,17 +2826,17 @@
         <v>18</v>
       </c>
       <c r="N27" s="80"/>
-      <c r="O27" s="163"/>
-      <c r="P27" s="169"/>
-      <c r="Q27" s="165" t="s">
+      <c r="O27" s="186"/>
+      <c r="P27" s="187"/>
+      <c r="Q27" s="188" t="s">
         <v>64</v>
       </c>
-      <c r="R27" s="166"/>
-      <c r="S27" s="167"/>
-      <c r="T27" s="176" t="s">
+      <c r="R27" s="189"/>
+      <c r="S27" s="190"/>
+      <c r="T27" s="205" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="177"/>
+      <c r="U27" s="206"/>
       <c r="V27" s="19"/>
       <c r="W27" s="92" t="s">
         <v>76</v>
@@ -2873,21 +2852,21 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="174" t="s">
+      <c r="M28" s="203" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="175"/>
-      <c r="O28" s="163"/>
-      <c r="P28" s="169"/>
-      <c r="Q28" s="165" t="s">
+      <c r="N28" s="204"/>
+      <c r="O28" s="186"/>
+      <c r="P28" s="187"/>
+      <c r="Q28" s="188" t="s">
         <v>65</v>
       </c>
-      <c r="R28" s="166"/>
-      <c r="S28" s="167"/>
-      <c r="T28" s="172" t="s">
+      <c r="R28" s="189"/>
+      <c r="S28" s="190"/>
+      <c r="T28" s="201" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="173"/>
+      <c r="U28" s="202"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2902,21 +2881,21 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="174" t="s">
+      <c r="M29" s="203" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="175"/>
-      <c r="O29" s="163"/>
-      <c r="P29" s="169"/>
-      <c r="Q29" s="165" t="s">
+      <c r="N29" s="204"/>
+      <c r="O29" s="186"/>
+      <c r="P29" s="187"/>
+      <c r="Q29" s="188" t="s">
         <v>66</v>
       </c>
-      <c r="R29" s="166"/>
-      <c r="S29" s="167"/>
-      <c r="T29" s="170" t="s">
+      <c r="R29" s="189"/>
+      <c r="S29" s="190"/>
+      <c r="T29" s="199" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="171"/>
+      <c r="U29" s="200"/>
       <c r="W29" s="93" t="str">
         <f>U23</f>
         <v>{{extraction.cant_fact.valor}}</v>
@@ -2933,21 +2912,21 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="174" t="s">
+      <c r="M30" s="203" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="175"/>
-      <c r="O30" s="163"/>
-      <c r="P30" s="164"/>
-      <c r="Q30" s="165" t="s">
+      <c r="N30" s="204"/>
+      <c r="O30" s="186"/>
+      <c r="P30" s="217"/>
+      <c r="Q30" s="188" t="s">
         <v>67</v>
       </c>
-      <c r="R30" s="166"/>
-      <c r="S30" s="167"/>
-      <c r="T30" s="178" t="s">
+      <c r="R30" s="189"/>
+      <c r="S30" s="190"/>
+      <c r="T30" s="218" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="179"/>
+      <c r="U30" s="219"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2965,17 +2944,17 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="174" t="s">
+      <c r="M31" s="203" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="175"/>
-      <c r="O31" s="163"/>
-      <c r="P31" s="169"/>
-      <c r="Q31" s="165" t="s">
+      <c r="N31" s="204"/>
+      <c r="O31" s="186"/>
+      <c r="P31" s="187"/>
+      <c r="Q31" s="188" t="s">
         <v>68</v>
       </c>
-      <c r="R31" s="166"/>
-      <c r="S31" s="167"/>
+      <c r="R31" s="189"/>
+      <c r="S31" s="190"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2990,17 +2969,17 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="174" t="s">
+      <c r="M32" s="203" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="175"/>
-      <c r="O32" s="163"/>
-      <c r="P32" s="169"/>
-      <c r="Q32" s="165" t="s">
+      <c r="N32" s="204"/>
+      <c r="O32" s="186"/>
+      <c r="P32" s="187"/>
+      <c r="Q32" s="188" t="s">
         <v>69</v>
       </c>
-      <c r="R32" s="166"/>
-      <c r="S32" s="167"/>
+      <c r="R32" s="189"/>
+      <c r="S32" s="190"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="82" t="s">
@@ -3022,13 +3001,13 @@
         <v>25</v>
       </c>
       <c r="N33" s="81"/>
-      <c r="O33" s="163"/>
-      <c r="P33" s="169"/>
-      <c r="Q33" s="165" t="s">
+      <c r="O33" s="186"/>
+      <c r="P33" s="187"/>
+      <c r="Q33" s="188" t="s">
         <v>70</v>
       </c>
-      <c r="R33" s="166"/>
-      <c r="S33" s="167"/>
+      <c r="R33" s="189"/>
+      <c r="S33" s="190"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="117" t="e">
@@ -3047,17 +3026,17 @@
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="183" t="s">
+      <c r="M34" s="191" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="184"/>
-      <c r="O34" s="185"/>
-      <c r="P34" s="186"/>
-      <c r="Q34" s="165" t="s">
+      <c r="N34" s="192"/>
+      <c r="O34" s="193"/>
+      <c r="P34" s="194"/>
+      <c r="Q34" s="188" t="s">
         <v>71</v>
       </c>
-      <c r="R34" s="166"/>
-      <c r="S34" s="167"/>
+      <c r="R34" s="189"/>
+      <c r="S34" s="190"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3075,23 +3054,23 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="193" t="s">
+      <c r="M35" s="195" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="194"/>
-      <c r="O35" s="195"/>
-      <c r="P35" s="181" t="s">
+      <c r="N35" s="196"/>
+      <c r="O35" s="197"/>
+      <c r="P35" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="182"/>
-      <c r="R35" s="181" t="s">
+      <c r="Q35" s="169"/>
+      <c r="R35" s="167" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="182"/>
-      <c r="T35" s="181" t="s">
+      <c r="S35" s="169"/>
+      <c r="T35" s="167" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="182"/>
+      <c r="U35" s="169"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3157,19 +3136,19 @@
       <c r="O37" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="P37" s="205" t="s">
+      <c r="P37" s="151" t="s">
         <v>80</v>
       </c>
       <c r="Q37" s="77" t="s">
         <v>81</v>
       </c>
-      <c r="R37" s="207" t="s">
+      <c r="R37" s="153" t="s">
         <v>82</v>
       </c>
       <c r="S37" s="78" t="s">
         <v>83</v>
       </c>
-      <c r="T37" s="206" t="s">
+      <c r="T37" s="152" t="s">
         <v>84</v>
       </c>
       <c r="U37" s="74" t="s">
@@ -3192,18 +3171,18 @@
         <v>0</v>
       </c>
       <c r="L38" s="105"/>
-      <c r="M38" s="159" t="s">
+      <c r="M38" s="171" t="s">
         <v>42</v>
       </c>
-      <c r="N38" s="160"/>
+      <c r="N38" s="179"/>
       <c r="O38" s="150" t="s">
         <v>64</v>
       </c>
-      <c r="P38" s="206"/>
+      <c r="P38" s="152"/>
       <c r="Q38" s="75"/>
-      <c r="R38" s="208"/>
+      <c r="R38" s="154"/>
       <c r="S38" s="73"/>
-      <c r="T38" s="206"/>
+      <c r="T38" s="152"/>
       <c r="U38" s="76"/>
       <c r="V38" s="1"/>
       <c r="W38" s="1"/>
@@ -3230,11 +3209,11 @@
       <c r="O39" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="P39" s="206"/>
+      <c r="P39" s="152"/>
       <c r="Q39" s="68"/>
-      <c r="R39" s="208"/>
+      <c r="R39" s="154"/>
       <c r="S39" s="73"/>
-      <c r="T39" s="206"/>
+      <c r="T39" s="152"/>
       <c r="U39" s="68"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1"/>
@@ -3257,11 +3236,11 @@
       <c r="M40" s="37"/>
       <c r="N40" s="38"/>
       <c r="O40" s="39"/>
-      <c r="P40" s="206"/>
+      <c r="P40" s="152"/>
       <c r="Q40" s="66"/>
-      <c r="R40" s="208"/>
+      <c r="R40" s="154"/>
       <c r="S40" s="74"/>
-      <c r="T40" s="206"/>
+      <c r="T40" s="152"/>
       <c r="U40" s="68"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1"/>
@@ -3284,11 +3263,11 @@
       <c r="M41" s="37"/>
       <c r="N41" s="38"/>
       <c r="O41" s="39"/>
-      <c r="P41" s="206"/>
+      <c r="P41" s="152"/>
       <c r="Q41" s="66"/>
-      <c r="R41" s="208"/>
+      <c r="R41" s="154"/>
       <c r="S41" s="74"/>
-      <c r="T41" s="206"/>
+      <c r="T41" s="152"/>
       <c r="U41" s="68"/>
       <c r="V41" s="1"/>
       <c r="W41" s="1"/>
@@ -3311,11 +3290,11 @@
       <c r="M42" s="37"/>
       <c r="N42" s="38"/>
       <c r="O42" s="39"/>
-      <c r="P42" s="206"/>
+      <c r="P42" s="152"/>
       <c r="Q42" s="66"/>
-      <c r="R42" s="208"/>
+      <c r="R42" s="154"/>
       <c r="S42" s="73"/>
-      <c r="T42" s="206"/>
+      <c r="T42" s="152"/>
       <c r="U42" s="68"/>
       <c r="V42" s="1"/>
       <c r="W42" s="1"/>
@@ -3324,8 +3303,8 @@
       <c r="A43" s="104"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="180"/>
-      <c r="E43" s="180"/>
+      <c r="D43" s="170"/>
+      <c r="E43" s="170"/>
       <c r="F43" s="47"/>
       <c r="G43" s="8"/>
       <c r="I43" s="41">
@@ -3341,19 +3320,19 @@
       <c r="M43" s="37"/>
       <c r="N43" s="38"/>
       <c r="O43" s="39"/>
-      <c r="P43" s="206"/>
+      <c r="P43" s="152"/>
       <c r="Q43" s="66"/>
-      <c r="R43" s="206"/>
+      <c r="R43" s="152"/>
       <c r="S43" s="67"/>
-      <c r="T43" s="206"/>
+      <c r="T43" s="152"/>
       <c r="U43" s="68"/>
     </row>
     <row r="44" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="180"/>
-      <c r="E44" s="180"/>
+      <c r="D44" s="170"/>
+      <c r="E44" s="170"/>
       <c r="F44" s="48"/>
       <c r="H44" s="64"/>
       <c r="I44" s="41">
@@ -3369,19 +3348,19 @@
       <c r="M44" s="37"/>
       <c r="N44" s="38"/>
       <c r="O44" s="39"/>
-      <c r="P44" s="206"/>
+      <c r="P44" s="152"/>
       <c r="Q44" s="66"/>
-      <c r="R44" s="206"/>
+      <c r="R44" s="152"/>
       <c r="S44" s="67"/>
-      <c r="T44" s="206"/>
+      <c r="T44" s="152"/>
       <c r="U44" s="68"/>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="40"/>
-      <c r="D45" s="180"/>
-      <c r="E45" s="180"/>
+      <c r="D45" s="170"/>
+      <c r="E45" s="170"/>
       <c r="F45" s="23"/>
       <c r="H45" s="64"/>
       <c r="I45" s="41">
@@ -3396,19 +3375,19 @@
       <c r="M45" s="37"/>
       <c r="N45" s="38"/>
       <c r="O45" s="39"/>
-      <c r="P45" s="206"/>
+      <c r="P45" s="152"/>
       <c r="Q45" s="66"/>
-      <c r="R45" s="206"/>
+      <c r="R45" s="152"/>
       <c r="S45" s="72"/>
-      <c r="T45" s="206"/>
+      <c r="T45" s="152"/>
       <c r="U45" s="68"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="40"/>
-      <c r="D46" s="180"/>
-      <c r="E46" s="180"/>
+      <c r="D46" s="170"/>
+      <c r="E46" s="170"/>
       <c r="F46" s="49"/>
       <c r="H46" s="64"/>
       <c r="I46" s="13"/>
@@ -3420,19 +3399,19 @@
       <c r="M46" s="37"/>
       <c r="N46" s="38"/>
       <c r="O46" s="39"/>
-      <c r="P46" s="206"/>
+      <c r="P46" s="152"/>
       <c r="Q46" s="66"/>
-      <c r="R46" s="206"/>
+      <c r="R46" s="152"/>
       <c r="S46" s="67"/>
-      <c r="T46" s="206"/>
+      <c r="T46" s="152"/>
       <c r="U46" s="68"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="40"/>
-      <c r="D47" s="180"/>
-      <c r="E47" s="180"/>
+      <c r="D47" s="170"/>
+      <c r="E47" s="170"/>
       <c r="F47" s="17"/>
       <c r="G47" s="1"/>
       <c r="H47" s="64"/>
@@ -3443,19 +3422,19 @@
       <c r="M47" s="37"/>
       <c r="N47" s="38"/>
       <c r="O47" s="39"/>
-      <c r="P47" s="206"/>
+      <c r="P47" s="152"/>
       <c r="Q47" s="66"/>
-      <c r="R47" s="206"/>
+      <c r="R47" s="152"/>
       <c r="S47" s="67"/>
-      <c r="T47" s="206"/>
+      <c r="T47" s="152"/>
       <c r="U47" s="68"/>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="40"/>
-      <c r="D48" s="180"/>
-      <c r="E48" s="180"/>
+      <c r="D48" s="170"/>
+      <c r="E48" s="170"/>
       <c r="F48" s="23"/>
       <c r="G48" s="1"/>
       <c r="H48" s="64"/>
@@ -3465,19 +3444,19 @@
       <c r="M48" s="37"/>
       <c r="N48" s="38"/>
       <c r="O48" s="39"/>
-      <c r="P48" s="206"/>
+      <c r="P48" s="152"/>
       <c r="Q48" s="66"/>
-      <c r="R48" s="206"/>
+      <c r="R48" s="152"/>
       <c r="S48" s="67"/>
-      <c r="T48" s="208"/>
+      <c r="T48" s="154"/>
       <c r="U48" s="68"/>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="40"/>
-      <c r="D49" s="180"/>
-      <c r="E49" s="180"/>
+      <c r="D49" s="170"/>
+      <c r="E49" s="170"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
       <c r="H49" s="46"/>
@@ -3487,11 +3466,11 @@
       <c r="M49" s="37"/>
       <c r="N49" s="38"/>
       <c r="O49" s="39"/>
-      <c r="P49" s="206"/>
+      <c r="P49" s="152"/>
       <c r="Q49" s="66"/>
-      <c r="R49" s="206"/>
+      <c r="R49" s="152"/>
       <c r="S49" s="67"/>
-      <c r="T49" s="208"/>
+      <c r="T49" s="154"/>
       <c r="U49" s="68"/>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.3">
@@ -3509,19 +3488,19 @@
       <c r="M50" s="37"/>
       <c r="N50" s="38"/>
       <c r="O50" s="39"/>
-      <c r="P50" s="206"/>
+      <c r="P50" s="152"/>
       <c r="Q50" s="66"/>
-      <c r="R50" s="206"/>
+      <c r="R50" s="152"/>
       <c r="S50" s="67"/>
-      <c r="T50" s="208"/>
+      <c r="T50" s="154"/>
       <c r="U50" s="68"/>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="40"/>
-      <c r="D51" s="190"/>
-      <c r="E51" s="190"/>
+      <c r="D51" s="185"/>
+      <c r="E51" s="185"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="46"/>
@@ -3531,19 +3510,19 @@
       <c r="M51" s="37"/>
       <c r="N51" s="38"/>
       <c r="O51" s="39"/>
-      <c r="P51" s="205"/>
+      <c r="P51" s="151"/>
       <c r="Q51" s="66"/>
-      <c r="R51" s="206"/>
+      <c r="R51" s="152"/>
       <c r="S51" s="67"/>
-      <c r="T51" s="208"/>
+      <c r="T51" s="154"/>
       <c r="U51" s="68"/>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A52" s="20"/>
       <c r="B52" s="51"/>
       <c r="C52" s="40"/>
-      <c r="D52" s="202"/>
-      <c r="E52" s="202"/>
+      <c r="D52" s="178"/>
+      <c r="E52" s="178"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="46"/>
@@ -3553,19 +3532,19 @@
       <c r="M52" s="37"/>
       <c r="N52" s="38"/>
       <c r="O52" s="39"/>
-      <c r="P52" s="205"/>
+      <c r="P52" s="151"/>
       <c r="Q52" s="66"/>
-      <c r="R52" s="206"/>
+      <c r="R52" s="152"/>
       <c r="S52" s="67"/>
-      <c r="T52" s="208"/>
+      <c r="T52" s="154"/>
       <c r="U52" s="68"/>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A53" s="25"/>
       <c r="B53" s="51"/>
       <c r="C53" s="40"/>
-      <c r="D53" s="189"/>
-      <c r="E53" s="189"/>
+      <c r="D53" s="166"/>
+      <c r="E53" s="166"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="46"/>
@@ -3575,19 +3554,19 @@
       <c r="M53" s="37"/>
       <c r="N53" s="38"/>
       <c r="O53" s="39"/>
-      <c r="P53" s="206"/>
+      <c r="P53" s="152"/>
       <c r="Q53" s="66"/>
-      <c r="R53" s="206"/>
+      <c r="R53" s="152"/>
       <c r="S53" s="67"/>
-      <c r="T53" s="208"/>
+      <c r="T53" s="154"/>
       <c r="U53" s="68"/>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A54" s="20"/>
       <c r="B54" s="51"/>
       <c r="C54" s="40"/>
-      <c r="D54" s="189"/>
-      <c r="E54" s="189"/>
+      <c r="D54" s="166"/>
+      <c r="E54" s="166"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="46"/>
@@ -3597,11 +3576,11 @@
       <c r="M54" s="37"/>
       <c r="N54" s="38"/>
       <c r="O54" s="39"/>
-      <c r="P54" s="206"/>
+      <c r="P54" s="152"/>
       <c r="Q54" s="66"/>
-      <c r="R54" s="206"/>
+      <c r="R54" s="152"/>
       <c r="S54" s="67"/>
-      <c r="T54" s="208"/>
+      <c r="T54" s="154"/>
       <c r="U54" s="68"/>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.3">
@@ -3619,11 +3598,11 @@
       <c r="M55" s="37"/>
       <c r="N55" s="38"/>
       <c r="O55" s="39"/>
-      <c r="P55" s="206"/>
+      <c r="P55" s="152"/>
       <c r="Q55" s="66"/>
-      <c r="R55" s="206"/>
+      <c r="R55" s="152"/>
       <c r="S55" s="67"/>
-      <c r="T55" s="208"/>
+      <c r="T55" s="154"/>
       <c r="U55" s="68"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.3">
@@ -3641,11 +3620,11 @@
       <c r="M56" s="37"/>
       <c r="N56" s="38"/>
       <c r="O56" s="39"/>
-      <c r="P56" s="206"/>
+      <c r="P56" s="152"/>
       <c r="Q56" s="66"/>
-      <c r="R56" s="206"/>
+      <c r="R56" s="152"/>
       <c r="S56" s="67"/>
-      <c r="T56" s="208"/>
+      <c r="T56" s="154"/>
       <c r="U56" s="68"/>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.3">
@@ -3663,11 +3642,11 @@
       <c r="M57" s="37"/>
       <c r="N57" s="38"/>
       <c r="O57" s="39"/>
-      <c r="P57" s="206"/>
+      <c r="P57" s="152"/>
       <c r="Q57" s="66"/>
-      <c r="R57" s="206"/>
+      <c r="R57" s="152"/>
       <c r="S57" s="67"/>
-      <c r="T57" s="208"/>
+      <c r="T57" s="154"/>
       <c r="U57" s="68"/>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.3">
@@ -3685,11 +3664,11 @@
       <c r="M58" s="37"/>
       <c r="N58" s="38"/>
       <c r="O58" s="39"/>
-      <c r="P58" s="206"/>
+      <c r="P58" s="152"/>
       <c r="Q58" s="66"/>
-      <c r="R58" s="206"/>
+      <c r="R58" s="152"/>
       <c r="S58" s="67"/>
-      <c r="T58" s="208"/>
+      <c r="T58" s="154"/>
       <c r="U58" s="68"/>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.3">
@@ -3707,19 +3686,19 @@
       <c r="M59" s="37"/>
       <c r="N59" s="38"/>
       <c r="O59" s="39"/>
-      <c r="P59" s="206"/>
+      <c r="P59" s="152"/>
       <c r="Q59" s="66"/>
-      <c r="R59" s="206"/>
+      <c r="R59" s="152"/>
       <c r="S59" s="67"/>
-      <c r="T59" s="208"/>
+      <c r="T59" s="154"/>
       <c r="U59" s="68"/>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="40"/>
-      <c r="D60" s="189"/>
-      <c r="E60" s="189"/>
+      <c r="D60" s="166"/>
+      <c r="E60" s="166"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="46"/>
@@ -3729,11 +3708,11 @@
       <c r="M60" s="37"/>
       <c r="N60" s="38"/>
       <c r="O60" s="39"/>
-      <c r="P60" s="206"/>
+      <c r="P60" s="152"/>
       <c r="Q60" s="66"/>
-      <c r="R60" s="206"/>
+      <c r="R60" s="152"/>
       <c r="S60" s="67"/>
-      <c r="T60" s="208"/>
+      <c r="T60" s="154"/>
       <c r="U60" s="68"/>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.3">
@@ -3751,11 +3730,11 @@
       <c r="M61" s="37"/>
       <c r="N61" s="38"/>
       <c r="O61" s="39"/>
-      <c r="P61" s="206"/>
+      <c r="P61" s="152"/>
       <c r="Q61" s="135"/>
-      <c r="R61" s="209"/>
+      <c r="R61" s="155"/>
       <c r="S61" s="88"/>
-      <c r="T61" s="208"/>
+      <c r="T61" s="154"/>
       <c r="U61" s="68"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.3">
@@ -3773,11 +3752,11 @@
       <c r="M62" s="37"/>
       <c r="N62" s="38"/>
       <c r="O62" s="39"/>
-      <c r="P62" s="206"/>
+      <c r="P62" s="152"/>
       <c r="Q62" s="135"/>
-      <c r="R62" s="209"/>
+      <c r="R62" s="155"/>
       <c r="S62" s="88"/>
-      <c r="T62" s="208"/>
+      <c r="T62" s="154"/>
       <c r="U62" s="68"/>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.3">
@@ -3795,19 +3774,19 @@
       <c r="M63" s="37"/>
       <c r="N63" s="38"/>
       <c r="O63" s="39"/>
-      <c r="P63" s="206"/>
+      <c r="P63" s="152"/>
       <c r="Q63" s="135"/>
-      <c r="R63" s="209"/>
+      <c r="R63" s="155"/>
       <c r="S63" s="88"/>
-      <c r="T63" s="208"/>
+      <c r="T63" s="154"/>
       <c r="U63" s="68"/>
     </row>
     <row r="64" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="40"/>
-      <c r="D64" s="189"/>
-      <c r="E64" s="189"/>
+      <c r="D64" s="166"/>
+      <c r="E64" s="166"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="46"/>
@@ -3817,29 +3796,29 @@
       <c r="M64" s="37"/>
       <c r="N64" s="38"/>
       <c r="O64" s="39"/>
-      <c r="P64" s="206"/>
+      <c r="P64" s="152"/>
       <c r="Q64" s="84"/>
-      <c r="R64" s="209"/>
+      <c r="R64" s="155"/>
       <c r="S64" s="88"/>
-      <c r="T64" s="208"/>
+      <c r="T64" s="154"/>
       <c r="U64" s="71"/>
     </row>
     <row r="65" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="40"/>
-      <c r="D65" s="189"/>
-      <c r="E65" s="189"/>
+      <c r="D65" s="166"/>
+      <c r="E65" s="166"/>
       <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="46"/>
       <c r="I65" s="50"/>
       <c r="J65" s="53"/>
       <c r="L65"/>
-      <c r="M65" s="159" t="s">
+      <c r="M65" s="171" t="s">
         <v>34</v>
       </c>
-      <c r="N65" s="196"/>
+      <c r="N65" s="172"/>
       <c r="O65" s="42" t="s">
         <v>65</v>
       </c>
@@ -3866,8 +3845,8 @@
       <c r="A66" s="25"/>
       <c r="B66"/>
       <c r="C66" s="90"/>
-      <c r="D66" s="189"/>
-      <c r="E66" s="189"/>
+      <c r="D66" s="166"/>
+      <c r="E66" s="166"/>
       <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="46"/>
@@ -3895,29 +3874,29 @@
       <c r="I67" s="50"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="181" t="s">
+      <c r="M67" s="167" t="s">
         <v>47</v>
       </c>
-      <c r="N67" s="204"/>
-      <c r="O67" s="182"/>
-      <c r="P67" s="191"/>
-      <c r="Q67" s="192"/>
-      <c r="R67" s="181" t="s">
+      <c r="N67" s="168"/>
+      <c r="O67" s="169"/>
+      <c r="P67" s="181"/>
+      <c r="Q67" s="182"/>
+      <c r="R67" s="167" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="204"/>
-      <c r="T67" s="187" t="str">
+      <c r="S67" s="168"/>
+      <c r="T67" s="183" t="str">
         <f>Q25</f>
         <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
-      <c r="U67" s="188"/>
+      <c r="U67" s="184"/>
     </row>
     <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="189"/>
-      <c r="E68" s="189"/>
+      <c r="D68" s="166"/>
+      <c r="E68" s="166"/>
       <c r="F68" s="63"/>
       <c r="G68" s="1"/>
       <c r="H68" s="46"/>
@@ -3938,33 +3917,33 @@
       <c r="A69" s="25"/>
       <c r="B69" s="90"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="189"/>
-      <c r="E69" s="189"/>
+      <c r="D69" s="166"/>
+      <c r="E69" s="166"/>
       <c r="F69" s="63"/>
       <c r="G69" s="1"/>
       <c r="H69" s="46"/>
       <c r="I69" s="50"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="159" t="s">
+      <c r="M69" s="171" t="s">
         <v>35</v>
       </c>
-      <c r="N69" s="160"/>
-      <c r="O69" s="160"/>
-      <c r="P69" s="160"/>
-      <c r="Q69" s="160"/>
-      <c r="R69" s="160"/>
-      <c r="S69" s="160"/>
-      <c r="T69" s="160"/>
-      <c r="U69" s="203"/>
+      <c r="N69" s="179"/>
+      <c r="O69" s="179"/>
+      <c r="P69" s="179"/>
+      <c r="Q69" s="179"/>
+      <c r="R69" s="179"/>
+      <c r="S69" s="179"/>
+      <c r="T69" s="179"/>
+      <c r="U69" s="180"/>
       <c r="V69" s="51"/>
     </row>
     <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
       <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="189"/>
-      <c r="E70" s="189"/>
+      <c r="D70" s="166"/>
+      <c r="E70" s="166"/>
       <c r="F70" s="63"/>
       <c r="G70" s="1"/>
       <c r="H70" s="46"/>
@@ -4001,8 +3980,8 @@
       <c r="A71" s="25"/>
       <c r="B71" s="115"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="189"/>
-      <c r="E71" s="189"/>
+      <c r="D71" s="166"/>
+      <c r="E71" s="166"/>
       <c r="F71" s="63"/>
       <c r="G71" s="1"/>
       <c r="H71" s="46"/>
@@ -4022,10 +4001,10 @@
         <v>87</v>
       </c>
       <c r="Q71" s="61"/>
-      <c r="R71" s="201" t="s">
+      <c r="R71" s="177" t="s">
         <v>6</v>
       </c>
-      <c r="S71" s="201"/>
+      <c r="S71" s="177"/>
       <c r="T71" s="133" t="s">
         <v>88</v>
       </c>
@@ -4037,8 +4016,8 @@
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B72" s="51"/>
       <c r="C72" s="89"/>
-      <c r="D72" s="189"/>
-      <c r="E72" s="189"/>
+      <c r="D72" s="166"/>
+      <c r="E72" s="166"/>
       <c r="F72" s="63"/>
       <c r="I72" s="115"/>
       <c r="L72"/>
@@ -4047,8 +4026,8 @@
       <c r="O72" s="18"/>
       <c r="P72" s="87"/>
       <c r="Q72" s="56"/>
-      <c r="R72" s="199"/>
-      <c r="S72" s="199"/>
+      <c r="R72" s="175"/>
+      <c r="S72" s="175"/>
       <c r="T72" s="65"/>
       <c r="U72" s="95"/>
       <c r="V72" s="51"/>
@@ -4075,10 +4054,10 @@
         <v>92</v>
       </c>
       <c r="Q73" s="56"/>
-      <c r="R73" s="199" t="s">
+      <c r="R73" s="175" t="s">
         <v>10</v>
       </c>
-      <c r="S73" s="199"/>
+      <c r="S73" s="175"/>
       <c r="T73" s="65" t="s">
         <v>93</v>
       </c>
@@ -4094,8 +4073,8 @@
       <c r="O74" s="123"/>
       <c r="P74" s="87"/>
       <c r="Q74" s="56"/>
-      <c r="R74" s="199"/>
-      <c r="S74" s="199"/>
+      <c r="R74" s="175"/>
+      <c r="S74" s="175"/>
       <c r="T74" s="65"/>
       <c r="U74" s="95"/>
       <c r="V74" s="51"/>
@@ -4109,10 +4088,10 @@
       <c r="O75" s="139"/>
       <c r="P75" s="140"/>
       <c r="Q75" s="141"/>
-      <c r="R75" s="200"/>
-      <c r="S75" s="200"/>
-      <c r="T75" s="197"/>
-      <c r="U75" s="198"/>
+      <c r="R75" s="176"/>
+      <c r="S75" s="176"/>
+      <c r="T75" s="173"/>
+      <c r="U75" s="174"/>
       <c r="V75" s="51"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4126,8 +4105,8 @@
       <c r="Q76" s="141"/>
       <c r="R76" s="142"/>
       <c r="S76" s="142"/>
-      <c r="T76" s="197"/>
-      <c r="U76" s="198"/>
+      <c r="T76" s="173"/>
+      <c r="U76" s="174"/>
       <c r="V76" s="51"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4305,48 +4284,17 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T75:U75"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="M69:U69"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="T67:U67"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="O32:P32"/>
     <mergeCell ref="M22:U22"/>
     <mergeCell ref="Q26:S26"/>
     <mergeCell ref="O29:P29"/>
@@ -4363,18 +4311,49 @@
     <mergeCell ref="N23:S23"/>
     <mergeCell ref="N24:S24"/>
     <mergeCell ref="T25:U25"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="M35:O35"/>
     <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="M69:U69"/>
+    <mergeCell ref="R67:S67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="P67:Q67"/>
+    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D51:E51"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(excel): reparación con qwen-max de render.ts
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD33005-EBB4-4B92-8E86-6A1E6A6B1D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CE3932-A707-489F-9A00-25060A485336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1447,164 +1447,164 @@
     <xf numFmtId="42" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1641,9 +1641,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>365616</xdr:colOff>
+      <xdr:colOff>361806</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>133262</xdr:rowOff>
+      <xdr:rowOff>137072</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2698,17 +2698,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="177" t="s">
+      <c r="M22" s="197" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="177"/>
-      <c r="O22" s="177"/>
-      <c r="P22" s="177"/>
-      <c r="Q22" s="177"/>
-      <c r="R22" s="177"/>
-      <c r="S22" s="177"/>
-      <c r="T22" s="177"/>
-      <c r="U22" s="177"/>
+      <c r="N22" s="197"/>
+      <c r="O22" s="197"/>
+      <c r="P22" s="197"/>
+      <c r="Q22" s="197"/>
+      <c r="R22" s="197"/>
+      <c r="S22" s="197"/>
+      <c r="T22" s="197"/>
+      <c r="U22" s="197"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2717,14 +2717,14 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="184" t="s">
+      <c r="N23" s="206" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="185"/>
-      <c r="P23" s="185"/>
-      <c r="Q23" s="185"/>
-      <c r="R23" s="185"/>
-      <c r="S23" s="186"/>
+      <c r="O23" s="207"/>
+      <c r="P23" s="207"/>
+      <c r="Q23" s="207"/>
+      <c r="R23" s="207"/>
+      <c r="S23" s="208"/>
       <c r="T23" s="118" t="s">
         <v>38</v>
       </c>
@@ -2742,14 +2742,14 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="187" t="s">
+      <c r="N24" s="209" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="188"/>
-      <c r="P24" s="188"/>
-      <c r="Q24" s="188"/>
-      <c r="R24" s="188"/>
-      <c r="S24" s="189"/>
+      <c r="O24" s="210"/>
+      <c r="P24" s="210"/>
+      <c r="Q24" s="210"/>
+      <c r="R24" s="210"/>
+      <c r="S24" s="211"/>
       <c r="T24" s="107" t="s">
         <v>11</v>
       </c>
@@ -2769,10 +2769,10 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="165" t="s">
+      <c r="M25" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="166"/>
+      <c r="N25" s="215"/>
       <c r="O25" s="147"/>
       <c r="P25" s="148"/>
       <c r="Q25" s="144" t="s">
@@ -2780,10 +2780,10 @@
       </c>
       <c r="R25" s="145"/>
       <c r="S25" s="146"/>
-      <c r="T25" s="190" t="s">
+      <c r="T25" s="212" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="191"/>
+      <c r="U25" s="213"/>
       <c r="V25" s="13"/>
       <c r="W25" s="81" t="s">
         <v>45</v>
@@ -2799,11 +2799,11 @@
       <c r="N26" s="79"/>
       <c r="O26" s="125"/>
       <c r="P26" s="126"/>
-      <c r="Q26" s="169" t="s">
+      <c r="Q26" s="187" t="s">
         <v>95</v>
       </c>
-      <c r="R26" s="170"/>
-      <c r="S26" s="171"/>
+      <c r="R26" s="188"/>
+      <c r="S26" s="189"/>
       <c r="T26" s="123"/>
       <c r="U26" s="124"/>
       <c r="V26" s="13"/>
@@ -2823,17 +2823,17 @@
         <v>18</v>
       </c>
       <c r="N27" s="79"/>
-      <c r="O27" s="167"/>
-      <c r="P27" s="176"/>
-      <c r="Q27" s="169" t="s">
+      <c r="O27" s="185"/>
+      <c r="P27" s="186"/>
+      <c r="Q27" s="187" t="s">
         <v>64</v>
       </c>
-      <c r="R27" s="170"/>
-      <c r="S27" s="171"/>
-      <c r="T27" s="182" t="s">
+      <c r="R27" s="188"/>
+      <c r="S27" s="189"/>
+      <c r="T27" s="204" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="183"/>
+      <c r="U27" s="205"/>
       <c r="V27" s="19"/>
       <c r="W27" s="91" t="s">
         <v>76</v>
@@ -2849,21 +2849,21 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="174" t="s">
+      <c r="M28" s="202" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="175"/>
-      <c r="O28" s="167"/>
-      <c r="P28" s="176"/>
-      <c r="Q28" s="169" t="s">
+      <c r="N28" s="203"/>
+      <c r="O28" s="185"/>
+      <c r="P28" s="186"/>
+      <c r="Q28" s="187" t="s">
         <v>65</v>
       </c>
-      <c r="R28" s="170"/>
-      <c r="S28" s="171"/>
-      <c r="T28" s="180" t="s">
+      <c r="R28" s="188"/>
+      <c r="S28" s="189"/>
+      <c r="T28" s="200" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="181"/>
+      <c r="U28" s="201"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2878,21 +2878,21 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="174" t="s">
+      <c r="M29" s="202" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="175"/>
-      <c r="O29" s="167"/>
-      <c r="P29" s="176"/>
-      <c r="Q29" s="169" t="s">
+      <c r="N29" s="203"/>
+      <c r="O29" s="185"/>
+      <c r="P29" s="186"/>
+      <c r="Q29" s="187" t="s">
         <v>66</v>
       </c>
-      <c r="R29" s="170"/>
-      <c r="S29" s="171"/>
-      <c r="T29" s="178" t="s">
+      <c r="R29" s="188"/>
+      <c r="S29" s="189"/>
+      <c r="T29" s="198" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="179"/>
+      <c r="U29" s="199"/>
       <c r="W29" s="92" t="str">
         <f>U23</f>
         <v>{{extraction.cant_fact.valor}}</v>
@@ -2909,21 +2909,21 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="174" t="s">
+      <c r="M30" s="202" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="175"/>
-      <c r="O30" s="167"/>
-      <c r="P30" s="168"/>
-      <c r="Q30" s="169" t="s">
+      <c r="N30" s="203"/>
+      <c r="O30" s="185"/>
+      <c r="P30" s="216"/>
+      <c r="Q30" s="187" t="s">
         <v>67</v>
       </c>
-      <c r="R30" s="170"/>
-      <c r="S30" s="171"/>
-      <c r="T30" s="172" t="s">
+      <c r="R30" s="188"/>
+      <c r="S30" s="189"/>
+      <c r="T30" s="217" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="173"/>
+      <c r="U30" s="218"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2941,17 +2941,17 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="174" t="s">
+      <c r="M31" s="202" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="175"/>
-      <c r="O31" s="167"/>
-      <c r="P31" s="176"/>
-      <c r="Q31" s="169" t="s">
+      <c r="N31" s="203"/>
+      <c r="O31" s="185"/>
+      <c r="P31" s="186"/>
+      <c r="Q31" s="187" t="s">
         <v>68</v>
       </c>
-      <c r="R31" s="170"/>
-      <c r="S31" s="171"/>
+      <c r="R31" s="188"/>
+      <c r="S31" s="189"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2966,17 +2966,17 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="174" t="s">
+      <c r="M32" s="202" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="175"/>
-      <c r="O32" s="167"/>
-      <c r="P32" s="176"/>
-      <c r="Q32" s="169" t="s">
+      <c r="N32" s="203"/>
+      <c r="O32" s="185"/>
+      <c r="P32" s="186"/>
+      <c r="Q32" s="187" t="s">
         <v>69</v>
       </c>
-      <c r="R32" s="170"/>
-      <c r="S32" s="171"/>
+      <c r="R32" s="188"/>
+      <c r="S32" s="189"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="81" t="s">
@@ -2998,13 +2998,13 @@
         <v>25</v>
       </c>
       <c r="N33" s="80"/>
-      <c r="O33" s="167"/>
-      <c r="P33" s="176"/>
-      <c r="Q33" s="169" t="s">
+      <c r="O33" s="185"/>
+      <c r="P33" s="186"/>
+      <c r="Q33" s="187" t="s">
         <v>70</v>
       </c>
-      <c r="R33" s="170"/>
-      <c r="S33" s="171"/>
+      <c r="R33" s="188"/>
+      <c r="S33" s="189"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="116" t="e">
@@ -3023,17 +3023,17 @@
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="195" t="s">
+      <c r="M34" s="190" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="196"/>
-      <c r="O34" s="197"/>
-      <c r="P34" s="198"/>
-      <c r="Q34" s="169" t="s">
+      <c r="N34" s="191"/>
+      <c r="O34" s="192"/>
+      <c r="P34" s="193"/>
+      <c r="Q34" s="187" t="s">
         <v>71</v>
       </c>
-      <c r="R34" s="170"/>
-      <c r="S34" s="171"/>
+      <c r="R34" s="188"/>
+      <c r="S34" s="189"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3051,23 +3051,23 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="199" t="s">
+      <c r="M35" s="194" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="200"/>
-      <c r="O35" s="201"/>
-      <c r="P35" s="193" t="s">
+      <c r="N35" s="195"/>
+      <c r="O35" s="196"/>
+      <c r="P35" s="165" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="194"/>
-      <c r="R35" s="193" t="s">
+      <c r="Q35" s="167"/>
+      <c r="R35" s="165" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="194"/>
-      <c r="T35" s="193" t="s">
+      <c r="S35" s="167"/>
+      <c r="T35" s="165" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="194"/>
+      <c r="U35" s="167"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3114,14 +3114,8 @@
     </row>
     <row r="37" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
-      <c r="I37" s="108">
-        <f>L$1</f>
-        <v>0</v>
-      </c>
-      <c r="J37" s="27">
-        <f>L9</f>
-        <v>0</v>
-      </c>
+      <c r="I37" s="13"/>
+      <c r="J37" s="52"/>
       <c r="K37" s="24"/>
       <c r="L37"/>
       <c r="M37" s="37" t="s">
@@ -3159,19 +3153,13 @@
     <row r="38" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="20"/>
       <c r="C38" s="32"/>
-      <c r="I38" s="108">
-        <f>M$1</f>
-        <v>0</v>
-      </c>
-      <c r="J38" s="27">
-        <f t="shared" ref="J38:J45" si="6">L10</f>
-        <v>0</v>
-      </c>
+      <c r="I38" s="13"/>
+      <c r="J38" s="52"/>
       <c r="L38" s="104"/>
-      <c r="M38" s="202" t="s">
+      <c r="M38" s="169" t="s">
         <v>42</v>
       </c>
-      <c r="N38" s="203"/>
+      <c r="N38" s="179"/>
       <c r="O38" s="149" t="s">
         <v>64</v>
       </c>
@@ -3187,14 +3175,8 @@
     <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B39" s="20"/>
       <c r="C39" s="32"/>
-      <c r="I39" s="108">
-        <f>N$1</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I39" s="13"/>
+      <c r="J39" s="52"/>
       <c r="K39" s="24"/>
       <c r="L39" s="104"/>
       <c r="M39" s="37" t="s">
@@ -3220,14 +3202,8 @@
       <c r="C40" s="32"/>
       <c r="D40" s="43"/>
       <c r="E40" s="42"/>
-      <c r="I40" s="108">
-        <f>O$1</f>
-        <v>0</v>
-      </c>
-      <c r="J40" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I40" s="13"/>
+      <c r="J40" s="52"/>
       <c r="K40" s="24"/>
       <c r="L40" s="104"/>
       <c r="M40" s="37"/>
@@ -3247,14 +3223,8 @@
       <c r="C41" s="32"/>
       <c r="D41" s="23"/>
       <c r="E41" s="23"/>
-      <c r="I41" s="108">
-        <f>P$1</f>
-        <v>0</v>
-      </c>
-      <c r="J41" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I41" s="13"/>
+      <c r="J41" s="52"/>
       <c r="K41" s="24"/>
       <c r="L41" s="104"/>
       <c r="M41" s="37"/>
@@ -3275,14 +3245,8 @@
       <c r="D42" s="23"/>
       <c r="E42" s="23"/>
       <c r="F42" s="46"/>
-      <c r="I42" s="108">
-        <f>Q$1</f>
-        <v>0</v>
-      </c>
-      <c r="J42" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I42" s="13"/>
+      <c r="J42" s="52"/>
       <c r="L42" s="104"/>
       <c r="M42" s="37"/>
       <c r="N42" s="38"/>
@@ -3300,18 +3264,12 @@
       <c r="A43" s="103"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="192"/>
-      <c r="E43" s="192"/>
+      <c r="D43" s="168"/>
+      <c r="E43" s="168"/>
       <c r="F43" s="46"/>
       <c r="G43" s="8"/>
-      <c r="I43" s="108">
-        <f>R$1</f>
-        <v>0</v>
-      </c>
-      <c r="J43" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I43" s="13"/>
+      <c r="J43" s="52"/>
       <c r="K43" s="24"/>
       <c r="L43" s="104"/>
       <c r="M43" s="37"/>
@@ -3328,18 +3286,12 @@
       <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="192"/>
-      <c r="E44" s="192"/>
+      <c r="D44" s="168"/>
+      <c r="E44" s="168"/>
       <c r="F44" s="47"/>
       <c r="H44" s="63"/>
-      <c r="I44" s="108">
-        <f>S$1</f>
-        <v>0</v>
-      </c>
-      <c r="J44" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I44" s="13"/>
+      <c r="J44" s="52"/>
       <c r="K44" s="24"/>
       <c r="L44" s="104"/>
       <c r="M44" s="37"/>
@@ -3356,18 +3308,12 @@
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="40"/>
-      <c r="D45" s="192"/>
-      <c r="E45" s="192"/>
+      <c r="D45" s="168"/>
+      <c r="E45" s="168"/>
       <c r="F45" s="23"/>
       <c r="H45" s="63"/>
-      <c r="I45" s="108">
-        <f t="shared" ref="I30:I45" si="7">C$1</f>
-        <v>0</v>
-      </c>
-      <c r="J45" s="27">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
+      <c r="I45" s="13"/>
+      <c r="J45" s="52"/>
       <c r="L45" s="104"/>
       <c r="M45" s="37"/>
       <c r="N45" s="38"/>
@@ -3383,15 +3329,12 @@
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="40"/>
-      <c r="D46" s="192"/>
-      <c r="E46" s="192"/>
+      <c r="D46" s="168"/>
+      <c r="E46" s="168"/>
       <c r="F46" s="48"/>
       <c r="H46" s="63"/>
-      <c r="I46" s="108"/>
-      <c r="J46" s="52">
-        <f>SUM(J28:J45)</f>
-        <v>0</v>
-      </c>
+      <c r="I46" s="13"/>
+      <c r="J46" s="52"/>
       <c r="L46" s="104"/>
       <c r="M46" s="37"/>
       <c r="N46" s="38"/>
@@ -3407,8 +3350,8 @@
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="40"/>
-      <c r="D47" s="192"/>
-      <c r="E47" s="192"/>
+      <c r="D47" s="168"/>
+      <c r="E47" s="168"/>
       <c r="F47" s="17"/>
       <c r="G47" s="1"/>
       <c r="H47" s="63"/>
@@ -3430,8 +3373,8 @@
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="40"/>
-      <c r="D48" s="192"/>
-      <c r="E48" s="192"/>
+      <c r="D48" s="168"/>
+      <c r="E48" s="168"/>
       <c r="F48" s="23"/>
       <c r="G48" s="1"/>
       <c r="H48" s="63"/>
@@ -3452,8 +3395,8 @@
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="40"/>
-      <c r="D49" s="192"/>
-      <c r="E49" s="192"/>
+      <c r="D49" s="168"/>
+      <c r="E49" s="168"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
       <c r="H49" s="45"/>
@@ -3496,8 +3439,8 @@
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="40"/>
-      <c r="D51" s="218"/>
-      <c r="E51" s="218"/>
+      <c r="D51" s="171"/>
+      <c r="E51" s="171"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="45"/>
@@ -3518,8 +3461,8 @@
       <c r="A52" s="20"/>
       <c r="B52" s="50"/>
       <c r="C52" s="40"/>
-      <c r="D52" s="205"/>
-      <c r="E52" s="205"/>
+      <c r="D52" s="178"/>
+      <c r="E52" s="178"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="45"/>
@@ -3540,8 +3483,8 @@
       <c r="A53" s="25"/>
       <c r="B53" s="50"/>
       <c r="C53" s="40"/>
-      <c r="D53" s="204"/>
-      <c r="E53" s="204"/>
+      <c r="D53" s="177"/>
+      <c r="E53" s="177"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="45"/>
@@ -3562,8 +3505,8 @@
       <c r="A54" s="20"/>
       <c r="B54" s="50"/>
       <c r="C54" s="40"/>
-      <c r="D54" s="204"/>
-      <c r="E54" s="204"/>
+      <c r="D54" s="177"/>
+      <c r="E54" s="177"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="45"/>
@@ -3694,8 +3637,8 @@
       <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="40"/>
-      <c r="D60" s="204"/>
-      <c r="E60" s="204"/>
+      <c r="D60" s="177"/>
+      <c r="E60" s="177"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="45"/>
@@ -3782,8 +3725,8 @@
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="40"/>
-      <c r="D64" s="204"/>
-      <c r="E64" s="204"/>
+      <c r="D64" s="177"/>
+      <c r="E64" s="177"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="45"/>
@@ -3804,18 +3747,18 @@
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="40"/>
-      <c r="D65" s="204"/>
-      <c r="E65" s="204"/>
+      <c r="D65" s="177"/>
+      <c r="E65" s="177"/>
       <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="45"/>
       <c r="I65" s="49"/>
       <c r="J65" s="52"/>
       <c r="L65"/>
-      <c r="M65" s="202" t="s">
+      <c r="M65" s="169" t="s">
         <v>34</v>
       </c>
-      <c r="N65" s="217"/>
+      <c r="N65" s="170"/>
       <c r="O65" s="41" t="s">
         <v>65</v>
       </c>
@@ -3842,8 +3785,8 @@
       <c r="A66" s="25"/>
       <c r="B66"/>
       <c r="C66" s="89"/>
-      <c r="D66" s="204"/>
-      <c r="E66" s="204"/>
+      <c r="D66" s="177"/>
+      <c r="E66" s="177"/>
       <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="45"/>
@@ -3871,29 +3814,29 @@
       <c r="I67" s="49"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="193" t="s">
+      <c r="M67" s="165" t="s">
         <v>47</v>
       </c>
-      <c r="N67" s="207"/>
-      <c r="O67" s="194"/>
-      <c r="P67" s="208"/>
-      <c r="Q67" s="209"/>
-      <c r="R67" s="193" t="s">
+      <c r="N67" s="166"/>
+      <c r="O67" s="167"/>
+      <c r="P67" s="181"/>
+      <c r="Q67" s="182"/>
+      <c r="R67" s="165" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="207"/>
-      <c r="T67" s="210" t="str">
+      <c r="S67" s="166"/>
+      <c r="T67" s="183" t="str">
         <f>Q25</f>
         <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
-      <c r="U67" s="211"/>
+      <c r="U67" s="184"/>
     </row>
     <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="204"/>
-      <c r="E68" s="204"/>
+      <c r="D68" s="177"/>
+      <c r="E68" s="177"/>
       <c r="F68" s="62"/>
       <c r="G68" s="1"/>
       <c r="H68" s="45"/>
@@ -3914,33 +3857,33 @@
       <c r="A69" s="25"/>
       <c r="B69" s="89"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="204"/>
-      <c r="E69" s="204"/>
+      <c r="D69" s="177"/>
+      <c r="E69" s="177"/>
       <c r="F69" s="62"/>
       <c r="G69" s="1"/>
       <c r="H69" s="45"/>
       <c r="I69" s="49"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="202" t="s">
+      <c r="M69" s="169" t="s">
         <v>35</v>
       </c>
-      <c r="N69" s="203"/>
-      <c r="O69" s="203"/>
-      <c r="P69" s="203"/>
-      <c r="Q69" s="203"/>
-      <c r="R69" s="203"/>
-      <c r="S69" s="203"/>
-      <c r="T69" s="203"/>
-      <c r="U69" s="206"/>
+      <c r="N69" s="179"/>
+      <c r="O69" s="179"/>
+      <c r="P69" s="179"/>
+      <c r="Q69" s="179"/>
+      <c r="R69" s="179"/>
+      <c r="S69" s="179"/>
+      <c r="T69" s="179"/>
+      <c r="U69" s="180"/>
       <c r="V69" s="50"/>
     </row>
     <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
       <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="204"/>
-      <c r="E70" s="204"/>
+      <c r="D70" s="177"/>
+      <c r="E70" s="177"/>
       <c r="F70" s="62"/>
       <c r="G70" s="1"/>
       <c r="H70" s="45"/>
@@ -3977,8 +3920,8 @@
       <c r="A71" s="25"/>
       <c r="B71" s="114"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="204"/>
-      <c r="E71" s="204"/>
+      <c r="D71" s="177"/>
+      <c r="E71" s="177"/>
       <c r="F71" s="62"/>
       <c r="G71" s="1"/>
       <c r="H71" s="45"/>
@@ -3998,10 +3941,10 @@
         <v>87</v>
       </c>
       <c r="Q71" s="60"/>
-      <c r="R71" s="216" t="s">
+      <c r="R71" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="S71" s="216"/>
+      <c r="S71" s="176"/>
       <c r="T71" s="132" t="s">
         <v>88</v>
       </c>
@@ -4013,8 +3956,8 @@
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B72" s="50"/>
       <c r="C72" s="88"/>
-      <c r="D72" s="204"/>
-      <c r="E72" s="204"/>
+      <c r="D72" s="177"/>
+      <c r="E72" s="177"/>
       <c r="F72" s="62"/>
       <c r="I72" s="114"/>
       <c r="L72"/>
@@ -4023,8 +3966,8 @@
       <c r="O72" s="18"/>
       <c r="P72" s="86"/>
       <c r="Q72" s="55"/>
-      <c r="R72" s="214"/>
-      <c r="S72" s="214"/>
+      <c r="R72" s="174"/>
+      <c r="S72" s="174"/>
       <c r="T72" s="64"/>
       <c r="U72" s="94"/>
       <c r="V72" s="50"/>
@@ -4051,10 +3994,10 @@
         <v>92</v>
       </c>
       <c r="Q73" s="55"/>
-      <c r="R73" s="214" t="s">
+      <c r="R73" s="174" t="s">
         <v>10</v>
       </c>
-      <c r="S73" s="214"/>
+      <c r="S73" s="174"/>
       <c r="T73" s="64" t="s">
         <v>93</v>
       </c>
@@ -4070,8 +4013,8 @@
       <c r="O74" s="122"/>
       <c r="P74" s="86"/>
       <c r="Q74" s="55"/>
-      <c r="R74" s="214"/>
-      <c r="S74" s="214"/>
+      <c r="R74" s="174"/>
+      <c r="S74" s="174"/>
       <c r="T74" s="64"/>
       <c r="U74" s="94"/>
       <c r="V74" s="50"/>
@@ -4085,10 +4028,10 @@
       <c r="O75" s="138"/>
       <c r="P75" s="139"/>
       <c r="Q75" s="140"/>
-      <c r="R75" s="215"/>
-      <c r="S75" s="215"/>
-      <c r="T75" s="212"/>
-      <c r="U75" s="213"/>
+      <c r="R75" s="175"/>
+      <c r="S75" s="175"/>
+      <c r="T75" s="172"/>
+      <c r="U75" s="173"/>
       <c r="V75" s="50"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -4102,8 +4045,8 @@
       <c r="Q76" s="140"/>
       <c r="R76" s="141"/>
       <c r="S76" s="141"/>
-      <c r="T76" s="212"/>
-      <c r="U76" s="213"/>
+      <c r="T76" s="172"/>
+      <c r="U76" s="173"/>
       <c r="V76" s="50"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4281,22 +4224,44 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="M22:U22"/>
+    <mergeCell ref="Q26:S26"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="Q29:S29"/>
+    <mergeCell ref="T29:U29"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="Q28:S28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="Q27:S27"/>
+    <mergeCell ref="T27:U27"/>
+    <mergeCell ref="N23:S23"/>
+    <mergeCell ref="N24:S24"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M38:N38"/>
     <mergeCell ref="D71:E71"/>
     <mergeCell ref="D72:E72"/>
     <mergeCell ref="D52:E52"/>
@@ -4313,44 +4278,22 @@
     <mergeCell ref="D64:E64"/>
     <mergeCell ref="D70:E70"/>
     <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M22:U22"/>
-    <mergeCell ref="Q26:S26"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="Q29:S29"/>
-    <mergeCell ref="T29:U29"/>
-    <mergeCell ref="T28:U28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="Q28:S28"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="Q27:S27"/>
-    <mergeCell ref="T27:U27"/>
-    <mergeCell ref="N23:S23"/>
-    <mergeCell ref="N24:S24"/>
-    <mergeCell ref="T25:U25"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D51:E51"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
manual: modificación de estilo del excel
</commit_message>
<xml_diff>
--- a/templates/RUTA CFT-ABL -2026.xlsx
+++ b/templates/RUTA CFT-ABL -2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CE3932-A707-489F-9A00-25060A485336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100C0C9F-C791-4729-92BF-40C3BDE9C62E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -533,7 +533,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -987,17 +987,6 @@
       </right>
       <top/>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1021,7 +1010,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="219">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1152,18 +1141,6 @@
     <xf numFmtId="167" fontId="9" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1335,12 +1312,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1356,12 +1327,6 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1386,9 +1351,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1401,8 +1363,6 @@
     <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1437,7 +1397,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1447,38 +1407,119 @@
     <xf numFmtId="42" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1487,12 +1528,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1505,106 +1546,22 @@
     <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1975,698 +1932,698 @@
       <c r="A1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="111" t="s">
+      <c r="B1" s="107" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="111"/>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
-      <c r="O1" s="111"/>
-      <c r="P1" s="111"/>
-      <c r="Q1" s="111"/>
-      <c r="R1" s="111"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
+      <c r="C1" s="115"/>
+      <c r="D1" s="115"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="115"/>
+      <c r="G1" s="115"/>
+      <c r="H1" s="107"/>
+      <c r="I1" s="107"/>
+      <c r="J1" s="115"/>
+      <c r="K1" s="115"/>
+      <c r="L1" s="107"/>
+      <c r="M1" s="107"/>
+      <c r="N1" s="107"/>
+      <c r="O1" s="107"/>
+      <c r="P1" s="107"/>
+      <c r="Q1" s="107"/>
+      <c r="R1" s="107"/>
+      <c r="S1" s="115"/>
+      <c r="T1" s="115"/>
       <c r="U1" s="7"/>
       <c r="V1" s="7"/>
-      <c r="W1" s="113"/>
+      <c r="W1" s="109"/>
     </row>
     <row r="2" spans="1:23" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="107" t="s">
         <v>101</v>
       </c>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="111"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="111"/>
-      <c r="I2" s="111"/>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="111"/>
-      <c r="M2" s="111"/>
-      <c r="N2" s="111"/>
-      <c r="O2" s="111"/>
-      <c r="P2" s="111"/>
-      <c r="Q2" s="111"/>
-      <c r="R2" s="120"/>
-      <c r="S2" s="119"/>
-      <c r="T2" s="119"/>
+      <c r="C2" s="115"/>
+      <c r="D2" s="115"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="115"/>
+      <c r="G2" s="121"/>
+      <c r="H2" s="107"/>
+      <c r="I2" s="107"/>
+      <c r="J2" s="115"/>
+      <c r="K2" s="115"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107"/>
+      <c r="O2" s="107"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="116"/>
+      <c r="S2" s="115"/>
+      <c r="T2" s="115"/>
       <c r="U2" s="7"/>
       <c r="V2" s="7"/>
-      <c r="W2" s="113"/>
+      <c r="W2" s="109"/>
     </row>
     <row r="3" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="121" t="s">
+      <c r="A3" s="117" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="119" t="s">
+      <c r="B3" s="115" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="119"/>
-      <c r="D3" s="119"/>
-      <c r="E3" s="119"/>
-      <c r="F3" s="119"/>
-      <c r="G3" s="119"/>
-      <c r="H3" s="119"/>
-      <c r="I3" s="119"/>
-      <c r="J3" s="119"/>
-      <c r="K3" s="119"/>
-      <c r="L3" s="119"/>
-      <c r="M3" s="119"/>
-      <c r="N3" s="119"/>
-      <c r="O3" s="119"/>
-      <c r="P3" s="119"/>
-      <c r="Q3" s="119"/>
-      <c r="R3" s="119"/>
-      <c r="S3" s="119"/>
-      <c r="T3" s="119"/>
-      <c r="U3" s="109"/>
-      <c r="V3" s="162"/>
-      <c r="W3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="115"/>
+      <c r="S3" s="115"/>
+      <c r="T3" s="115"/>
+      <c r="U3" s="105"/>
+      <c r="V3" s="151"/>
+      <c r="W3" s="111"/>
     </row>
     <row r="4" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="121" t="s">
+      <c r="A4" s="117" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="119" t="s">
+      <c r="B4" s="115" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="119"/>
-      <c r="D4" s="119"/>
-      <c r="E4" s="119"/>
-      <c r="F4" s="119"/>
-      <c r="G4" s="119"/>
-      <c r="H4" s="119"/>
-      <c r="I4" s="119"/>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="119"/>
-      <c r="M4" s="119"/>
-      <c r="N4" s="119"/>
-      <c r="O4" s="119"/>
-      <c r="P4" s="119"/>
-      <c r="Q4" s="119"/>
-      <c r="R4" s="119"/>
-      <c r="S4" s="119"/>
-      <c r="T4" s="119"/>
-      <c r="U4" s="109"/>
-      <c r="V4" s="162"/>
-      <c r="W4" s="115"/>
+      <c r="C4" s="115"/>
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="115"/>
+      <c r="I4" s="115"/>
+      <c r="J4" s="115"/>
+      <c r="K4" s="115"/>
+      <c r="L4" s="115"/>
+      <c r="M4" s="115"/>
+      <c r="N4" s="115"/>
+      <c r="O4" s="115"/>
+      <c r="P4" s="115"/>
+      <c r="Q4" s="115"/>
+      <c r="R4" s="115"/>
+      <c r="S4" s="115"/>
+      <c r="T4" s="115"/>
+      <c r="U4" s="105"/>
+      <c r="V4" s="151"/>
+      <c r="W4" s="111"/>
     </row>
     <row r="5" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="121" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="128" t="s">
+      <c r="A5" s="117" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="122" t="s">
         <v>104</v>
       </c>
-      <c r="C5" s="128"/>
-      <c r="D5" s="128"/>
-      <c r="E5" s="128"/>
-      <c r="F5" s="128"/>
-      <c r="G5" s="128"/>
-      <c r="H5" s="128"/>
-      <c r="I5" s="128"/>
-      <c r="J5" s="128"/>
-      <c r="K5" s="128"/>
-      <c r="L5" s="128"/>
-      <c r="M5" s="128"/>
-      <c r="N5" s="128"/>
-      <c r="O5" s="128"/>
-      <c r="P5" s="128"/>
-      <c r="Q5" s="128"/>
-      <c r="R5" s="119"/>
-      <c r="S5" s="119"/>
-      <c r="T5" s="119"/>
-      <c r="U5" s="110"/>
-      <c r="V5" s="110"/>
-      <c r="W5" s="110"/>
+      <c r="C5" s="122"/>
+      <c r="D5" s="122"/>
+      <c r="E5" s="122"/>
+      <c r="F5" s="122"/>
+      <c r="G5" s="122"/>
+      <c r="H5" s="122"/>
+      <c r="I5" s="122"/>
+      <c r="J5" s="122"/>
+      <c r="K5" s="122"/>
+      <c r="L5" s="122"/>
+      <c r="M5" s="122"/>
+      <c r="N5" s="122"/>
+      <c r="O5" s="122"/>
+      <c r="P5" s="122"/>
+      <c r="Q5" s="122"/>
+      <c r="R5" s="115"/>
+      <c r="S5" s="115"/>
+      <c r="T5" s="115"/>
+      <c r="U5" s="106"/>
+      <c r="V5" s="106"/>
+      <c r="W5" s="106"/>
     </row>
     <row r="6" spans="1:23" s="44" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="121" t="s">
+      <c r="A6" s="117" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="119" t="s">
+      <c r="B6" s="115" t="s">
         <v>105</v>
       </c>
-      <c r="C6" s="119"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="119"/>
-      <c r="F6" s="119"/>
-      <c r="G6" s="119"/>
-      <c r="H6" s="119"/>
-      <c r="I6" s="119"/>
-      <c r="J6" s="119"/>
-      <c r="K6" s="119"/>
-      <c r="L6" s="119"/>
-      <c r="M6" s="110"/>
-      <c r="N6" s="110"/>
-      <c r="O6" s="110"/>
-      <c r="P6" s="110"/>
-      <c r="Q6" s="110"/>
-      <c r="R6" s="119"/>
-      <c r="S6" s="119"/>
-      <c r="T6" s="119"/>
-      <c r="U6" s="110"/>
-      <c r="V6" s="110"/>
-      <c r="W6" s="110"/>
+      <c r="C6" s="115"/>
+      <c r="D6" s="115"/>
+      <c r="E6" s="115"/>
+      <c r="F6" s="115"/>
+      <c r="G6" s="115"/>
+      <c r="H6" s="115"/>
+      <c r="I6" s="115"/>
+      <c r="J6" s="115"/>
+      <c r="K6" s="115"/>
+      <c r="L6" s="115"/>
+      <c r="M6" s="106"/>
+      <c r="N6" s="106"/>
+      <c r="O6" s="106"/>
+      <c r="P6" s="106"/>
+      <c r="Q6" s="106"/>
+      <c r="R6" s="115"/>
+      <c r="S6" s="115"/>
+      <c r="T6" s="115"/>
+      <c r="U6" s="106"/>
+      <c r="V6" s="106"/>
+      <c r="W6" s="106"/>
     </row>
     <row r="7" spans="1:23" s="44" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="163" t="s">
+      <c r="B7" s="152" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="163"/>
-      <c r="D7" s="163"/>
-      <c r="E7" s="163"/>
-      <c r="F7" s="163"/>
-      <c r="G7" s="163"/>
-      <c r="H7" s="163"/>
-      <c r="I7" s="163"/>
-      <c r="J7" s="163"/>
-      <c r="K7" s="163"/>
-      <c r="L7" s="163"/>
-      <c r="M7" s="163"/>
-      <c r="N7" s="163"/>
-      <c r="O7" s="163"/>
-      <c r="P7" s="163"/>
-      <c r="Q7" s="163"/>
-      <c r="R7" s="155"/>
-      <c r="S7" s="155"/>
-      <c r="T7" s="155"/>
-      <c r="U7" s="156"/>
-      <c r="V7" s="156"/>
-      <c r="W7" s="156"/>
+      <c r="C7" s="152"/>
+      <c r="D7" s="152"/>
+      <c r="E7" s="152"/>
+      <c r="F7" s="152"/>
+      <c r="G7" s="152"/>
+      <c r="H7" s="152"/>
+      <c r="I7" s="152"/>
+      <c r="J7" s="152"/>
+      <c r="K7" s="152"/>
+      <c r="L7" s="152"/>
+      <c r="M7" s="152"/>
+      <c r="N7" s="152"/>
+      <c r="O7" s="152"/>
+      <c r="P7" s="152"/>
+      <c r="Q7" s="152"/>
+      <c r="R7" s="144"/>
+      <c r="S7" s="144"/>
+      <c r="T7" s="144"/>
+      <c r="U7" s="145"/>
+      <c r="V7" s="145"/>
+      <c r="W7" s="145"/>
     </row>
     <row r="8" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="111"/>
-      <c r="B8" s="156"/>
-      <c r="C8" s="110"/>
-      <c r="D8" s="156"/>
-      <c r="E8" s="110"/>
-      <c r="F8" s="109"/>
-      <c r="G8" s="110"/>
-      <c r="H8" s="156"/>
-      <c r="I8" s="110"/>
-      <c r="J8" s="156"/>
-      <c r="K8" s="110"/>
-      <c r="L8" s="109"/>
-      <c r="M8" s="110"/>
-      <c r="N8" s="109"/>
-      <c r="O8" s="110"/>
-      <c r="P8" s="157"/>
-      <c r="Q8" s="110"/>
-      <c r="R8" s="157"/>
-      <c r="S8" s="110"/>
-      <c r="T8" s="157"/>
-      <c r="U8" s="110"/>
-      <c r="V8" s="109"/>
-      <c r="W8" s="110"/>
-    </row>
-    <row r="9" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="112" t="s">
+      <c r="A8" s="107"/>
+      <c r="B8" s="145"/>
+      <c r="C8" s="106"/>
+      <c r="D8" s="145"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="105"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="145"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="145"/>
+      <c r="K8" s="106"/>
+      <c r="L8" s="105"/>
+      <c r="M8" s="106"/>
+      <c r="N8" s="105"/>
+      <c r="O8" s="106"/>
+      <c r="P8" s="146"/>
+      <c r="Q8" s="106"/>
+      <c r="R8" s="146"/>
+      <c r="S8" s="106"/>
+      <c r="T8" s="146"/>
+      <c r="U8" s="106"/>
+      <c r="V8" s="105"/>
+      <c r="W8" s="106"/>
+    </row>
+    <row r="9" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="108" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="164" t="s">
+      <c r="B9" s="153" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="164"/>
-      <c r="D9" s="164"/>
-      <c r="E9" s="156"/>
-      <c r="F9" s="109"/>
-      <c r="G9" s="156"/>
-      <c r="H9" s="109"/>
-      <c r="I9" s="156"/>
-      <c r="J9" s="109"/>
-      <c r="K9" s="156"/>
-      <c r="L9" s="109"/>
-      <c r="M9" s="156"/>
-      <c r="N9" s="109"/>
-      <c r="O9" s="156"/>
-      <c r="P9" s="157"/>
-      <c r="Q9" s="156"/>
-      <c r="R9" s="157"/>
-      <c r="S9" s="158"/>
-      <c r="T9" s="158"/>
-      <c r="U9" s="156"/>
-      <c r="V9" s="109"/>
-      <c r="W9" s="156"/>
-    </row>
-    <row r="10" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="112" t="s">
+      <c r="C9" s="153"/>
+      <c r="D9" s="153"/>
+      <c r="E9" s="145"/>
+      <c r="F9" s="105"/>
+      <c r="G9" s="145"/>
+      <c r="H9" s="105"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="105"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="105"/>
+      <c r="M9" s="145"/>
+      <c r="N9" s="105"/>
+      <c r="O9" s="145"/>
+      <c r="P9" s="146"/>
+      <c r="Q9" s="145"/>
+      <c r="R9" s="146"/>
+      <c r="S9" s="147"/>
+      <c r="T9" s="147"/>
+      <c r="U9" s="145"/>
+      <c r="V9" s="105"/>
+      <c r="W9" s="145"/>
+    </row>
+    <row r="10" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="164" t="s">
+      <c r="B10" s="153" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="164"/>
-      <c r="D10" s="164"/>
-      <c r="E10" s="156"/>
-      <c r="F10" s="109"/>
-      <c r="G10" s="156"/>
-      <c r="H10" s="109"/>
-      <c r="I10" s="156"/>
-      <c r="J10" s="109"/>
-      <c r="K10" s="156"/>
-      <c r="L10" s="109"/>
-      <c r="M10" s="156"/>
-      <c r="N10" s="109"/>
-      <c r="O10" s="156"/>
-      <c r="P10" s="157"/>
-      <c r="Q10" s="156"/>
-      <c r="R10" s="157"/>
-      <c r="S10" s="158"/>
-      <c r="T10" s="158"/>
-      <c r="U10" s="156"/>
-      <c r="V10" s="109"/>
-      <c r="W10" s="156"/>
-    </row>
-    <row r="11" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="112" t="s">
+      <c r="C10" s="153"/>
+      <c r="D10" s="153"/>
+      <c r="E10" s="145"/>
+      <c r="F10" s="105"/>
+      <c r="G10" s="145"/>
+      <c r="H10" s="105"/>
+      <c r="I10" s="145"/>
+      <c r="J10" s="105"/>
+      <c r="K10" s="145"/>
+      <c r="L10" s="105"/>
+      <c r="M10" s="145"/>
+      <c r="N10" s="105"/>
+      <c r="O10" s="145"/>
+      <c r="P10" s="146"/>
+      <c r="Q10" s="145"/>
+      <c r="R10" s="146"/>
+      <c r="S10" s="147"/>
+      <c r="T10" s="147"/>
+      <c r="U10" s="145"/>
+      <c r="V10" s="105"/>
+      <c r="W10" s="145"/>
+    </row>
+    <row r="11" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="164" t="s">
+      <c r="B11" s="153" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="164"/>
-      <c r="D11" s="164"/>
-      <c r="E11" s="156"/>
-      <c r="F11" s="109"/>
-      <c r="G11" s="156"/>
-      <c r="H11" s="109"/>
-      <c r="I11" s="156"/>
-      <c r="J11" s="109"/>
-      <c r="K11" s="156"/>
-      <c r="L11" s="109"/>
-      <c r="M11" s="156"/>
-      <c r="N11" s="109"/>
-      <c r="O11" s="156"/>
-      <c r="P11" s="157"/>
-      <c r="Q11" s="156"/>
-      <c r="R11" s="157"/>
-      <c r="S11" s="158"/>
-      <c r="T11" s="158"/>
-      <c r="U11" s="156"/>
-      <c r="V11" s="109"/>
-      <c r="W11" s="156"/>
-    </row>
-    <row r="12" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="112" t="s">
+      <c r="C11" s="153"/>
+      <c r="D11" s="153"/>
+      <c r="E11" s="145"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="145"/>
+      <c r="H11" s="105"/>
+      <c r="I11" s="145"/>
+      <c r="J11" s="105"/>
+      <c r="K11" s="145"/>
+      <c r="L11" s="105"/>
+      <c r="M11" s="145"/>
+      <c r="N11" s="105"/>
+      <c r="O11" s="145"/>
+      <c r="P11" s="146"/>
+      <c r="Q11" s="145"/>
+      <c r="R11" s="146"/>
+      <c r="S11" s="147"/>
+      <c r="T11" s="147"/>
+      <c r="U11" s="145"/>
+      <c r="V11" s="105"/>
+      <c r="W11" s="145"/>
+    </row>
+    <row r="12" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="108" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="164" t="s">
+      <c r="B12" s="153" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="164"/>
-      <c r="D12" s="164"/>
-      <c r="E12" s="156"/>
-      <c r="F12" s="109"/>
-      <c r="G12" s="156"/>
-      <c r="H12" s="109"/>
-      <c r="I12" s="156"/>
-      <c r="J12" s="109"/>
-      <c r="K12" s="156"/>
-      <c r="L12" s="109"/>
-      <c r="M12" s="156"/>
-      <c r="N12" s="109"/>
-      <c r="O12" s="156"/>
-      <c r="P12" s="157"/>
-      <c r="Q12" s="156"/>
-      <c r="R12" s="157"/>
-      <c r="S12" s="158"/>
-      <c r="T12" s="158"/>
-      <c r="U12" s="156"/>
-      <c r="V12" s="109"/>
-      <c r="W12" s="156"/>
-    </row>
-    <row r="13" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="112" t="s">
+      <c r="C12" s="153"/>
+      <c r="D12" s="153"/>
+      <c r="E12" s="145"/>
+      <c r="F12" s="105"/>
+      <c r="G12" s="145"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="145"/>
+      <c r="J12" s="105"/>
+      <c r="K12" s="145"/>
+      <c r="L12" s="105"/>
+      <c r="M12" s="145"/>
+      <c r="N12" s="105"/>
+      <c r="O12" s="145"/>
+      <c r="P12" s="146"/>
+      <c r="Q12" s="145"/>
+      <c r="R12" s="146"/>
+      <c r="S12" s="147"/>
+      <c r="T12" s="147"/>
+      <c r="U12" s="145"/>
+      <c r="V12" s="105"/>
+      <c r="W12" s="145"/>
+    </row>
+    <row r="13" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="164" t="s">
+      <c r="B13" s="153" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="164"/>
-      <c r="D13" s="164"/>
-      <c r="E13" s="156"/>
-      <c r="F13" s="109"/>
-      <c r="G13" s="156"/>
-      <c r="H13" s="109"/>
-      <c r="I13" s="156"/>
-      <c r="J13" s="109"/>
-      <c r="K13" s="156"/>
-      <c r="L13" s="109"/>
-      <c r="M13" s="156"/>
-      <c r="N13" s="109"/>
-      <c r="O13" s="156"/>
-      <c r="P13" s="157"/>
-      <c r="Q13" s="156"/>
-      <c r="R13" s="157"/>
-      <c r="S13" s="158"/>
-      <c r="T13" s="158"/>
-      <c r="U13" s="156"/>
-      <c r="V13" s="109"/>
-      <c r="W13" s="156"/>
-    </row>
-    <row r="14" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="112" t="s">
+      <c r="C13" s="153"/>
+      <c r="D13" s="153"/>
+      <c r="E13" s="145"/>
+      <c r="F13" s="105"/>
+      <c r="G13" s="145"/>
+      <c r="H13" s="105"/>
+      <c r="I13" s="145"/>
+      <c r="J13" s="105"/>
+      <c r="K13" s="145"/>
+      <c r="L13" s="105"/>
+      <c r="M13" s="145"/>
+      <c r="N13" s="105"/>
+      <c r="O13" s="145"/>
+      <c r="P13" s="146"/>
+      <c r="Q13" s="145"/>
+      <c r="R13" s="146"/>
+      <c r="S13" s="147"/>
+      <c r="T13" s="147"/>
+      <c r="U13" s="145"/>
+      <c r="V13" s="105"/>
+      <c r="W13" s="145"/>
+    </row>
+    <row r="14" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="108" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="164" t="s">
+      <c r="B14" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="164"/>
-      <c r="D14" s="164"/>
-      <c r="E14" s="156"/>
-      <c r="F14" s="109"/>
-      <c r="G14" s="156"/>
-      <c r="H14" s="109"/>
-      <c r="I14" s="156"/>
-      <c r="J14" s="109"/>
-      <c r="K14" s="156"/>
-      <c r="L14" s="109"/>
-      <c r="M14" s="156"/>
-      <c r="N14" s="109"/>
-      <c r="O14" s="156"/>
-      <c r="P14" s="157"/>
-      <c r="Q14" s="156"/>
-      <c r="R14" s="157"/>
-      <c r="S14" s="158"/>
-      <c r="T14" s="158"/>
-      <c r="U14" s="156"/>
-      <c r="V14" s="109"/>
-      <c r="W14" s="156"/>
-    </row>
-    <row r="15" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="112" t="s">
+      <c r="C14" s="153"/>
+      <c r="D14" s="153"/>
+      <c r="E14" s="145"/>
+      <c r="F14" s="105"/>
+      <c r="G14" s="145"/>
+      <c r="H14" s="105"/>
+      <c r="I14" s="145"/>
+      <c r="J14" s="105"/>
+      <c r="K14" s="145"/>
+      <c r="L14" s="105"/>
+      <c r="M14" s="145"/>
+      <c r="N14" s="105"/>
+      <c r="O14" s="145"/>
+      <c r="P14" s="146"/>
+      <c r="Q14" s="145"/>
+      <c r="R14" s="146"/>
+      <c r="S14" s="147"/>
+      <c r="T14" s="147"/>
+      <c r="U14" s="145"/>
+      <c r="V14" s="105"/>
+      <c r="W14" s="145"/>
+    </row>
+    <row r="15" spans="1:23" s="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="164" t="s">
+      <c r="B15" s="153" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="164"/>
-      <c r="D15" s="164"/>
-      <c r="E15" s="156"/>
-      <c r="F15" s="109"/>
-      <c r="G15" s="156"/>
-      <c r="H15" s="109"/>
-      <c r="I15" s="156"/>
-      <c r="J15" s="109"/>
-      <c r="K15" s="156"/>
-      <c r="L15" s="109"/>
-      <c r="M15" s="156"/>
-      <c r="N15" s="109"/>
-      <c r="O15" s="156"/>
-      <c r="P15" s="157"/>
-      <c r="Q15" s="156"/>
-      <c r="R15" s="157"/>
-      <c r="S15" s="158"/>
-      <c r="T15" s="158"/>
-      <c r="U15" s="156"/>
-      <c r="V15" s="109"/>
-      <c r="W15" s="156"/>
-    </row>
-    <row r="16" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="112" t="s">
+      <c r="C15" s="153"/>
+      <c r="D15" s="153"/>
+      <c r="E15" s="145"/>
+      <c r="F15" s="105"/>
+      <c r="G15" s="145"/>
+      <c r="H15" s="105"/>
+      <c r="I15" s="145"/>
+      <c r="J15" s="105"/>
+      <c r="K15" s="145"/>
+      <c r="L15" s="105"/>
+      <c r="M15" s="145"/>
+      <c r="N15" s="105"/>
+      <c r="O15" s="145"/>
+      <c r="P15" s="146"/>
+      <c r="Q15" s="145"/>
+      <c r="R15" s="146"/>
+      <c r="S15" s="147"/>
+      <c r="T15" s="147"/>
+      <c r="U15" s="145"/>
+      <c r="V15" s="105"/>
+      <c r="W15" s="145"/>
+    </row>
+    <row r="16" spans="1:23" s="149" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="108" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="164" t="s">
+      <c r="B16" s="153" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="164"/>
-      <c r="D16" s="164"/>
-      <c r="E16" s="156"/>
-      <c r="F16" s="109"/>
-      <c r="G16" s="156"/>
-      <c r="H16" s="109"/>
-      <c r="I16" s="159"/>
-      <c r="J16" s="109"/>
-      <c r="K16" s="159"/>
-      <c r="L16" s="109"/>
-      <c r="M16" s="156"/>
-      <c r="N16" s="109"/>
-      <c r="O16" s="156"/>
-      <c r="P16" s="157"/>
-      <c r="Q16" s="156"/>
-      <c r="R16" s="157"/>
-      <c r="S16" s="158"/>
-      <c r="T16" s="158"/>
-      <c r="U16" s="156"/>
-      <c r="V16" s="109"/>
-      <c r="W16" s="156"/>
-    </row>
-    <row r="17" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="112" t="s">
+      <c r="C16" s="153"/>
+      <c r="D16" s="153"/>
+      <c r="E16" s="145"/>
+      <c r="F16" s="105"/>
+      <c r="G16" s="145"/>
+      <c r="H16" s="105"/>
+      <c r="I16" s="148"/>
+      <c r="J16" s="105"/>
+      <c r="K16" s="148"/>
+      <c r="L16" s="105"/>
+      <c r="M16" s="145"/>
+      <c r="N16" s="105"/>
+      <c r="O16" s="145"/>
+      <c r="P16" s="146"/>
+      <c r="Q16" s="145"/>
+      <c r="R16" s="146"/>
+      <c r="S16" s="147"/>
+      <c r="T16" s="147"/>
+      <c r="U16" s="145"/>
+      <c r="V16" s="105"/>
+      <c r="W16" s="145"/>
+    </row>
+    <row r="17" spans="1:23" s="149" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="108" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="164" t="s">
+      <c r="B17" s="153" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="164"/>
-      <c r="D17" s="164"/>
-      <c r="E17" s="156"/>
-      <c r="F17" s="109"/>
-      <c r="G17" s="156"/>
-      <c r="H17" s="109"/>
-      <c r="I17" s="159"/>
-      <c r="J17" s="109"/>
-      <c r="K17" s="156"/>
-      <c r="L17" s="109"/>
-      <c r="M17" s="156"/>
-      <c r="N17" s="109"/>
-      <c r="O17" s="156"/>
-      <c r="P17" s="157"/>
-      <c r="Q17" s="156"/>
-      <c r="R17" s="157"/>
-      <c r="S17" s="158"/>
-      <c r="T17" s="158"/>
-      <c r="U17" s="156"/>
-      <c r="V17" s="109"/>
-      <c r="W17" s="156"/>
-    </row>
-    <row r="18" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="112" t="s">
+      <c r="C17" s="153"/>
+      <c r="D17" s="153"/>
+      <c r="E17" s="145"/>
+      <c r="F17" s="105"/>
+      <c r="G17" s="145"/>
+      <c r="H17" s="105"/>
+      <c r="I17" s="148"/>
+      <c r="J17" s="105"/>
+      <c r="K17" s="145"/>
+      <c r="L17" s="105"/>
+      <c r="M17" s="145"/>
+      <c r="N17" s="105"/>
+      <c r="O17" s="145"/>
+      <c r="P17" s="146"/>
+      <c r="Q17" s="145"/>
+      <c r="R17" s="146"/>
+      <c r="S17" s="147"/>
+      <c r="T17" s="147"/>
+      <c r="U17" s="145"/>
+      <c r="V17" s="105"/>
+      <c r="W17" s="145"/>
+    </row>
+    <row r="18" spans="1:23" s="149" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="109">
+      <c r="B18" s="105">
         <f>SUM(B9:B17)</f>
         <v>0</v>
       </c>
-      <c r="C18" s="109">
+      <c r="C18" s="105">
         <f t="shared" ref="C18:O18" si="0">SUM(C9:C17)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="109">
+      <c r="D18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E18" s="109">
+      <c r="E18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="109">
+      <c r="F18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G18" s="109">
+      <c r="G18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="109">
+      <c r="H18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I18" s="109">
+      <c r="I18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="109">
+      <c r="J18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K18" s="109">
+      <c r="K18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L18" s="109">
+      <c r="L18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M18" s="109">
+      <c r="M18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N18" s="109">
+      <c r="N18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O18" s="109">
+      <c r="O18" s="105">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P18" s="109">
+      <c r="P18" s="105">
         <f t="shared" ref="P18" si="1">SUM(P9:P17)</f>
         <v>0</v>
       </c>
-      <c r="Q18" s="109">
+      <c r="Q18" s="105">
         <f>SUM(Q9:Q17)</f>
         <v>0</v>
       </c>
-      <c r="R18" s="109">
+      <c r="R18" s="105">
         <f>SUM(R9:R17)</f>
         <v>0</v>
       </c>
-      <c r="S18" s="115">
+      <c r="S18" s="111">
         <f>SUM(S9:S17)</f>
         <v>0</v>
       </c>
-      <c r="T18" s="115">
+      <c r="T18" s="111">
         <f>SUM(T9:T17)</f>
         <v>0</v>
       </c>
-      <c r="U18" s="109">
+      <c r="U18" s="105">
         <f t="shared" ref="U18:W18" si="2">SUM(U9:U17)</f>
         <v>0</v>
       </c>
-      <c r="V18" s="109">
+      <c r="V18" s="105">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="W18" s="109">
+      <c r="W18" s="105">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="112"/>
-      <c r="B19" s="109"/>
-      <c r="C19" s="109"/>
-      <c r="D19" s="109"/>
-      <c r="E19" s="109"/>
-      <c r="F19" s="156"/>
-      <c r="G19" s="109"/>
-      <c r="H19" s="109"/>
-      <c r="I19" s="109"/>
-      <c r="J19" s="109"/>
-      <c r="K19" s="109"/>
-      <c r="L19" s="109"/>
-      <c r="M19" s="109"/>
-      <c r="N19" s="109"/>
-      <c r="O19" s="109"/>
-      <c r="P19" s="109"/>
-      <c r="Q19" s="109"/>
-      <c r="R19" s="109"/>
-      <c r="S19" s="115"/>
-      <c r="T19" s="115"/>
-      <c r="U19" s="109"/>
-      <c r="V19" s="109"/>
-      <c r="W19" s="109"/>
-    </row>
-    <row r="20" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="112" t="s">
+    <row r="19" spans="1:23" s="149" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="108"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="105"/>
+      <c r="F19" s="145"/>
+      <c r="G19" s="105"/>
+      <c r="H19" s="105"/>
+      <c r="I19" s="105"/>
+      <c r="J19" s="105"/>
+      <c r="K19" s="105"/>
+      <c r="L19" s="105"/>
+      <c r="M19" s="105"/>
+      <c r="N19" s="105"/>
+      <c r="O19" s="105"/>
+      <c r="P19" s="105"/>
+      <c r="Q19" s="105"/>
+      <c r="R19" s="105"/>
+      <c r="S19" s="111"/>
+      <c r="T19" s="111"/>
+      <c r="U19" s="105"/>
+      <c r="V19" s="105"/>
+      <c r="W19" s="105"/>
+    </row>
+    <row r="20" spans="1:23" s="150" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="108" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="109" t="e">
+      <c r="B20" s="105" t="e">
         <f t="shared" ref="B20:O20" si="3">B18-B7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C20" s="109">
+      <c r="C20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="D20" s="109">
+      <c r="D20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="E20" s="109">
+      <c r="E20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F20" s="109">
+      <c r="F20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G20" s="109">
+      <c r="G20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H20" s="109">
+      <c r="H20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I20" s="109">
+      <c r="I20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J20" s="109">
+      <c r="J20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K20" s="109">
+      <c r="K20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L20" s="109">
+      <c r="L20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M20" s="109">
+      <c r="M20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="N20" s="109">
+      <c r="N20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="O20" s="109">
+      <c r="O20" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P20" s="109">
+      <c r="P20" s="105">
         <f t="shared" ref="P20" si="4">P18-P7</f>
         <v>0</v>
       </c>
-      <c r="Q20" s="109">
+      <c r="Q20" s="105">
         <f>Q18-Q7</f>
         <v>0</v>
       </c>
-      <c r="R20" s="109">
+      <c r="R20" s="105">
         <f>R18-R7</f>
         <v>0</v>
       </c>
-      <c r="S20" s="109">
+      <c r="S20" s="105">
         <f>S18-S7</f>
         <v>0</v>
       </c>
-      <c r="T20" s="109">
+      <c r="T20" s="105">
         <f>T18-T7</f>
         <v>0</v>
       </c>
-      <c r="U20" s="109">
+      <c r="U20" s="105">
         <f t="shared" ref="U20:W20" si="5">U18-U7</f>
         <v>0</v>
       </c>
-      <c r="V20" s="109">
+      <c r="V20" s="105">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="W20" s="109">
+      <c r="W20" s="105">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2698,17 +2655,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="197" t="s">
+      <c r="M22" s="166" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="197"/>
-      <c r="O22" s="197"/>
-      <c r="P22" s="197"/>
-      <c r="Q22" s="197"/>
-      <c r="R22" s="197"/>
-      <c r="S22" s="197"/>
-      <c r="T22" s="197"/>
-      <c r="U22" s="197"/>
+      <c r="N22" s="166"/>
+      <c r="O22" s="166"/>
+      <c r="P22" s="166"/>
+      <c r="Q22" s="166"/>
+      <c r="R22" s="166"/>
+      <c r="S22" s="166"/>
+      <c r="T22" s="166"/>
+      <c r="U22" s="166"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2717,21 +2674,21 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="206" t="s">
+      <c r="N23" s="173" t="s">
         <v>63</v>
       </c>
-      <c r="O23" s="207"/>
-      <c r="P23" s="207"/>
-      <c r="Q23" s="207"/>
-      <c r="R23" s="207"/>
-      <c r="S23" s="208"/>
-      <c r="T23" s="118" t="s">
+      <c r="O23" s="174"/>
+      <c r="P23" s="174"/>
+      <c r="Q23" s="174"/>
+      <c r="R23" s="174"/>
+      <c r="S23" s="175"/>
+      <c r="T23" s="114" t="s">
         <v>38</v>
       </c>
-      <c r="U23" s="105" t="s">
+      <c r="U23" s="101" t="s">
         <v>75</v>
       </c>
-      <c r="W23" s="90" t="s">
+      <c r="W23" s="86" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2742,50 +2699,50 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="209" t="s">
+      <c r="N24" s="176" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="210"/>
-      <c r="P24" s="210"/>
-      <c r="Q24" s="210"/>
-      <c r="R24" s="210"/>
-      <c r="S24" s="211"/>
-      <c r="T24" s="107" t="s">
+      <c r="O24" s="177"/>
+      <c r="P24" s="177"/>
+      <c r="Q24" s="177"/>
+      <c r="R24" s="177"/>
+      <c r="S24" s="178"/>
+      <c r="T24" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="U24" s="106" t="s">
+      <c r="U24" s="102" t="s">
         <v>76</v>
       </c>
-      <c r="W24" s="117" t="s">
+      <c r="W24" s="113" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B25" s="2"/>
-      <c r="C25" s="102"/>
+      <c r="C25" s="98"/>
       <c r="D25" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="214" t="s">
+      <c r="M25" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="215"/>
-      <c r="O25" s="147"/>
-      <c r="P25" s="148"/>
-      <c r="Q25" s="144" t="s">
+      <c r="N25" s="155"/>
+      <c r="O25" s="156"/>
+      <c r="P25" s="165"/>
+      <c r="Q25" s="135" t="s">
         <v>94</v>
       </c>
-      <c r="R25" s="145"/>
-      <c r="S25" s="146"/>
-      <c r="T25" s="212" t="s">
+      <c r="R25" s="136"/>
+      <c r="S25" s="137"/>
+      <c r="T25" s="179" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="213"/>
+      <c r="U25" s="180"/>
       <c r="V25" s="13"/>
-      <c r="W25" s="81" t="s">
+      <c r="W25" s="77" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2793,137 +2750,137 @@
       <c r="E26" s="4"/>
       <c r="J26"/>
       <c r="L26"/>
-      <c r="M26" s="78" t="s">
+      <c r="M26" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="N26" s="79"/>
-      <c r="O26" s="125"/>
-      <c r="P26" s="126"/>
-      <c r="Q26" s="187" t="s">
+      <c r="N26" s="75"/>
+      <c r="O26" s="156"/>
+      <c r="P26" s="165"/>
+      <c r="Q26" s="158" t="s">
         <v>95</v>
       </c>
-      <c r="R26" s="188"/>
-      <c r="S26" s="189"/>
-      <c r="T26" s="123"/>
-      <c r="U26" s="124"/>
+      <c r="R26" s="159"/>
+      <c r="S26" s="160"/>
+      <c r="T26" s="119"/>
+      <c r="U26" s="120"/>
       <c r="V26" s="13"/>
-      <c r="W26" s="81"/>
+      <c r="W26" s="77"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="I27" s="108" t="str">
+      <c r="I27" s="104" t="str">
         <f>B$1</f>
         <v>{{extraction._meta.bitacora.excel.conductor}}</v>
       </c>
-      <c r="J27" s="135" t="str">
+      <c r="J27" s="127" t="str">
         <f>B9</f>
         <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
       <c r="L27"/>
-      <c r="M27" s="78" t="s">
+      <c r="M27" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="N27" s="79"/>
-      <c r="O27" s="185"/>
-      <c r="P27" s="186"/>
-      <c r="Q27" s="187" t="s">
+      <c r="N27" s="75"/>
+      <c r="O27" s="156"/>
+      <c r="P27" s="165"/>
+      <c r="Q27" s="158" t="s">
         <v>64</v>
       </c>
-      <c r="R27" s="188"/>
-      <c r="S27" s="189"/>
-      <c r="T27" s="204" t="s">
+      <c r="R27" s="159"/>
+      <c r="S27" s="160"/>
+      <c r="T27" s="171" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="205"/>
+      <c r="U27" s="172"/>
       <c r="V27" s="19"/>
-      <c r="W27" s="91" t="s">
+      <c r="W27" s="87" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="I28" s="108">
+      <c r="I28" s="104">
         <f>C$1</f>
         <v>0</v>
       </c>
-      <c r="J28" s="135">
+      <c r="J28" s="127">
         <f>C9</f>
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="202" t="s">
+      <c r="M28" s="163" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="203"/>
-      <c r="O28" s="185"/>
-      <c r="P28" s="186"/>
-      <c r="Q28" s="187" t="s">
+      <c r="N28" s="164"/>
+      <c r="O28" s="156"/>
+      <c r="P28" s="165"/>
+      <c r="Q28" s="158" t="s">
         <v>65</v>
       </c>
-      <c r="R28" s="188"/>
-      <c r="S28" s="189"/>
-      <c r="T28" s="200" t="s">
+      <c r="R28" s="159"/>
+      <c r="S28" s="160"/>
+      <c r="T28" s="169" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="201"/>
+      <c r="U28" s="170"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="I29" s="108">
+      <c r="I29" s="104">
         <f>D$1</f>
         <v>0</v>
       </c>
-      <c r="J29" s="135">
+      <c r="J29" s="127">
         <f>D9</f>
         <v>0</v>
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="202" t="s">
+      <c r="M29" s="163" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="203"/>
-      <c r="O29" s="185"/>
-      <c r="P29" s="186"/>
-      <c r="Q29" s="187" t="s">
+      <c r="N29" s="164"/>
+      <c r="O29" s="156"/>
+      <c r="P29" s="165"/>
+      <c r="Q29" s="158" t="s">
         <v>66</v>
       </c>
-      <c r="R29" s="188"/>
-      <c r="S29" s="189"/>
-      <c r="T29" s="198" t="s">
+      <c r="R29" s="159"/>
+      <c r="S29" s="160"/>
+      <c r="T29" s="167" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="199"/>
-      <c r="W29" s="92" t="str">
+      <c r="U29" s="168"/>
+      <c r="W29" s="88" t="str">
         <f>U23</f>
         <v>{{extraction.cant_fact.valor}}</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="I30" s="108">
+      <c r="I30" s="104">
         <f>E$1</f>
         <v>0</v>
       </c>
-      <c r="J30" s="135">
+      <c r="J30" s="127">
         <f>E9</f>
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="202" t="s">
+      <c r="M30" s="163" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="203"/>
-      <c r="O30" s="185"/>
-      <c r="P30" s="216"/>
-      <c r="Q30" s="187" t="s">
+      <c r="N30" s="164"/>
+      <c r="O30" s="156"/>
+      <c r="P30" s="157"/>
+      <c r="Q30" s="158" t="s">
         <v>67</v>
       </c>
-      <c r="R30" s="188"/>
-      <c r="S30" s="189"/>
-      <c r="T30" s="217" t="s">
+      <c r="R30" s="159"/>
+      <c r="S30" s="160"/>
+      <c r="T30" s="161" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="218"/>
+      <c r="U30" s="162"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2932,108 +2889,108 @@
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="I31" s="108">
+      <c r="I31" s="104">
         <f>F$1</f>
         <v>0</v>
       </c>
-      <c r="J31" s="135">
+      <c r="J31" s="127">
         <f>F9</f>
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="202" t="s">
+      <c r="M31" s="163" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="203"/>
-      <c r="O31" s="185"/>
-      <c r="P31" s="186"/>
-      <c r="Q31" s="187" t="s">
+      <c r="N31" s="164"/>
+      <c r="O31" s="156"/>
+      <c r="P31" s="165"/>
+      <c r="Q31" s="158" t="s">
         <v>68</v>
       </c>
-      <c r="R31" s="188"/>
-      <c r="S31" s="189"/>
+      <c r="R31" s="159"/>
+      <c r="S31" s="160"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="I32" s="108">
+      <c r="I32" s="104">
         <f>G$1</f>
         <v>0</v>
       </c>
-      <c r="J32" s="135">
+      <c r="J32" s="127">
         <f>G9</f>
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="202" t="s">
+      <c r="M32" s="163" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="203"/>
-      <c r="O32" s="185"/>
-      <c r="P32" s="186"/>
-      <c r="Q32" s="187" t="s">
+      <c r="N32" s="164"/>
+      <c r="O32" s="156"/>
+      <c r="P32" s="165"/>
+      <c r="Q32" s="158" t="s">
         <v>69</v>
       </c>
-      <c r="R32" s="188"/>
-      <c r="S32" s="189"/>
+      <c r="R32" s="159"/>
+      <c r="S32" s="160"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
-      <c r="W32" s="81" t="s">
+      <c r="W32" s="77" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="I33" s="108">
+      <c r="I33" s="104">
         <f>H$1</f>
         <v>0</v>
       </c>
-      <c r="J33" s="135">
+      <c r="J33" s="127">
         <f>H9</f>
         <v>0</v>
       </c>
       <c r="L33"/>
-      <c r="M33" s="78" t="s">
+      <c r="M33" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="N33" s="80"/>
-      <c r="O33" s="185"/>
-      <c r="P33" s="186"/>
-      <c r="Q33" s="187" t="s">
+      <c r="N33" s="76"/>
+      <c r="O33" s="156"/>
+      <c r="P33" s="165"/>
+      <c r="Q33" s="158" t="s">
         <v>70</v>
       </c>
-      <c r="R33" s="188"/>
-      <c r="S33" s="189"/>
+      <c r="R33" s="159"/>
+      <c r="S33" s="160"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
-      <c r="W33" s="116" t="e">
+      <c r="W33" s="112" t="e">
         <f>W30-W27</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="34" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
-      <c r="I34" s="108">
+      <c r="I34" s="104">
         <f>I$1</f>
         <v>0</v>
       </c>
-      <c r="J34" s="135">
+      <c r="J34" s="127">
         <f>I9</f>
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="190" t="s">
+      <c r="M34" s="184" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="191"/>
-      <c r="O34" s="192"/>
-      <c r="P34" s="193"/>
-      <c r="Q34" s="187" t="s">
+      <c r="N34" s="185"/>
+      <c r="O34" s="186"/>
+      <c r="P34" s="187"/>
+      <c r="Q34" s="158" t="s">
         <v>71</v>
       </c>
-      <c r="R34" s="188"/>
-      <c r="S34" s="189"/>
+      <c r="R34" s="159"/>
+      <c r="S34" s="160"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3042,7 +2999,7 @@
     <row r="35" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="D35" s="31"/>
-      <c r="I35" s="108">
+      <c r="I35" s="104">
         <f>J$1</f>
         <v>0</v>
       </c>
@@ -3051,29 +3008,29 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="194" t="s">
+      <c r="M35" s="188" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="195"/>
-      <c r="O35" s="196"/>
-      <c r="P35" s="165" t="s">
+      <c r="N35" s="189"/>
+      <c r="O35" s="190"/>
+      <c r="P35" s="182" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="167"/>
-      <c r="R35" s="165" t="s">
+      <c r="Q35" s="183"/>
+      <c r="R35" s="182" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="167"/>
-      <c r="T35" s="165" t="s">
+      <c r="S35" s="183"/>
+      <c r="T35" s="182" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="167"/>
+      <c r="U35" s="183"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
     <row r="36" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="9"/>
-      <c r="I36" s="108">
+      <c r="I36" s="104">
         <f>K$1</f>
         <v>0</v>
       </c>
@@ -3127,22 +3084,22 @@
       <c r="O37" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="P37" s="150" t="s">
+      <c r="P37" s="139" t="s">
         <v>80</v>
       </c>
-      <c r="Q37" s="76" t="s">
+      <c r="Q37" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="R37" s="152" t="s">
+      <c r="R37" s="141" t="s">
         <v>82</v>
       </c>
-      <c r="S37" s="77" t="s">
+      <c r="S37" s="73" t="s">
         <v>83</v>
       </c>
-      <c r="T37" s="151" t="s">
+      <c r="T37" s="140" t="s">
         <v>84</v>
       </c>
-      <c r="U37" s="73" t="s">
+      <c r="U37" s="69" t="s">
         <v>85</v>
       </c>
       <c r="V37" s="1"/>
@@ -3155,20 +3112,20 @@
       <c r="C38" s="32"/>
       <c r="I38" s="13"/>
       <c r="J38" s="52"/>
-      <c r="L38" s="104"/>
-      <c r="M38" s="169" t="s">
+      <c r="L38" s="100"/>
+      <c r="M38" s="191" t="s">
         <v>42</v>
       </c>
-      <c r="N38" s="179"/>
-      <c r="O38" s="149" t="s">
+      <c r="N38" s="192"/>
+      <c r="O38" s="138" t="s">
         <v>64</v>
       </c>
-      <c r="P38" s="151"/>
-      <c r="Q38" s="74"/>
-      <c r="R38" s="153"/>
-      <c r="S38" s="72"/>
-      <c r="T38" s="151"/>
-      <c r="U38" s="75"/>
+      <c r="P38" s="140"/>
+      <c r="Q38" s="70"/>
+      <c r="R38" s="142"/>
+      <c r="S38" s="68"/>
+      <c r="T38" s="140"/>
+      <c r="U38" s="71"/>
       <c r="V38" s="1"/>
       <c r="W38" s="1"/>
     </row>
@@ -3178,7 +3135,7 @@
       <c r="I39" s="13"/>
       <c r="J39" s="52"/>
       <c r="K39" s="24"/>
-      <c r="L39" s="104"/>
+      <c r="L39" s="100"/>
       <c r="M39" s="37" t="s">
         <v>77</v>
       </c>
@@ -3188,12 +3145,12 @@
       <c r="O39" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="P39" s="151"/>
-      <c r="Q39" s="67"/>
-      <c r="R39" s="153"/>
-      <c r="S39" s="72"/>
-      <c r="T39" s="151"/>
-      <c r="U39" s="67"/>
+      <c r="P39" s="140"/>
+      <c r="Q39" s="63"/>
+      <c r="R39" s="142"/>
+      <c r="S39" s="68"/>
+      <c r="T39" s="140"/>
+      <c r="U39" s="63"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1"/>
     </row>
@@ -3205,16 +3162,16 @@
       <c r="I40" s="13"/>
       <c r="J40" s="52"/>
       <c r="K40" s="24"/>
-      <c r="L40" s="104"/>
+      <c r="L40" s="100"/>
       <c r="M40" s="37"/>
       <c r="N40" s="38"/>
       <c r="O40" s="39"/>
-      <c r="P40" s="151"/>
-      <c r="Q40" s="65"/>
-      <c r="R40" s="153"/>
-      <c r="S40" s="73"/>
-      <c r="T40" s="151"/>
-      <c r="U40" s="67"/>
+      <c r="P40" s="140"/>
+      <c r="Q40" s="61"/>
+      <c r="R40" s="142"/>
+      <c r="S40" s="69"/>
+      <c r="T40" s="140"/>
+      <c r="U40" s="63"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1"/>
     </row>
@@ -3226,16 +3183,16 @@
       <c r="I41" s="13"/>
       <c r="J41" s="52"/>
       <c r="K41" s="24"/>
-      <c r="L41" s="104"/>
+      <c r="L41" s="100"/>
       <c r="M41" s="37"/>
       <c r="N41" s="38"/>
       <c r="O41" s="39"/>
-      <c r="P41" s="151"/>
-      <c r="Q41" s="65"/>
-      <c r="R41" s="153"/>
-      <c r="S41" s="73"/>
-      <c r="T41" s="151"/>
-      <c r="U41" s="67"/>
+      <c r="P41" s="140"/>
+      <c r="Q41" s="61"/>
+      <c r="R41" s="142"/>
+      <c r="S41" s="69"/>
+      <c r="T41" s="140"/>
+      <c r="U41" s="63"/>
       <c r="V41" s="1"/>
       <c r="W41" s="1"/>
     </row>
@@ -3247,171 +3204,171 @@
       <c r="F42" s="46"/>
       <c r="I42" s="13"/>
       <c r="J42" s="52"/>
-      <c r="L42" s="104"/>
+      <c r="L42" s="100"/>
       <c r="M42" s="37"/>
       <c r="N42" s="38"/>
       <c r="O42" s="39"/>
-      <c r="P42" s="151"/>
-      <c r="Q42" s="65"/>
-      <c r="R42" s="153"/>
-      <c r="S42" s="72"/>
-      <c r="T42" s="151"/>
-      <c r="U42" s="67"/>
+      <c r="P42" s="140"/>
+      <c r="Q42" s="61"/>
+      <c r="R42" s="142"/>
+      <c r="S42" s="68"/>
+      <c r="T42" s="140"/>
+      <c r="U42" s="63"/>
       <c r="V42" s="1"/>
       <c r="W42" s="1"/>
     </row>
     <row r="43" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A43" s="103"/>
+      <c r="A43" s="99"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="168"/>
-      <c r="E43" s="168"/>
+      <c r="D43" s="181"/>
+      <c r="E43" s="181"/>
       <c r="F43" s="46"/>
       <c r="G43" s="8"/>
       <c r="I43" s="13"/>
       <c r="J43" s="52"/>
       <c r="K43" s="24"/>
-      <c r="L43" s="104"/>
+      <c r="L43" s="100"/>
       <c r="M43" s="37"/>
       <c r="N43" s="38"/>
       <c r="O43" s="39"/>
-      <c r="P43" s="151"/>
-      <c r="Q43" s="65"/>
-      <c r="R43" s="151"/>
-      <c r="S43" s="66"/>
-      <c r="T43" s="151"/>
-      <c r="U43" s="67"/>
+      <c r="P43" s="140"/>
+      <c r="Q43" s="61"/>
+      <c r="R43" s="140"/>
+      <c r="S43" s="62"/>
+      <c r="T43" s="140"/>
+      <c r="U43" s="63"/>
     </row>
     <row r="44" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="168"/>
-      <c r="E44" s="168"/>
+      <c r="D44" s="181"/>
+      <c r="E44" s="181"/>
       <c r="F44" s="47"/>
-      <c r="H44" s="63"/>
+      <c r="H44" s="59"/>
       <c r="I44" s="13"/>
       <c r="J44" s="52"/>
       <c r="K44" s="24"/>
-      <c r="L44" s="104"/>
+      <c r="L44" s="100"/>
       <c r="M44" s="37"/>
       <c r="N44" s="38"/>
       <c r="O44" s="39"/>
-      <c r="P44" s="151"/>
-      <c r="Q44" s="65"/>
-      <c r="R44" s="151"/>
-      <c r="S44" s="66"/>
-      <c r="T44" s="151"/>
-      <c r="U44" s="67"/>
+      <c r="P44" s="140"/>
+      <c r="Q44" s="61"/>
+      <c r="R44" s="140"/>
+      <c r="S44" s="62"/>
+      <c r="T44" s="140"/>
+      <c r="U44" s="63"/>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="40"/>
-      <c r="D45" s="168"/>
-      <c r="E45" s="168"/>
+      <c r="D45" s="181"/>
+      <c r="E45" s="181"/>
       <c r="F45" s="23"/>
-      <c r="H45" s="63"/>
+      <c r="H45" s="59"/>
       <c r="I45" s="13"/>
       <c r="J45" s="52"/>
-      <c r="L45" s="104"/>
+      <c r="L45" s="100"/>
       <c r="M45" s="37"/>
       <c r="N45" s="38"/>
       <c r="O45" s="39"/>
-      <c r="P45" s="151"/>
-      <c r="Q45" s="65"/>
-      <c r="R45" s="151"/>
-      <c r="S45" s="71"/>
-      <c r="T45" s="151"/>
-      <c r="U45" s="67"/>
+      <c r="P45" s="140"/>
+      <c r="Q45" s="61"/>
+      <c r="R45" s="140"/>
+      <c r="S45" s="67"/>
+      <c r="T45" s="140"/>
+      <c r="U45" s="63"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="40"/>
-      <c r="D46" s="168"/>
-      <c r="E46" s="168"/>
+      <c r="D46" s="181"/>
+      <c r="E46" s="181"/>
       <c r="F46" s="48"/>
-      <c r="H46" s="63"/>
+      <c r="H46" s="59"/>
       <c r="I46" s="13"/>
       <c r="J46" s="52"/>
-      <c r="L46" s="104"/>
+      <c r="L46" s="100"/>
       <c r="M46" s="37"/>
       <c r="N46" s="38"/>
       <c r="O46" s="39"/>
-      <c r="P46" s="151"/>
-      <c r="Q46" s="65"/>
-      <c r="R46" s="151"/>
-      <c r="S46" s="66"/>
-      <c r="T46" s="151"/>
-      <c r="U46" s="67"/>
+      <c r="P46" s="140"/>
+      <c r="Q46" s="61"/>
+      <c r="R46" s="140"/>
+      <c r="S46" s="62"/>
+      <c r="T46" s="140"/>
+      <c r="U46" s="63"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="40"/>
-      <c r="D47" s="168"/>
-      <c r="E47" s="168"/>
+      <c r="D47" s="181"/>
+      <c r="E47" s="181"/>
       <c r="F47" s="17"/>
       <c r="G47" s="1"/>
-      <c r="H47" s="63"/>
+      <c r="H47" s="59"/>
       <c r="I47" s="13"/>
       <c r="J47" s="52"/>
       <c r="K47" s="24"/>
-      <c r="L47" s="104"/>
+      <c r="L47" s="100"/>
       <c r="M47" s="37"/>
       <c r="N47" s="38"/>
       <c r="O47" s="39"/>
-      <c r="P47" s="151"/>
-      <c r="Q47" s="65"/>
-      <c r="R47" s="151"/>
-      <c r="S47" s="66"/>
-      <c r="T47" s="151"/>
-      <c r="U47" s="67"/>
+      <c r="P47" s="140"/>
+      <c r="Q47" s="61"/>
+      <c r="R47" s="140"/>
+      <c r="S47" s="62"/>
+      <c r="T47" s="140"/>
+      <c r="U47" s="63"/>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="40"/>
-      <c r="D48" s="168"/>
-      <c r="E48" s="168"/>
+      <c r="D48" s="181"/>
+      <c r="E48" s="181"/>
       <c r="F48" s="23"/>
       <c r="G48" s="1"/>
-      <c r="H48" s="63"/>
+      <c r="H48" s="59"/>
       <c r="I48" s="13"/>
       <c r="J48" s="52"/>
-      <c r="L48" s="104"/>
+      <c r="L48" s="100"/>
       <c r="M48" s="37"/>
       <c r="N48" s="38"/>
       <c r="O48" s="39"/>
-      <c r="P48" s="151"/>
-      <c r="Q48" s="65"/>
-      <c r="R48" s="151"/>
-      <c r="S48" s="66"/>
-      <c r="T48" s="153"/>
-      <c r="U48" s="67"/>
+      <c r="P48" s="140"/>
+      <c r="Q48" s="61"/>
+      <c r="R48" s="140"/>
+      <c r="S48" s="62"/>
+      <c r="T48" s="142"/>
+      <c r="U48" s="63"/>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="40"/>
-      <c r="D49" s="168"/>
-      <c r="E49" s="168"/>
+      <c r="D49" s="181"/>
+      <c r="E49" s="181"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
       <c r="H49" s="45"/>
       <c r="I49" s="13"/>
       <c r="J49" s="52"/>
-      <c r="L49" s="104"/>
+      <c r="L49" s="100"/>
       <c r="M49" s="37"/>
       <c r="N49" s="38"/>
       <c r="O49" s="39"/>
-      <c r="P49" s="151"/>
-      <c r="Q49" s="65"/>
-      <c r="R49" s="151"/>
-      <c r="S49" s="66"/>
-      <c r="T49" s="153"/>
-      <c r="U49" s="67"/>
+      <c r="P49" s="140"/>
+      <c r="Q49" s="61"/>
+      <c r="R49" s="140"/>
+      <c r="S49" s="62"/>
+      <c r="T49" s="142"/>
+      <c r="U49" s="63"/>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A50" s="20"/>
@@ -3424,67 +3381,67 @@
       <c r="H50" s="45"/>
       <c r="I50" s="13"/>
       <c r="J50" s="52"/>
-      <c r="L50" s="104"/>
+      <c r="L50" s="100"/>
       <c r="M50" s="37"/>
       <c r="N50" s="38"/>
       <c r="O50" s="39"/>
-      <c r="P50" s="151"/>
-      <c r="Q50" s="65"/>
-      <c r="R50" s="151"/>
-      <c r="S50" s="66"/>
-      <c r="T50" s="153"/>
-      <c r="U50" s="67"/>
+      <c r="P50" s="140"/>
+      <c r="Q50" s="61"/>
+      <c r="R50" s="140"/>
+      <c r="S50" s="62"/>
+      <c r="T50" s="142"/>
+      <c r="U50" s="63"/>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="40"/>
-      <c r="D51" s="171"/>
-      <c r="E51" s="171"/>
+      <c r="D51" s="206"/>
+      <c r="E51" s="206"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="45"/>
       <c r="I51" s="13"/>
       <c r="J51" s="52"/>
-      <c r="L51" s="104"/>
+      <c r="L51" s="100"/>
       <c r="M51" s="37"/>
       <c r="N51" s="38"/>
       <c r="O51" s="39"/>
-      <c r="P51" s="150"/>
-      <c r="Q51" s="65"/>
-      <c r="R51" s="151"/>
-      <c r="S51" s="66"/>
-      <c r="T51" s="153"/>
-      <c r="U51" s="67"/>
+      <c r="P51" s="139"/>
+      <c r="Q51" s="61"/>
+      <c r="R51" s="140"/>
+      <c r="S51" s="62"/>
+      <c r="T51" s="142"/>
+      <c r="U51" s="63"/>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A52" s="20"/>
       <c r="B52" s="50"/>
       <c r="C52" s="40"/>
-      <c r="D52" s="178"/>
-      <c r="E52" s="178"/>
+      <c r="D52" s="194"/>
+      <c r="E52" s="194"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="45"/>
       <c r="I52" s="49"/>
       <c r="J52" s="52"/>
-      <c r="L52" s="104"/>
+      <c r="L52" s="100"/>
       <c r="M52" s="37"/>
       <c r="N52" s="38"/>
       <c r="O52" s="39"/>
-      <c r="P52" s="150"/>
-      <c r="Q52" s="65"/>
-      <c r="R52" s="151"/>
-      <c r="S52" s="66"/>
-      <c r="T52" s="153"/>
-      <c r="U52" s="67"/>
+      <c r="P52" s="139"/>
+      <c r="Q52" s="61"/>
+      <c r="R52" s="140"/>
+      <c r="S52" s="62"/>
+      <c r="T52" s="142"/>
+      <c r="U52" s="63"/>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A53" s="25"/>
       <c r="B53" s="50"/>
       <c r="C53" s="40"/>
-      <c r="D53" s="177"/>
-      <c r="E53" s="177"/>
+      <c r="D53" s="193"/>
+      <c r="E53" s="193"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="45"/>
@@ -3494,19 +3451,19 @@
       <c r="M53" s="37"/>
       <c r="N53" s="38"/>
       <c r="O53" s="39"/>
-      <c r="P53" s="151"/>
-      <c r="Q53" s="65"/>
-      <c r="R53" s="151"/>
-      <c r="S53" s="66"/>
-      <c r="T53" s="153"/>
-      <c r="U53" s="67"/>
+      <c r="P53" s="140"/>
+      <c r="Q53" s="61"/>
+      <c r="R53" s="140"/>
+      <c r="S53" s="62"/>
+      <c r="T53" s="142"/>
+      <c r="U53" s="63"/>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A54" s="20"/>
       <c r="B54" s="50"/>
       <c r="C54" s="40"/>
-      <c r="D54" s="177"/>
-      <c r="E54" s="177"/>
+      <c r="D54" s="193"/>
+      <c r="E54" s="193"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="45"/>
@@ -3516,12 +3473,12 @@
       <c r="M54" s="37"/>
       <c r="N54" s="38"/>
       <c r="O54" s="39"/>
-      <c r="P54" s="151"/>
-      <c r="Q54" s="65"/>
-      <c r="R54" s="151"/>
-      <c r="S54" s="66"/>
-      <c r="T54" s="153"/>
-      <c r="U54" s="67"/>
+      <c r="P54" s="140"/>
+      <c r="Q54" s="61"/>
+      <c r="R54" s="140"/>
+      <c r="S54" s="62"/>
+      <c r="T54" s="142"/>
+      <c r="U54" s="63"/>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A55" s="20"/>
@@ -3538,12 +3495,12 @@
       <c r="M55" s="37"/>
       <c r="N55" s="38"/>
       <c r="O55" s="39"/>
-      <c r="P55" s="151"/>
-      <c r="Q55" s="65"/>
-      <c r="R55" s="151"/>
-      <c r="S55" s="66"/>
-      <c r="T55" s="153"/>
-      <c r="U55" s="67"/>
+      <c r="P55" s="140"/>
+      <c r="Q55" s="61"/>
+      <c r="R55" s="140"/>
+      <c r="S55" s="62"/>
+      <c r="T55" s="142"/>
+      <c r="U55" s="63"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A56" s="20"/>
@@ -3560,12 +3517,12 @@
       <c r="M56" s="37"/>
       <c r="N56" s="38"/>
       <c r="O56" s="39"/>
-      <c r="P56" s="151"/>
-      <c r="Q56" s="65"/>
-      <c r="R56" s="151"/>
-      <c r="S56" s="66"/>
-      <c r="T56" s="153"/>
-      <c r="U56" s="67"/>
+      <c r="P56" s="140"/>
+      <c r="Q56" s="61"/>
+      <c r="R56" s="140"/>
+      <c r="S56" s="62"/>
+      <c r="T56" s="142"/>
+      <c r="U56" s="63"/>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A57" s="20"/>
@@ -3582,12 +3539,12 @@
       <c r="M57" s="37"/>
       <c r="N57" s="38"/>
       <c r="O57" s="39"/>
-      <c r="P57" s="151"/>
-      <c r="Q57" s="65"/>
-      <c r="R57" s="151"/>
-      <c r="S57" s="66"/>
-      <c r="T57" s="153"/>
-      <c r="U57" s="67"/>
+      <c r="P57" s="140"/>
+      <c r="Q57" s="61"/>
+      <c r="R57" s="140"/>
+      <c r="S57" s="62"/>
+      <c r="T57" s="142"/>
+      <c r="U57" s="63"/>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A58" s="20"/>
@@ -3604,12 +3561,12 @@
       <c r="M58" s="37"/>
       <c r="N58" s="38"/>
       <c r="O58" s="39"/>
-      <c r="P58" s="151"/>
-      <c r="Q58" s="65"/>
-      <c r="R58" s="151"/>
-      <c r="S58" s="66"/>
-      <c r="T58" s="153"/>
-      <c r="U58" s="67"/>
+      <c r="P58" s="140"/>
+      <c r="Q58" s="61"/>
+      <c r="R58" s="140"/>
+      <c r="S58" s="62"/>
+      <c r="T58" s="142"/>
+      <c r="U58" s="63"/>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A59" s="20"/>
@@ -3626,19 +3583,19 @@
       <c r="M59" s="37"/>
       <c r="N59" s="38"/>
       <c r="O59" s="39"/>
-      <c r="P59" s="151"/>
-      <c r="Q59" s="65"/>
-      <c r="R59" s="151"/>
-      <c r="S59" s="66"/>
-      <c r="T59" s="153"/>
-      <c r="U59" s="67"/>
+      <c r="P59" s="140"/>
+      <c r="Q59" s="61"/>
+      <c r="R59" s="140"/>
+      <c r="S59" s="62"/>
+      <c r="T59" s="142"/>
+      <c r="U59" s="63"/>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="40"/>
-      <c r="D60" s="177"/>
-      <c r="E60" s="177"/>
+      <c r="D60" s="193"/>
+      <c r="E60" s="193"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="45"/>
@@ -3648,12 +3605,12 @@
       <c r="M60" s="37"/>
       <c r="N60" s="38"/>
       <c r="O60" s="39"/>
-      <c r="P60" s="151"/>
-      <c r="Q60" s="65"/>
-      <c r="R60" s="151"/>
-      <c r="S60" s="66"/>
-      <c r="T60" s="153"/>
-      <c r="U60" s="67"/>
+      <c r="P60" s="140"/>
+      <c r="Q60" s="61"/>
+      <c r="R60" s="140"/>
+      <c r="S60" s="62"/>
+      <c r="T60" s="142"/>
+      <c r="U60" s="63"/>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A61" s="25"/>
@@ -3670,12 +3627,12 @@
       <c r="M61" s="37"/>
       <c r="N61" s="38"/>
       <c r="O61" s="39"/>
-      <c r="P61" s="151"/>
-      <c r="Q61" s="134"/>
-      <c r="R61" s="154"/>
-      <c r="S61" s="87"/>
-      <c r="T61" s="153"/>
-      <c r="U61" s="67"/>
+      <c r="P61" s="140"/>
+      <c r="Q61" s="126"/>
+      <c r="R61" s="143"/>
+      <c r="S61" s="83"/>
+      <c r="T61" s="142"/>
+      <c r="U61" s="63"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A62" s="25"/>
@@ -3692,12 +3649,12 @@
       <c r="M62" s="37"/>
       <c r="N62" s="38"/>
       <c r="O62" s="39"/>
-      <c r="P62" s="151"/>
-      <c r="Q62" s="134"/>
-      <c r="R62" s="154"/>
-      <c r="S62" s="87"/>
-      <c r="T62" s="153"/>
-      <c r="U62" s="67"/>
+      <c r="P62" s="140"/>
+      <c r="Q62" s="126"/>
+      <c r="R62" s="143"/>
+      <c r="S62" s="83"/>
+      <c r="T62" s="142"/>
+      <c r="U62" s="63"/>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A63" s="25"/>
@@ -3714,19 +3671,19 @@
       <c r="M63" s="37"/>
       <c r="N63" s="38"/>
       <c r="O63" s="39"/>
-      <c r="P63" s="151"/>
-      <c r="Q63" s="134"/>
-      <c r="R63" s="154"/>
-      <c r="S63" s="87"/>
-      <c r="T63" s="153"/>
-      <c r="U63" s="67"/>
+      <c r="P63" s="140"/>
+      <c r="Q63" s="126"/>
+      <c r="R63" s="143"/>
+      <c r="S63" s="83"/>
+      <c r="T63" s="142"/>
+      <c r="U63" s="63"/>
     </row>
     <row r="64" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="40"/>
-      <c r="D64" s="177"/>
-      <c r="E64" s="177"/>
+      <c r="D64" s="193"/>
+      <c r="E64" s="193"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="45"/>
@@ -3736,29 +3693,29 @@
       <c r="M64" s="37"/>
       <c r="N64" s="38"/>
       <c r="O64" s="39"/>
-      <c r="P64" s="151"/>
-      <c r="Q64" s="83"/>
-      <c r="R64" s="154"/>
-      <c r="S64" s="87"/>
-      <c r="T64" s="153"/>
-      <c r="U64" s="70"/>
+      <c r="P64" s="140"/>
+      <c r="Q64" s="79"/>
+      <c r="R64" s="143"/>
+      <c r="S64" s="83"/>
+      <c r="T64" s="142"/>
+      <c r="U64" s="66"/>
     </row>
     <row r="65" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="40"/>
-      <c r="D65" s="177"/>
-      <c r="E65" s="177"/>
+      <c r="D65" s="193"/>
+      <c r="E65" s="193"/>
       <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="45"/>
       <c r="I65" s="49"/>
       <c r="J65" s="52"/>
       <c r="L65"/>
-      <c r="M65" s="169" t="s">
+      <c r="M65" s="191" t="s">
         <v>34</v>
       </c>
-      <c r="N65" s="170"/>
+      <c r="N65" s="205"/>
       <c r="O65" s="41" t="s">
         <v>65</v>
       </c>
@@ -3784,9 +3741,9 @@
     <row r="66" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="25"/>
       <c r="B66"/>
-      <c r="C66" s="89"/>
-      <c r="D66" s="177"/>
-      <c r="E66" s="177"/>
+      <c r="C66" s="85"/>
+      <c r="D66" s="193"/>
+      <c r="E66" s="193"/>
       <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="45"/>
@@ -3795,11 +3752,11 @@
       <c r="L66"/>
       <c r="M66" s="53"/>
       <c r="N66" s="54"/>
-      <c r="O66" s="69"/>
+      <c r="O66" s="65"/>
       <c r="P66" s="23"/>
-      <c r="Q66" s="68"/>
-      <c r="R66" s="69"/>
-      <c r="S66" s="69"/>
+      <c r="Q66" s="64"/>
+      <c r="R66" s="65"/>
+      <c r="S66" s="65"/>
       <c r="T66" s="6"/>
     </row>
     <row r="67" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -3814,38 +3771,38 @@
       <c r="I67" s="49"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="165" t="s">
+      <c r="M67" s="182" t="s">
         <v>47</v>
       </c>
-      <c r="N67" s="166"/>
-      <c r="O67" s="167"/>
-      <c r="P67" s="181"/>
-      <c r="Q67" s="182"/>
-      <c r="R67" s="165" t="s">
+      <c r="N67" s="196"/>
+      <c r="O67" s="183"/>
+      <c r="P67" s="197"/>
+      <c r="Q67" s="198"/>
+      <c r="R67" s="182" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="166"/>
-      <c r="T67" s="183" t="str">
+      <c r="S67" s="196"/>
+      <c r="T67" s="199" t="str">
         <f>Q25</f>
         <v>{{extraction.rendicion.detalles_cheques.total_billetes.valor}}</v>
       </c>
-      <c r="U67" s="184"/>
+      <c r="U67" s="200"/>
     </row>
     <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="177"/>
-      <c r="E68" s="177"/>
-      <c r="F68" s="62"/>
+      <c r="D68" s="193"/>
+      <c r="E68" s="193"/>
+      <c r="F68" s="58"/>
       <c r="G68" s="1"/>
       <c r="H68" s="45"/>
       <c r="I68" s="49"/>
       <c r="J68"/>
       <c r="L68"/>
       <c r="M68" s="55"/>
-      <c r="N68" s="82"/>
-      <c r="O68" s="82"/>
+      <c r="N68" s="78"/>
+      <c r="O68" s="78"/>
       <c r="P68" s="56"/>
       <c r="Q68" s="57"/>
       <c r="R68" s="57"/>
@@ -3855,36 +3812,36 @@
     </row>
     <row r="69" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="25"/>
-      <c r="B69" s="89"/>
+      <c r="B69" s="85"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="177"/>
-      <c r="E69" s="177"/>
-      <c r="F69" s="62"/>
+      <c r="D69" s="193"/>
+      <c r="E69" s="193"/>
+      <c r="F69" s="58"/>
       <c r="G69" s="1"/>
       <c r="H69" s="45"/>
       <c r="I69" s="49"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="169" t="s">
+      <c r="M69" s="191" t="s">
         <v>35</v>
       </c>
-      <c r="N69" s="179"/>
-      <c r="O69" s="179"/>
-      <c r="P69" s="179"/>
-      <c r="Q69" s="179"/>
-      <c r="R69" s="179"/>
-      <c r="S69" s="179"/>
-      <c r="T69" s="179"/>
-      <c r="U69" s="180"/>
+      <c r="N69" s="192"/>
+      <c r="O69" s="192"/>
+      <c r="P69" s="192"/>
+      <c r="Q69" s="192"/>
+      <c r="R69" s="192"/>
+      <c r="S69" s="192"/>
+      <c r="T69" s="192"/>
+      <c r="U69" s="195"/>
       <c r="V69" s="50"/>
     </row>
     <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
       <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="177"/>
-      <c r="E70" s="177"/>
-      <c r="F70" s="62"/>
+      <c r="D70" s="193"/>
+      <c r="E70" s="193"/>
+      <c r="F70" s="58"/>
       <c r="G70" s="1"/>
       <c r="H70" s="45"/>
       <c r="I70" s="49"/>
@@ -3892,37 +3849,37 @@
       <c r="L70" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="M70" s="129" t="s">
+      <c r="M70" s="123" t="s">
         <v>55</v>
       </c>
-      <c r="N70" s="130"/>
-      <c r="O70" s="130"/>
-      <c r="P70" s="130" t="s">
+      <c r="N70" s="124"/>
+      <c r="O70" s="124"/>
+      <c r="P70" s="124" t="s">
         <v>56</v>
       </c>
-      <c r="Q70" s="130"/>
-      <c r="R70" s="130"/>
-      <c r="S70" s="130"/>
-      <c r="T70" s="130" t="s">
+      <c r="Q70" s="124"/>
+      <c r="R70" s="124"/>
+      <c r="S70" s="124"/>
+      <c r="T70" s="124" t="s">
         <v>57</v>
       </c>
-      <c r="U70" s="131" t="s">
+      <c r="U70" s="125" t="s">
         <v>60</v>
       </c>
-      <c r="V70" s="143" t="s">
+      <c r="V70" s="134" t="s">
         <v>58</v>
       </c>
-      <c r="W70" s="143" t="s">
+      <c r="W70" s="134" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="25"/>
-      <c r="B71" s="114"/>
+      <c r="B71" s="110"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="177"/>
-      <c r="E71" s="177"/>
-      <c r="F71" s="62"/>
+      <c r="D71" s="193"/>
+      <c r="E71" s="193"/>
+      <c r="F71" s="58"/>
       <c r="G71" s="1"/>
       <c r="H71" s="45"/>
       <c r="I71" s="49"/>
@@ -3930,154 +3887,154 @@
       <c r="L71" t="s">
         <v>107</v>
       </c>
-      <c r="M71" s="58" t="s">
+      <c r="M71" s="80" t="s">
         <v>86</v>
       </c>
-      <c r="N71" s="59"/>
-      <c r="O71" s="142" t="s">
+      <c r="N71" s="81"/>
+      <c r="O71" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="P71" s="61" t="s">
+      <c r="P71" s="82" t="s">
         <v>87</v>
       </c>
-      <c r="Q71" s="60"/>
-      <c r="R71" s="176" t="s">
+      <c r="Q71" s="55"/>
+      <c r="R71" s="203" t="s">
         <v>6</v>
       </c>
-      <c r="S71" s="176"/>
-      <c r="T71" s="132" t="s">
+      <c r="S71" s="203"/>
+      <c r="T71" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="U71" s="133"/>
+      <c r="U71" s="90"/>
       <c r="V71" s="50" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B72" s="50"/>
-      <c r="C72" s="88"/>
-      <c r="D72" s="177"/>
-      <c r="E72" s="177"/>
-      <c r="F72" s="62"/>
-      <c r="I72" s="114"/>
+      <c r="C72" s="84"/>
+      <c r="D72" s="193"/>
+      <c r="E72" s="193"/>
+      <c r="F72" s="58"/>
+      <c r="I72" s="110"/>
       <c r="L72"/>
-      <c r="M72" s="84"/>
-      <c r="N72" s="85"/>
+      <c r="M72" s="80"/>
+      <c r="N72" s="81"/>
       <c r="O72" s="18"/>
-      <c r="P72" s="86"/>
+      <c r="P72" s="82"/>
       <c r="Q72" s="55"/>
-      <c r="R72" s="174"/>
-      <c r="S72" s="174"/>
-      <c r="T72" s="64"/>
-      <c r="U72" s="94"/>
+      <c r="R72" s="203"/>
+      <c r="S72" s="203"/>
+      <c r="T72" s="60"/>
+      <c r="U72" s="90"/>
       <c r="V72" s="50"/>
     </row>
     <row r="73" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="48"/>
-      <c r="B73" s="88"/>
-      <c r="C73" s="88"/>
+      <c r="B73" s="84"/>
+      <c r="C73" s="84"/>
       <c r="D73" s="23"/>
       <c r="E73" s="25"/>
-      <c r="F73" s="62"/>
-      <c r="I73" s="114"/>
+      <c r="F73" s="58"/>
+      <c r="I73" s="110"/>
       <c r="L73" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="M73" s="84" t="s">
+      <c r="M73" s="80" t="s">
         <v>91</v>
       </c>
-      <c r="N73" s="85"/>
+      <c r="N73" s="81"/>
       <c r="O73" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="P73" s="86" t="s">
+      <c r="P73" s="82" t="s">
         <v>92</v>
       </c>
       <c r="Q73" s="55"/>
-      <c r="R73" s="174" t="s">
+      <c r="R73" s="203" t="s">
         <v>10</v>
       </c>
-      <c r="S73" s="174"/>
-      <c r="T73" s="64" t="s">
+      <c r="S73" s="203"/>
+      <c r="T73" s="60" t="s">
         <v>93</v>
       </c>
-      <c r="U73" s="94" t="s">
+      <c r="U73" s="90" t="s">
         <v>96</v>
       </c>
       <c r="V73" s="50"/>
     </row>
     <row r="74" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="L74" s="44"/>
-      <c r="M74" s="84"/>
-      <c r="N74" s="85"/>
-      <c r="O74" s="122"/>
-      <c r="P74" s="86"/>
+      <c r="M74" s="80"/>
+      <c r="N74" s="81"/>
+      <c r="O74" s="118"/>
+      <c r="P74" s="82"/>
       <c r="Q74" s="55"/>
-      <c r="R74" s="174"/>
-      <c r="S74" s="174"/>
-      <c r="T74" s="64"/>
-      <c r="U74" s="94"/>
+      <c r="R74" s="203"/>
+      <c r="S74" s="203"/>
+      <c r="T74" s="60"/>
+      <c r="U74" s="90"/>
       <c r="V74" s="50"/>
     </row>
     <row r="75" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="L75" s="44"/>
-      <c r="M75" s="136" t="s">
+      <c r="M75" s="128" t="s">
         <v>61</v>
       </c>
-      <c r="N75" s="137"/>
-      <c r="O75" s="138"/>
-      <c r="P75" s="139"/>
-      <c r="Q75" s="140"/>
-      <c r="R75" s="175"/>
-      <c r="S75" s="175"/>
-      <c r="T75" s="172"/>
-      <c r="U75" s="173"/>
+      <c r="N75" s="129"/>
+      <c r="O75" s="130"/>
+      <c r="P75" s="131"/>
+      <c r="Q75" s="132"/>
+      <c r="R75" s="204"/>
+      <c r="S75" s="204"/>
+      <c r="T75" s="201"/>
+      <c r="U75" s="202"/>
       <c r="V75" s="50"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="L76" s="44"/>
-      <c r="M76" s="136" t="s">
+      <c r="M76" s="128" t="s">
         <v>62</v>
       </c>
-      <c r="N76" s="137"/>
-      <c r="O76" s="138"/>
-      <c r="P76" s="139"/>
-      <c r="Q76" s="140"/>
-      <c r="R76" s="141"/>
-      <c r="S76" s="141"/>
-      <c r="T76" s="172"/>
-      <c r="U76" s="173"/>
+      <c r="N76" s="129"/>
+      <c r="O76" s="130"/>
+      <c r="P76" s="131"/>
+      <c r="Q76" s="132"/>
+      <c r="R76" s="133"/>
+      <c r="S76" s="133"/>
+      <c r="T76" s="201"/>
+      <c r="U76" s="202"/>
       <c r="V76" s="50"/>
     </row>
     <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L77" s="44"/>
-      <c r="M77" s="93"/>
-      <c r="N77" s="63"/>
-      <c r="O77" s="122"/>
-      <c r="P77" s="86"/>
+      <c r="M77" s="89"/>
+      <c r="N77" s="59"/>
+      <c r="O77" s="118"/>
+      <c r="P77" s="82"/>
       <c r="Q77" s="55"/>
       <c r="R77" s="55"/>
       <c r="S77" s="55"/>
-      <c r="T77" s="64"/>
-      <c r="U77" s="94"/>
+      <c r="T77" s="60"/>
+      <c r="U77" s="90"/>
       <c r="V77" s="50"/>
     </row>
     <row r="78" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L78" s="44"/>
-      <c r="M78" s="100" t="s">
+      <c r="M78" s="96" t="s">
         <v>11</v>
       </c>
-      <c r="N78" s="101">
+      <c r="N78" s="97">
         <f>SUM(N76:N77)</f>
         <v>0</v>
       </c>
-      <c r="O78" s="95"/>
-      <c r="P78" s="97"/>
-      <c r="Q78" s="96"/>
-      <c r="R78" s="96"/>
-      <c r="S78" s="96"/>
-      <c r="T78" s="98"/>
-      <c r="U78" s="99"/>
+      <c r="O78" s="91"/>
+      <c r="P78" s="93"/>
+      <c r="Q78" s="92"/>
+      <c r="R78" s="92"/>
+      <c r="S78" s="92"/>
+      <c r="T78" s="94"/>
+      <c r="U78" s="95"/>
       <c r="V78" s="50"/>
     </row>
     <row r="79" spans="1:23" x14ac:dyDescent="0.3">
@@ -4223,18 +4180,50 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="O32:P32"/>
+  <mergeCells count="72">
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="M69:U69"/>
+    <mergeCell ref="R67:S67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="P67:Q67"/>
+    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M38:N38"/>
     <mergeCell ref="M22:U22"/>
     <mergeCell ref="Q26:S26"/>
     <mergeCell ref="O29:P29"/>
@@ -4251,49 +4240,19 @@
     <mergeCell ref="N23:S23"/>
     <mergeCell ref="N24:S24"/>
     <mergeCell ref="T25:U25"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="M69:U69"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="T67:U67"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T75:U75"/>
-    <mergeCell ref="M67:O67"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="O25:P25"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>